<commit_message>
feat: refresh datasets (865 commits across nested repos; weekends logged)
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/works.xlsx
+++ b/works.xlsx
@@ -528,11 +528,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R36"/>
+  <dimension ref="A1:R42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="44" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
@@ -1484,7 +1484,7 @@
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>approx</t>
+          <t>git</t>
         </is>
       </c>
       <c r="L14" s="3" t="inlineStr">
@@ -1496,7 +1496,7 @@
         <v>35</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>0</v>
+        <v>218</v>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
@@ -1551,12 +1551,12 @@
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>approx</t>
+          <t>git</t>
         </is>
       </c>
       <c r="L15" s="3" t="inlineStr">
@@ -1610,17 +1610,17 @@
       <c r="H16" s="6" t="inlineStr"/>
       <c r="I16" s="6" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="J16" s="6" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="K16" s="6" t="inlineStr">
         <is>
-          <t>approx</t>
+          <t>git</t>
         </is>
       </c>
       <c r="L16" s="7" t="inlineStr">
@@ -1674,17 +1674,17 @@
       <c r="H17" s="2" t="inlineStr"/>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>approx</t>
+          <t>git</t>
         </is>
       </c>
       <c r="L17" s="3" t="inlineStr">
@@ -1738,17 +1738,17 @@
       <c r="H18" s="2" t="inlineStr"/>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>approx</t>
+          <t>git</t>
         </is>
       </c>
       <c r="L18" s="3" t="inlineStr">
@@ -2287,22 +2287,22 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Umbrella of 5 products: SelfAware Continuum, Hyper, audit-shield, spatial-nexus, kimo-ai-agent.</t>
+          <t>Six-product local-AI suite (6 repos): Continuum (HVAC intelligence), AuditShield, Autonomous-Cortex, NeuralPulse, VisioScan, SpatialNexus.</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Multi-product workspace — design &amp; development across the portfolio.</t>
+          <t>Designed &amp; built the multi-product suite across six repositories.</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>React; Python; Docker</t>
+          <t>React; TypeScript; Python; Neo4j; pgvector; Ollama; Docker</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
@@ -2312,7 +2312,7 @@
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
-          <t>approx</t>
+          <t>git</t>
         </is>
       </c>
       <c r="L26" s="3" t="inlineStr">
@@ -2321,10 +2321,10 @@
         </is>
       </c>
       <c r="M26" s="2" t="n">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="N26" s="2" t="n">
-        <v>0</v>
+        <v>94</v>
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
@@ -2333,7 +2333,7 @@
       </c>
       <c r="P26" s="2" t="inlineStr">
         <is>
-          <t>5 flagship products grouped locally; Continuum, Hyper, audit-shield, spatial-nexus, kimo-ai-agent</t>
+          <t>6 products in one suite; SelfAware Continuum: Unicharm + Neo4j + pgvector + Ollama</t>
         </is>
       </c>
       <c r="Q26" s="2" t="inlineStr"/>
@@ -2342,18 +2342,22 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>concept-standard</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr"/>
+          <t>selfaware-suite.1</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>selfaware-suite</t>
+        </is>
+      </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>project</t>
+          <t>milestone</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Concept Standard — Graph Analytics</t>
+          <t>SelfAware Continuum — HVAC intelligence</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -2363,32 +2367,24 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Interactive concept-map viewer (1,159 concepts, 5,985 relations) for lesson generation.</t>
-        </is>
-      </c>
-      <c r="G27" s="2" t="inlineStr">
-        <is>
-          <t>Built the in-browser graph analytics tool (ECharts + Neo4j GDS).</t>
-        </is>
-      </c>
-      <c r="H27" s="2" t="inlineStr">
-        <is>
-          <t>Python; JavaScript; ECharts; Neo4j</t>
-        </is>
-      </c>
+          <t>Neo4j + pgvector + Ollama</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr"/>
+      <c r="H27" s="2" t="inlineStr"/>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>ongoing</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
-          <t>approx</t>
+          <t>git</t>
         </is>
       </c>
       <c r="L27" s="3" t="inlineStr">
@@ -2402,140 +2398,116 @@
       <c r="N27" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="O27" s="2" t="inlineStr">
-        <is>
-          <t>D:\Harshan\concept-standard</t>
-        </is>
-      </c>
-      <c r="P27" s="2" t="inlineStr">
-        <is>
-          <t>1,159 concepts / 5,985 relations; Force/circular graphs, command palette, light/dark, a11y</t>
-        </is>
-      </c>
+      <c r="O27" s="2" t="inlineStr"/>
+      <c r="P27" s="2" t="inlineStr"/>
       <c r="Q27" s="2" t="inlineStr"/>
       <c r="R27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="6" t="inlineStr">
-        <is>
-          <t>voxara</t>
-        </is>
-      </c>
-      <c r="B28" s="6" t="inlineStr"/>
-      <c r="C28" s="6" t="inlineStr">
-        <is>
-          <t>project</t>
-        </is>
-      </c>
-      <c r="D28" s="6" t="inlineStr">
-        <is>
-          <t>VOXARA AI — Voice Intelligence</t>
-        </is>
-      </c>
-      <c r="E28" s="6" t="inlineStr">
-        <is>
-          <t>Voice AI</t>
-        </is>
-      </c>
-      <c r="F28" s="6" t="inlineStr">
-        <is>
-          <t>Realtime on-prem AI voice intelligence platform — monorepo with local LLM, Whisper STT, Piper TTS.</t>
-        </is>
-      </c>
-      <c r="G28" s="6" t="inlineStr">
-        <is>
-          <t>Architecture &amp; monorepo setup (pnpm/Turbo), service scaffolding.</t>
-        </is>
-      </c>
-      <c r="H28" s="6" t="inlineStr">
-        <is>
-          <t>Node.js; pnpm; Turbo; Ollama; Whisper; Piper; Docker</t>
-        </is>
-      </c>
-      <c r="I28" s="6" t="inlineStr">
-        <is>
-          <t>2026-05-20</t>
-        </is>
-      </c>
-      <c r="J28" s="6" t="inlineStr">
-        <is>
-          <t>2026-05-21</t>
-        </is>
-      </c>
-      <c r="K28" s="6" t="inlineStr">
-        <is>
-          <t>approx</t>
-        </is>
-      </c>
-      <c r="L28" s="7" t="inlineStr">
-        <is>
-          <t>Paused</t>
-        </is>
-      </c>
-      <c r="M28" s="6" t="n">
-        <v>30</v>
-      </c>
-      <c r="N28" s="6" t="n">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>selfaware-suite.2</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>selfaware-suite</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>milestone</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>AuditShield — Compliance Ledger</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t>SelfAware Suite</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>Compliance ledger</t>
+        </is>
+      </c>
+      <c r="G28" s="4" t="inlineStr"/>
+      <c r="H28" s="4" t="inlineStr"/>
+      <c r="I28" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="J28" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="K28" s="4" t="inlineStr">
+        <is>
+          <t>git</t>
+        </is>
+      </c>
+      <c r="L28" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M28" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="N28" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="O28" s="6" t="inlineStr">
-        <is>
-          <t>D:\Harshan\VOXARA AI</t>
-        </is>
-      </c>
-      <c r="P28" s="6" t="inlineStr">
-        <is>
-          <t>Largest by file count (37 items); Local LLM + Whisper + Piper TTS</t>
-        </is>
-      </c>
-      <c r="Q28" s="6" t="inlineStr"/>
-      <c r="R28" s="6" t="inlineStr"/>
+      <c r="O28" s="4" t="inlineStr"/>
+      <c r="P28" s="4" t="inlineStr"/>
+      <c r="Q28" s="4" t="inlineStr"/>
+      <c r="R28" s="4" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>travel-app</t>
-        </is>
-      </c>
-      <c r="B29" s="4" t="inlineStr"/>
+          <t>selfaware-suite.3</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>selfaware-suite</t>
+        </is>
+      </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>project</t>
+          <t>milestone</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>TripTrail — Travel &amp; Expense (RANGSONS)</t>
+          <t>Autonomous-Cortex — Mission Console</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>Client Apps</t>
+          <t>SelfAware Suite</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>Buildless travel/expense reporting web app for RANGSONS LLP with HR approval + Google Sheets.</t>
-        </is>
-      </c>
-      <c r="G29" s="4" t="inlineStr">
-        <is>
-          <t>Sole developer — static web app, Supabase backend, approval flow.</t>
-        </is>
-      </c>
-      <c r="H29" s="4" t="inlineStr">
-        <is>
-          <t>HTML; Tailwind; JavaScript; Supabase</t>
-        </is>
-      </c>
+          <t>Mission console</t>
+        </is>
+      </c>
+      <c r="G29" s="4" t="inlineStr"/>
+      <c r="H29" s="4" t="inlineStr"/>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="J29" s="4" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="K29" s="4" t="inlineStr">
@@ -2552,219 +2524,187 @@
         <v>100</v>
       </c>
       <c r="N29" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="O29" s="4" t="inlineStr">
-        <is>
-          <t>D:\Harshan\travel-app</t>
-        </is>
-      </c>
-      <c r="P29" s="4" t="inlineStr">
-        <is>
-          <t>HR approval + Google Sheets integration; Buildless static deployment</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="O29" s="4" t="inlineStr"/>
+      <c r="P29" s="4" t="inlineStr"/>
       <c r="Q29" s="4" t="inlineStr"/>
       <c r="R29" s="4" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" s="6" t="inlineStr">
-        <is>
-          <t>konva</t>
-        </is>
-      </c>
-      <c r="B30" s="6" t="inlineStr"/>
-      <c r="C30" s="6" t="inlineStr">
-        <is>
-          <t>project</t>
-        </is>
-      </c>
-      <c r="D30" s="6" t="inlineStr">
-        <is>
-          <t>Konva Canvas App</t>
-        </is>
-      </c>
-      <c r="E30" s="6" t="inlineStr">
-        <is>
-          <t>Client Apps</t>
-        </is>
-      </c>
-      <c r="F30" s="6" t="inlineStr">
-        <is>
-          <t>React + TypeScript canvas/drawing app template (likely a UI/design component base).</t>
-        </is>
-      </c>
-      <c r="G30" s="6" t="inlineStr">
-        <is>
-          <t>Template/prototype setup.</t>
-        </is>
-      </c>
-      <c r="H30" s="6" t="inlineStr">
-        <is>
-          <t>React; TypeScript; Vite; Konva</t>
-        </is>
-      </c>
-      <c r="I30" s="6" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="J30" s="6" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="K30" s="6" t="inlineStr">
-        <is>
-          <t>approx</t>
-        </is>
-      </c>
-      <c r="L30" s="7" t="inlineStr">
-        <is>
-          <t>Paused</t>
-        </is>
-      </c>
-      <c r="M30" s="6" t="n">
-        <v>25</v>
-      </c>
-      <c r="N30" s="6" t="n">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>selfaware-suite.4</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>selfaware-suite</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>milestone</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>NeuralPulse — Signal Lab</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>SelfAware Suite</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>Signal lab</t>
+        </is>
+      </c>
+      <c r="G30" s="4" t="inlineStr"/>
+      <c r="H30" s="4" t="inlineStr"/>
+      <c r="I30" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="J30" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="K30" s="4" t="inlineStr">
+        <is>
+          <t>git</t>
+        </is>
+      </c>
+      <c r="L30" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M30" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="N30" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="O30" s="6" t="inlineStr">
-        <is>
-          <t>D:\Harshan\konva</t>
-        </is>
-      </c>
-      <c r="P30" s="6" t="inlineStr">
-        <is>
-          <t>Canvas/drawing UI base</t>
-        </is>
-      </c>
-      <c r="Q30" s="6" t="inlineStr"/>
-      <c r="R30" s="6" t="inlineStr"/>
+      <c r="O30" s="4" t="inlineStr"/>
+      <c r="P30" s="4" t="inlineStr"/>
+      <c r="Q30" s="4" t="inlineStr"/>
+      <c r="R30" s="4" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" s="6" t="inlineStr">
-        <is>
-          <t>farmer-app</t>
-        </is>
-      </c>
-      <c r="B31" s="6" t="inlineStr"/>
-      <c r="C31" s="6" t="inlineStr">
-        <is>
-          <t>project</t>
-        </is>
-      </c>
-      <c r="D31" s="6" t="inlineStr">
-        <is>
-          <t>Farmer App</t>
-        </is>
-      </c>
-      <c r="E31" s="6" t="inlineStr">
-        <is>
-          <t>Client Apps</t>
-        </is>
-      </c>
-      <c r="F31" s="6" t="inlineStr">
-        <is>
-          <t>Early/placeholder project.</t>
-        </is>
-      </c>
-      <c r="G31" s="6" t="inlineStr">
-        <is>
-          <t>Initial scaffolding.</t>
-        </is>
-      </c>
-      <c r="H31" s="6" t="inlineStr"/>
-      <c r="I31" s="6" t="inlineStr">
-        <is>
-          <t>2026-05-29</t>
-        </is>
-      </c>
-      <c r="J31" s="6" t="inlineStr">
-        <is>
-          <t>2026-06-03</t>
-        </is>
-      </c>
-      <c r="K31" s="6" t="inlineStr">
-        <is>
-          <t>approx</t>
-        </is>
-      </c>
-      <c r="L31" s="7" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="M31" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="N31" s="6" t="n">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>selfaware-suite.5</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>selfaware-suite</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>milestone</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>VisioScan — Light Studio</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>SelfAware Suite</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>Light studio</t>
+        </is>
+      </c>
+      <c r="G31" s="4" t="inlineStr"/>
+      <c r="H31" s="4" t="inlineStr"/>
+      <c r="I31" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="J31" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="K31" s="4" t="inlineStr">
+        <is>
+          <t>git</t>
+        </is>
+      </c>
+      <c r="L31" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M31" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="N31" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="O31" s="6" t="inlineStr">
-        <is>
-          <t>D:\Harshan\farmer-app</t>
-        </is>
-      </c>
-      <c r="P31" s="6" t="inlineStr">
-        <is>
-          <t>Placeholder — minimal contents</t>
-        </is>
-      </c>
-      <c r="Q31" s="6" t="inlineStr"/>
-      <c r="R31" s="6" t="inlineStr"/>
+      <c r="O31" s="4" t="inlineStr"/>
+      <c r="P31" s="4" t="inlineStr"/>
+      <c r="Q31" s="4" t="inlineStr"/>
+      <c r="R31" s="4" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>selfaware-dev-stack</t>
-        </is>
-      </c>
-      <c r="B32" s="4" t="inlineStr"/>
+          <t>selfaware-suite.6</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>selfaware-suite</t>
+        </is>
+      </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>project</t>
+          <t>milestone</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>SelfAware Dev Stack</t>
+          <t>SpatialNexus — Topology Atlas</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>Infra &amp; Tooling</t>
+          <t>SelfAware Suite</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>Canonical local Docker dev stack (MySQL, PostgreSQL, Neo4j, Redis) for the SelfAware products.</t>
-        </is>
-      </c>
-      <c r="G32" s="4" t="inlineStr">
-        <is>
-          <t>Authored the docker-compose environment for 4 products.</t>
-        </is>
-      </c>
-      <c r="H32" s="4" t="inlineStr">
-        <is>
-          <t>Docker; MySQL; PostgreSQL; Neo4j; Redis</t>
-        </is>
-      </c>
+          <t>Topology atlas</t>
+        </is>
+      </c>
+      <c r="G32" s="4" t="inlineStr"/>
+      <c r="H32" s="4" t="inlineStr"/>
       <c r="I32" s="4" t="inlineStr">
         <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="J32" s="4" t="inlineStr">
+        <is>
           <t>2026-05-21</t>
         </is>
       </c>
-      <c r="J32" s="4" t="inlineStr">
-        <is>
-          <t>2026-05-21</t>
-        </is>
-      </c>
       <c r="K32" s="4" t="inlineStr">
         <is>
-          <t>approx</t>
+          <t>git</t>
         </is>
       </c>
       <c r="L32" s="5" t="inlineStr">
@@ -2778,251 +2718,243 @@
       <c r="N32" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="O32" s="4" t="inlineStr">
-        <is>
-          <t>D:\Harshan\selfaware-dev-stack</t>
-        </is>
-      </c>
-      <c r="P32" s="4" t="inlineStr">
-        <is>
-          <t>One dev environment for 4 products</t>
-        </is>
-      </c>
+      <c r="O32" s="4" t="inlineStr"/>
+      <c r="P32" s="4" t="inlineStr"/>
       <c r="Q32" s="4" t="inlineStr"/>
       <c r="R32" s="4" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" s="4" t="inlineStr">
-        <is>
-          <t>mysql-unicharm-proxy</t>
-        </is>
-      </c>
-      <c r="B33" s="4" t="inlineStr"/>
-      <c r="C33" s="4" t="inlineStr">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>concept-standard</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr"/>
+      <c r="C33" s="2" t="inlineStr">
         <is>
           <t>project</t>
         </is>
       </c>
-      <c r="D33" s="4" t="inlineStr">
-        <is>
-          <t>MySQL Unicharm Proxy (deprecated)</t>
-        </is>
-      </c>
-      <c r="E33" s="4" t="inlineStr">
-        <is>
-          <t>Infra &amp; Tooling</t>
-        </is>
-      </c>
-      <c r="F33" s="4" t="inlineStr">
-        <is>
-          <t>Docker MySQL port-forwarding helper — superseded by selfaware-dev-stack.</t>
-        </is>
-      </c>
-      <c r="G33" s="4" t="inlineStr">
-        <is>
-          <t>Quick infra utility (now reference-only).</t>
-        </is>
-      </c>
-      <c r="H33" s="4" t="inlineStr">
-        <is>
-          <t>Docker; MySQL</t>
-        </is>
-      </c>
-      <c r="I33" s="4" t="inlineStr">
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Concept Standard — Graph Analytics</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>SelfAware Suite</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>Interactive concept-map viewer (1,159 concepts, 5,985 relations) for lesson generation.</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>Built the in-browser graph analytics tool (ECharts + Neo4j GDS).</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>Python; JavaScript; ECharts; Neo4j</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>ongoing</t>
+        </is>
+      </c>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>approx</t>
+        </is>
+      </c>
+      <c r="L33" s="3" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="M33" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="N33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O33" s="2" t="inlineStr">
+        <is>
+          <t>D:\Harshan\concept-standard</t>
+        </is>
+      </c>
+      <c r="P33" s="2" t="inlineStr">
+        <is>
+          <t>1,159 concepts / 5,985 relations; Force/circular graphs, command palette, light/dark, a11y</t>
+        </is>
+      </c>
+      <c r="Q33" s="2" t="inlineStr"/>
+      <c r="R33" s="2" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t>voxara</t>
+        </is>
+      </c>
+      <c r="B34" s="6" t="inlineStr"/>
+      <c r="C34" s="6" t="inlineStr">
+        <is>
+          <t>project</t>
+        </is>
+      </c>
+      <c r="D34" s="6" t="inlineStr">
+        <is>
+          <t>VOXARA AI — Voice Intelligence</t>
+        </is>
+      </c>
+      <c r="E34" s="6" t="inlineStr">
+        <is>
+          <t>Voice AI</t>
+        </is>
+      </c>
+      <c r="F34" s="6" t="inlineStr">
+        <is>
+          <t>Realtime on-prem AI voice intelligence platform — monorepo with local LLM, Whisper STT, Piper TTS.</t>
+        </is>
+      </c>
+      <c r="G34" s="6" t="inlineStr">
+        <is>
+          <t>Architecture &amp; monorepo setup (pnpm/Turbo), service scaffolding.</t>
+        </is>
+      </c>
+      <c r="H34" s="6" t="inlineStr">
+        <is>
+          <t>Node.js; pnpm; Turbo; Ollama; Whisper; Piper; Docker</t>
+        </is>
+      </c>
+      <c r="I34" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="J34" s="6" t="inlineStr">
         <is>
           <t>2026-05-21</t>
         </is>
       </c>
-      <c r="J33" s="4" t="inlineStr">
-        <is>
-          <t>2026-05-21</t>
-        </is>
-      </c>
-      <c r="K33" s="4" t="inlineStr">
+      <c r="K34" s="6" t="inlineStr">
         <is>
           <t>approx</t>
         </is>
       </c>
-      <c r="L33" s="5" t="inlineStr">
+      <c r="L34" s="7" t="inlineStr">
+        <is>
+          <t>Paused</t>
+        </is>
+      </c>
+      <c r="M34" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="N34" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O34" s="6" t="inlineStr">
+        <is>
+          <t>D:\Harshan\VOXARA AI</t>
+        </is>
+      </c>
+      <c r="P34" s="6" t="inlineStr">
+        <is>
+          <t>Largest by file count (37 items); Local LLM + Whisper + Piper TTS</t>
+        </is>
+      </c>
+      <c r="Q34" s="6" t="inlineStr"/>
+      <c r="R34" s="6" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>travel-app</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr"/>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>project</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>TripTrail — Travel &amp; Expense (RANGSONS)</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t>Client Apps</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="inlineStr">
+        <is>
+          <t>Buildless travel/expense reporting web app for RANGSONS LLP with HR approval + Google Sheets.</t>
+        </is>
+      </c>
+      <c r="G35" s="4" t="inlineStr">
+        <is>
+          <t>Sole developer — static web app, Supabase backend, approval flow.</t>
+        </is>
+      </c>
+      <c r="H35" s="4" t="inlineStr">
+        <is>
+          <t>HTML; Tailwind; JavaScript; Supabase</t>
+        </is>
+      </c>
+      <c r="I35" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="J35" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="K35" s="4" t="inlineStr">
+        <is>
+          <t>git</t>
+        </is>
+      </c>
+      <c r="L35" s="5" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="M33" s="4" t="n">
+      <c r="M35" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="N33" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O33" s="4" t="inlineStr">
-        <is>
-          <t>D:\Harshan\mysql-unicharm-proxy</t>
-        </is>
-      </c>
-      <c r="P33" s="4" t="inlineStr">
-        <is>
-          <t>Deprecated — replaced by selfaware-dev-stack</t>
-        </is>
-      </c>
-      <c r="Q33" s="4" t="inlineStr"/>
-      <c r="R33" s="4" t="inlineStr"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="4" t="inlineStr">
-        <is>
-          <t>kimo-ssh-keys</t>
-        </is>
-      </c>
-      <c r="B34" s="4" t="inlineStr"/>
-      <c r="C34" s="4" t="inlineStr">
-        <is>
-          <t>project</t>
-        </is>
-      </c>
-      <c r="D34" s="4" t="inlineStr">
-        <is>
-          <t>Kimo SSH Keys</t>
-        </is>
-      </c>
-      <c r="E34" s="4" t="inlineStr">
-        <is>
-          <t>Infra &amp; Tooling</t>
-        </is>
-      </c>
-      <c r="F34" s="4" t="inlineStr">
-        <is>
-          <t>SSH key storage / Graylinx laptop identity (kept out of git for security).</t>
-        </is>
-      </c>
-      <c r="G34" s="4" t="inlineStr">
-        <is>
-          <t>Access/identity setup.</t>
-        </is>
-      </c>
-      <c r="H34" s="4" t="inlineStr">
-        <is>
-          <t>SSH</t>
-        </is>
-      </c>
-      <c r="I34" s="4" t="inlineStr">
-        <is>
-          <t>2026-05-18</t>
-        </is>
-      </c>
-      <c r="J34" s="4" t="inlineStr">
-        <is>
-          <t>2026-05-18</t>
-        </is>
-      </c>
-      <c r="K34" s="4" t="inlineStr">
-        <is>
-          <t>approx</t>
-        </is>
-      </c>
-      <c r="L34" s="5" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="M34" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="N34" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O34" s="4" t="inlineStr">
-        <is>
-          <t>D:\Harshan\kimo-ssh-keys</t>
-        </is>
-      </c>
-      <c r="P34" s="4" t="inlineStr">
-        <is>
-          <t>Laptop identity &amp; access keys</t>
-        </is>
-      </c>
-      <c r="Q34" s="4" t="inlineStr"/>
-      <c r="R34" s="4" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="6" t="inlineStr">
-        <is>
-          <t>python-etl</t>
-        </is>
-      </c>
-      <c r="B35" s="6" t="inlineStr"/>
-      <c r="C35" s="6" t="inlineStr">
-        <is>
-          <t>project</t>
-        </is>
-      </c>
-      <c r="D35" s="6" t="inlineStr">
-        <is>
-          <t>Python ETL</t>
-        </is>
-      </c>
-      <c r="E35" s="6" t="inlineStr">
-        <is>
-          <t>Infra &amp; Tooling</t>
-        </is>
-      </c>
-      <c r="F35" s="6" t="inlineStr">
-        <is>
-          <t>ETL / transformer-layer workstream (planning + follow-ups in May).</t>
-        </is>
-      </c>
-      <c r="G35" s="6" t="inlineStr">
-        <is>
-          <t>ETL transformer-layer planning and conversion-workflow design.</t>
-        </is>
-      </c>
-      <c r="H35" s="6" t="inlineStr">
-        <is>
-          <t>Python; ETL</t>
-        </is>
-      </c>
-      <c r="I35" s="6" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="J35" s="6" t="inlineStr">
-        <is>
-          <t>2026-05-25</t>
-        </is>
-      </c>
-      <c r="K35" s="6" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-      <c r="L35" s="7" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="M35" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="N35" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="O35" s="6" t="inlineStr">
-        <is>
-          <t>D:\Harshan\python-etl</t>
-        </is>
-      </c>
-      <c r="P35" s="6" t="inlineStr">
-        <is>
-          <t>ETL transformer layer planning</t>
-        </is>
-      </c>
-      <c r="Q35" s="6" t="inlineStr"/>
-      <c r="R35" s="6" t="inlineStr"/>
+      <c r="N35" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="O35" s="4" t="inlineStr">
+        <is>
+          <t>D:\Harshan\travel-app</t>
+        </is>
+      </c>
+      <c r="P35" s="4" t="inlineStr">
+        <is>
+          <t>HR approval + Google Sheets integration; Buildless static deployment</t>
+        </is>
+      </c>
+      <c r="Q35" s="4" t="inlineStr"/>
+      <c r="R35" s="4" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>raspberry</t>
+          <t>konva</t>
         </is>
       </c>
       <c r="B36" s="6" t="inlineStr"/>
@@ -3033,37 +2965,37 @@
       </c>
       <c r="D36" s="6" t="inlineStr">
         <is>
-          <t>Raspberry Stuffs</t>
+          <t>Konva Canvas App</t>
         </is>
       </c>
       <c r="E36" s="6" t="inlineStr">
         <is>
-          <t>Infra &amp; Tooling</t>
+          <t>Client Apps</t>
         </is>
       </c>
       <c r="F36" s="6" t="inlineStr">
         <is>
-          <t>Raspberry Pi / edge experiments (placeholder).</t>
+          <t>React + TypeScript canvas/drawing app template (likely a UI/design component base).</t>
         </is>
       </c>
       <c r="G36" s="6" t="inlineStr">
         <is>
-          <t>Edge hardware experiments.</t>
+          <t>Template/prototype setup.</t>
         </is>
       </c>
       <c r="H36" s="6" t="inlineStr">
         <is>
-          <t>Raspberry Pi</t>
+          <t>React; TypeScript; Vite; Konva</t>
         </is>
       </c>
       <c r="I36" s="6" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="J36" s="6" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="K36" s="6" t="inlineStr">
@@ -3073,27 +3005,483 @@
       </c>
       <c r="L36" s="7" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Paused</t>
         </is>
       </c>
       <c r="M36" s="6" t="n">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="N36" s="6" t="n">
         <v>0</v>
       </c>
       <c r="O36" s="6" t="inlineStr">
         <is>
-          <t>D:\Harshan\Rasberry-stuffs</t>
+          <t>D:\Harshan\konva</t>
         </is>
       </c>
       <c r="P36" s="6" t="inlineStr">
         <is>
-          <t>Placeholder</t>
+          <t>Canvas/drawing UI base</t>
         </is>
       </c>
       <c r="Q36" s="6" t="inlineStr"/>
       <c r="R36" s="6" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>farmer-app</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr"/>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>project</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Nesso — Farm Traceability Platform</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>Client Apps</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>Farm-to-fork traceability platform for NR Group (Nesso).</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>Built the traceability web app — including a weekend build sprint (30–31 May).</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>TypeScript; React; Node.js</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="K37" s="2" t="inlineStr">
+        <is>
+          <t>git</t>
+        </is>
+      </c>
+      <c r="L37" s="3" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="M37" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="N37" s="2" t="n">
+        <v>190</v>
+      </c>
+      <c r="O37" s="2" t="inlineStr">
+        <is>
+          <t>D:\Harshan\farmer-app</t>
+        </is>
+      </c>
+      <c r="P37" s="2" t="inlineStr">
+        <is>
+          <t>Farm-to-fork traceability (NR Group); ~1-week build incl. weekend sprint</t>
+        </is>
+      </c>
+      <c r="Q37" s="2" t="inlineStr"/>
+      <c r="R37" s="2" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>selfaware-dev-stack</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr"/>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>project</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>SelfAware Dev Stack</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t>Infra &amp; Tooling</t>
+        </is>
+      </c>
+      <c r="F38" s="4" t="inlineStr">
+        <is>
+          <t>Canonical local Docker dev stack (MySQL, PostgreSQL, Neo4j, Redis) for the SelfAware products.</t>
+        </is>
+      </c>
+      <c r="G38" s="4" t="inlineStr">
+        <is>
+          <t>Authored the docker-compose environment for 4 products.</t>
+        </is>
+      </c>
+      <c r="H38" s="4" t="inlineStr">
+        <is>
+          <t>Docker; MySQL; PostgreSQL; Neo4j; Redis</t>
+        </is>
+      </c>
+      <c r="I38" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="J38" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="K38" s="4" t="inlineStr">
+        <is>
+          <t>approx</t>
+        </is>
+      </c>
+      <c r="L38" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M38" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="N38" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O38" s="4" t="inlineStr">
+        <is>
+          <t>D:\Harshan\selfaware-dev-stack</t>
+        </is>
+      </c>
+      <c r="P38" s="4" t="inlineStr">
+        <is>
+          <t>One dev environment for 4 products</t>
+        </is>
+      </c>
+      <c r="Q38" s="4" t="inlineStr"/>
+      <c r="R38" s="4" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>mysql-unicharm-proxy</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr"/>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>project</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>MySQL Unicharm Proxy (deprecated)</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>Infra &amp; Tooling</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t>Docker MySQL port-forwarding helper — superseded by selfaware-dev-stack.</t>
+        </is>
+      </c>
+      <c r="G39" s="4" t="inlineStr">
+        <is>
+          <t>Quick infra utility (now reference-only).</t>
+        </is>
+      </c>
+      <c r="H39" s="4" t="inlineStr">
+        <is>
+          <t>Docker; MySQL</t>
+        </is>
+      </c>
+      <c r="I39" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="J39" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="K39" s="4" t="inlineStr">
+        <is>
+          <t>approx</t>
+        </is>
+      </c>
+      <c r="L39" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M39" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="N39" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O39" s="4" t="inlineStr">
+        <is>
+          <t>D:\Harshan\mysql-unicharm-proxy</t>
+        </is>
+      </c>
+      <c r="P39" s="4" t="inlineStr">
+        <is>
+          <t>Deprecated — replaced by selfaware-dev-stack</t>
+        </is>
+      </c>
+      <c r="Q39" s="4" t="inlineStr"/>
+      <c r="R39" s="4" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>kimo-ssh-keys</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr"/>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>project</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>Kimo SSH Keys</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="inlineStr">
+        <is>
+          <t>Infra &amp; Tooling</t>
+        </is>
+      </c>
+      <c r="F40" s="4" t="inlineStr">
+        <is>
+          <t>SSH key storage / Graylinx laptop identity (kept out of git for security).</t>
+        </is>
+      </c>
+      <c r="G40" s="4" t="inlineStr">
+        <is>
+          <t>Access/identity setup.</t>
+        </is>
+      </c>
+      <c r="H40" s="4" t="inlineStr">
+        <is>
+          <t>SSH</t>
+        </is>
+      </c>
+      <c r="I40" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="J40" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="K40" s="4" t="inlineStr">
+        <is>
+          <t>approx</t>
+        </is>
+      </c>
+      <c r="L40" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M40" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="N40" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O40" s="4" t="inlineStr">
+        <is>
+          <t>D:\Harshan\kimo-ssh-keys</t>
+        </is>
+      </c>
+      <c r="P40" s="4" t="inlineStr">
+        <is>
+          <t>Laptop identity &amp; access keys</t>
+        </is>
+      </c>
+      <c r="Q40" s="4" t="inlineStr"/>
+      <c r="R40" s="4" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="inlineStr">
+        <is>
+          <t>python-etl</t>
+        </is>
+      </c>
+      <c r="B41" s="6" t="inlineStr"/>
+      <c r="C41" s="6" t="inlineStr">
+        <is>
+          <t>project</t>
+        </is>
+      </c>
+      <c r="D41" s="6" t="inlineStr">
+        <is>
+          <t>Python ETL</t>
+        </is>
+      </c>
+      <c r="E41" s="6" t="inlineStr">
+        <is>
+          <t>Infra &amp; Tooling</t>
+        </is>
+      </c>
+      <c r="F41" s="6" t="inlineStr">
+        <is>
+          <t>ETL / transformer-layer workstream (planning + follow-ups in May).</t>
+        </is>
+      </c>
+      <c r="G41" s="6" t="inlineStr">
+        <is>
+          <t>ETL transformer-layer planning and conversion-workflow design.</t>
+        </is>
+      </c>
+      <c r="H41" s="6" t="inlineStr">
+        <is>
+          <t>Python; ETL</t>
+        </is>
+      </c>
+      <c r="I41" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="J41" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="K41" s="6" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+      <c r="L41" s="7" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="M41" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="N41" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O41" s="6" t="inlineStr">
+        <is>
+          <t>D:\Harshan\python-etl</t>
+        </is>
+      </c>
+      <c r="P41" s="6" t="inlineStr">
+        <is>
+          <t>ETL transformer layer planning</t>
+        </is>
+      </c>
+      <c r="Q41" s="6" t="inlineStr"/>
+      <c r="R41" s="6" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="6" t="inlineStr">
+        <is>
+          <t>raspberry</t>
+        </is>
+      </c>
+      <c r="B42" s="6" t="inlineStr"/>
+      <c r="C42" s="6" t="inlineStr">
+        <is>
+          <t>project</t>
+        </is>
+      </c>
+      <c r="D42" s="6" t="inlineStr">
+        <is>
+          <t>Raspberry Stuffs</t>
+        </is>
+      </c>
+      <c r="E42" s="6" t="inlineStr">
+        <is>
+          <t>Infra &amp; Tooling</t>
+        </is>
+      </c>
+      <c r="F42" s="6" t="inlineStr">
+        <is>
+          <t>Raspberry Pi / edge experiments (placeholder).</t>
+        </is>
+      </c>
+      <c r="G42" s="6" t="inlineStr">
+        <is>
+          <t>Edge hardware experiments.</t>
+        </is>
+      </c>
+      <c r="H42" s="6" t="inlineStr">
+        <is>
+          <t>Raspberry Pi</t>
+        </is>
+      </c>
+      <c r="I42" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="J42" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="K42" s="6" t="inlineStr">
+        <is>
+          <t>approx</t>
+        </is>
+      </c>
+      <c r="L42" s="7" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="M42" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="N42" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O42" s="6" t="inlineStr">
+        <is>
+          <t>D:\Harshan\Rasberry-stuffs</t>
+        </is>
+      </c>
+      <c r="P42" s="6" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="Q42" s="6" t="inlineStr"/>
+      <c r="R42" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4629,17 +5017,33 @@
           <t>Tuesday</t>
         </is>
       </c>
-      <c r="C29" s="15" t="inlineStr"/>
-      <c r="D29" s="10" t="inlineStr"/>
+      <c r="C29" s="14" t="inlineStr">
+        <is>
+          <t>WFH</t>
+        </is>
+      </c>
+      <c r="D29" s="10" t="inlineStr">
+        <is>
+          <t>Mysore (residence)</t>
+        </is>
+      </c>
       <c r="E29" s="10" t="inlineStr"/>
       <c r="F29" s="10" t="inlineStr"/>
       <c r="G29" s="10" t="inlineStr"/>
       <c r="H29" s="10" t="inlineStr"/>
-      <c r="I29" s="10" t="inlineStr"/>
-      <c r="J29" s="10" t="inlineStr"/>
+      <c r="I29" s="10" t="inlineStr">
+        <is>
+          <t>Development activity on OMNYX — Universal IoT Operations Platform (auto-derived from git).</t>
+        </is>
+      </c>
+      <c r="J29" s="10" t="inlineStr">
+        <is>
+          <t>omnyx</t>
+        </is>
+      </c>
       <c r="K29" s="10" t="inlineStr">
         <is>
-          <t>needs-fill</t>
+          <t>derived</t>
         </is>
       </c>
     </row>
@@ -4711,12 +5115,12 @@
       <c r="H31" s="10" t="inlineStr"/>
       <c r="I31" s="10" t="inlineStr">
         <is>
-          <t>Development activity on THERMYNX — HVAC AI Operations Intelligence (auto-derived from git).</t>
+          <t>Development activity on Nesso — Farm Traceability Platform (auto-derived from git).</t>
         </is>
       </c>
       <c r="J31" s="10" t="inlineStr">
         <is>
-          <t>thermynx</t>
+          <t>farmer-app</t>
         </is>
       </c>
       <c r="K31" s="10" t="inlineStr">
@@ -4736,17 +5140,33 @@
           <t>Friday</t>
         </is>
       </c>
-      <c r="C32" s="15" t="inlineStr"/>
-      <c r="D32" s="10" t="inlineStr"/>
+      <c r="C32" s="14" t="inlineStr">
+        <is>
+          <t>WFH</t>
+        </is>
+      </c>
+      <c r="D32" s="10" t="inlineStr">
+        <is>
+          <t>Mysore (residence)</t>
+        </is>
+      </c>
       <c r="E32" s="10" t="inlineStr"/>
       <c r="F32" s="10" t="inlineStr"/>
       <c r="G32" s="10" t="inlineStr"/>
       <c r="H32" s="10" t="inlineStr"/>
-      <c r="I32" s="10" t="inlineStr"/>
-      <c r="J32" s="10" t="inlineStr"/>
+      <c r="I32" s="10" t="inlineStr">
+        <is>
+          <t>Development activity on Nesso — Farm Traceability Platform (auto-derived from git).</t>
+        </is>
+      </c>
+      <c r="J32" s="10" t="inlineStr">
+        <is>
+          <t>farmer-app</t>
+        </is>
+      </c>
       <c r="K32" s="10" t="inlineStr">
         <is>
-          <t>needs-fill</t>
+          <t>derived</t>
         </is>
       </c>
     </row>
@@ -4761,17 +5181,33 @@
           <t>Saturday</t>
         </is>
       </c>
-      <c r="C33" s="15" t="inlineStr"/>
-      <c r="D33" s="10" t="inlineStr"/>
+      <c r="C33" s="14" t="inlineStr">
+        <is>
+          <t>WFH</t>
+        </is>
+      </c>
+      <c r="D33" s="10" t="inlineStr">
+        <is>
+          <t>Mysore (residence)</t>
+        </is>
+      </c>
       <c r="E33" s="10" t="inlineStr"/>
       <c r="F33" s="10" t="inlineStr"/>
       <c r="G33" s="10" t="inlineStr"/>
       <c r="H33" s="10" t="inlineStr"/>
-      <c r="I33" s="10" t="inlineStr"/>
-      <c r="J33" s="10" t="inlineStr"/>
+      <c r="I33" s="10" t="inlineStr">
+        <is>
+          <t>Development activity on Nesso — Farm Traceability Platform (auto-derived from git).</t>
+        </is>
+      </c>
+      <c r="J33" s="10" t="inlineStr">
+        <is>
+          <t>farmer-app</t>
+        </is>
+      </c>
       <c r="K33" s="10" t="inlineStr">
         <is>
-          <t>needs-fill</t>
+          <t>derived</t>
         </is>
       </c>
     </row>
@@ -4786,17 +5222,33 @@
           <t>Sunday</t>
         </is>
       </c>
-      <c r="C34" s="15" t="inlineStr"/>
-      <c r="D34" s="10" t="inlineStr"/>
+      <c r="C34" s="14" t="inlineStr">
+        <is>
+          <t>WFH</t>
+        </is>
+      </c>
+      <c r="D34" s="10" t="inlineStr">
+        <is>
+          <t>Mysore (residence)</t>
+        </is>
+      </c>
       <c r="E34" s="10" t="inlineStr"/>
       <c r="F34" s="10" t="inlineStr"/>
       <c r="G34" s="10" t="inlineStr"/>
       <c r="H34" s="10" t="inlineStr"/>
-      <c r="I34" s="10" t="inlineStr"/>
-      <c r="J34" s="10" t="inlineStr"/>
+      <c r="I34" s="10" t="inlineStr">
+        <is>
+          <t>Development activity on Nesso — Farm Traceability Platform (auto-derived from git).</t>
+        </is>
+      </c>
+      <c r="J34" s="10" t="inlineStr">
+        <is>
+          <t>farmer-app</t>
+        </is>
+      </c>
       <c r="K34" s="10" t="inlineStr">
         <is>
-          <t>needs-fill</t>
+          <t>derived</t>
         </is>
       </c>
     </row>
@@ -4827,12 +5279,12 @@
       <c r="H35" s="10" t="inlineStr"/>
       <c r="I35" s="10" t="inlineStr">
         <is>
-          <t>Development activity on THERMYNX — HVAC AI Operations Intelligence (auto-derived from git).</t>
+          <t>Development activity on Nesso — Farm Traceability Platform (auto-derived from git).</t>
         </is>
       </c>
       <c r="J35" s="10" t="inlineStr">
         <is>
-          <t>thermynx</t>
+          <t>farmer-app</t>
         </is>
       </c>
       <c r="K35" s="10" t="inlineStr">
@@ -4868,12 +5320,12 @@
       <c r="H36" s="10" t="inlineStr"/>
       <c r="I36" s="10" t="inlineStr">
         <is>
-          <t>Development activity on THERMYNX — HVAC AI Operations Intelligence (auto-derived from git).</t>
+          <t>Development activity on Nesso — Farm Traceability Platform (auto-derived from git).</t>
         </is>
       </c>
       <c r="J36" s="10" t="inlineStr">
         <is>
-          <t>thermynx</t>
+          <t>farmer-app</t>
         </is>
       </c>
       <c r="K36" s="10" t="inlineStr">
@@ -4909,12 +5361,12 @@
       <c r="H37" s="10" t="inlineStr"/>
       <c r="I37" s="10" t="inlineStr">
         <is>
-          <t>Development activity on TripTrail — Travel &amp; Expense (RANGSONS) (auto-derived from git).</t>
+          <t>Development activity on Nesso — Farm Traceability Platform (auto-derived from git).</t>
         </is>
       </c>
       <c r="J37" s="10" t="inlineStr">
         <is>
-          <t>travel-app</t>
+          <t>farmer-app</t>
         </is>
       </c>
       <c r="K37" s="10" t="inlineStr">
@@ -4950,12 +5402,12 @@
       <c r="H38" s="10" t="inlineStr"/>
       <c r="I38" s="10" t="inlineStr">
         <is>
-          <t>Development activity on THERMYNX — HVAC AI Operations Intelligence (auto-derived from git).</t>
+          <t>Development activity on Current Works in GL — Core Monorepo (auto-derived from git).</t>
         </is>
       </c>
       <c r="J38" s="10" t="inlineStr">
         <is>
-          <t>thermynx</t>
+          <t>current-works</t>
         </is>
       </c>
       <c r="K38" s="10" t="inlineStr">
@@ -4991,12 +5443,12 @@
       <c r="H39" s="10" t="inlineStr"/>
       <c r="I39" s="10" t="inlineStr">
         <is>
-          <t>Development activity on THERMYNX — HVAC AI Operations Intelligence (auto-derived from git).</t>
+          <t>Development activity on OMNYX — Universal IoT Operations Platform (auto-derived from git).</t>
         </is>
       </c>
       <c r="J39" s="10" t="inlineStr">
         <is>
-          <t>thermynx</t>
+          <t>omnyx</t>
         </is>
       </c>
       <c r="K39" s="10" t="inlineStr">
@@ -5032,12 +5484,12 @@
       <c r="H40" s="10" t="inlineStr"/>
       <c r="I40" s="10" t="inlineStr">
         <is>
-          <t>Development activity on THERMYNX — HVAC AI Operations Intelligence (auto-derived from git).</t>
+          <t>Development activity on OMNYX — Universal IoT Operations Platform (auto-derived from git).</t>
         </is>
       </c>
       <c r="J40" s="10" t="inlineStr">
         <is>
-          <t>thermynx</t>
+          <t>omnyx</t>
         </is>
       </c>
       <c r="K40" s="10" t="inlineStr">
@@ -5057,17 +5509,33 @@
           <t>Sunday</t>
         </is>
       </c>
-      <c r="C41" s="15" t="inlineStr"/>
-      <c r="D41" s="10" t="inlineStr"/>
+      <c r="C41" s="14" t="inlineStr">
+        <is>
+          <t>WFH</t>
+        </is>
+      </c>
+      <c r="D41" s="10" t="inlineStr">
+        <is>
+          <t>Mysore (residence)</t>
+        </is>
+      </c>
       <c r="E41" s="10" t="inlineStr"/>
       <c r="F41" s="10" t="inlineStr"/>
       <c r="G41" s="10" t="inlineStr"/>
       <c r="H41" s="10" t="inlineStr"/>
-      <c r="I41" s="10" t="inlineStr"/>
-      <c r="J41" s="10" t="inlineStr"/>
+      <c r="I41" s="10" t="inlineStr">
+        <is>
+          <t>Development activity on OMNYX — Universal IoT Operations Platform (auto-derived from git).</t>
+        </is>
+      </c>
+      <c r="J41" s="10" t="inlineStr">
+        <is>
+          <t>omnyx</t>
+        </is>
+      </c>
       <c r="K41" s="10" t="inlineStr">
         <is>
-          <t>needs-fill</t>
+          <t>derived</t>
         </is>
       </c>
     </row>
@@ -5139,12 +5607,12 @@
       <c r="H43" s="10" t="inlineStr"/>
       <c r="I43" s="10" t="inlineStr">
         <is>
-          <t>Development activity on THERMYNX — HVAC AI Operations Intelligence (auto-derived from git).</t>
+          <t>Development activity on OMNYX — Universal IoT Operations Platform (auto-derived from git).</t>
         </is>
       </c>
       <c r="J43" s="10" t="inlineStr">
         <is>
-          <t>thermynx</t>
+          <t>omnyx</t>
         </is>
       </c>
       <c r="K43" s="10" t="inlineStr">
@@ -5221,12 +5689,12 @@
       <c r="H45" s="10" t="inlineStr"/>
       <c r="I45" s="10" t="inlineStr">
         <is>
-          <t>Development activity on THERMYNX — HVAC AI Operations Intelligence (auto-derived from git).</t>
+          <t>Development activity on OMNYX — Universal IoT Operations Platform (auto-derived from git).</t>
         </is>
       </c>
       <c r="J45" s="10" t="inlineStr">
         <is>
-          <t>thermynx</t>
+          <t>omnyx</t>
         </is>
       </c>
       <c r="K45" s="10" t="inlineStr">
@@ -5369,12 +5837,12 @@
       <c r="H49" s="10" t="inlineStr"/>
       <c r="I49" s="10" t="inlineStr">
         <is>
-          <t>Development activity on THERMYNX — HVAC AI Operations Intelligence (auto-derived from git).</t>
+          <t>Development activity on ClimaStream — Real-time HVAC Pipeline (auto-derived from git).</t>
         </is>
       </c>
       <c r="J49" s="10" t="inlineStr">
         <is>
-          <t>thermynx</t>
+          <t>climastream</t>
         </is>
       </c>
       <c r="K49" s="10" t="inlineStr">

</xml_diff>

<commit_message>
feat: descriptive per-day engagement notes from real git commit subjects (not a repeated line)
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/works.xlsx
+++ b/works.xlsx
@@ -704,7 +704,7 @@
         <v>70</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
@@ -1496,7 +1496,7 @@
         <v>35</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
@@ -1551,7 +1551,7 @@
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -1610,12 +1610,12 @@
       <c r="H16" s="6" t="inlineStr"/>
       <c r="I16" s="6" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="J16" s="6" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="K16" s="6" t="inlineStr">
@@ -1674,12 +1674,12 @@
       <c r="H17" s="2" t="inlineStr"/>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
@@ -1738,12 +1738,12 @@
       <c r="H18" s="2" t="inlineStr"/>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
@@ -3071,7 +3071,7 @@
       </c>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>ongoing</t>
         </is>
       </c>
       <c r="K37" s="2" t="inlineStr">
@@ -3088,7 +3088,7 @@
         <v>45</v>
       </c>
       <c r="N37" s="2" t="n">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
@@ -5033,7 +5033,7 @@
       <c r="H29" s="10" t="inlineStr"/>
       <c r="I29" s="10" t="inlineStr">
         <is>
-          <t>Development activity on OMNYX — Universal IoT Operations Platform (auto-derived from git).</t>
+          <t>OMNYX [9]: docs: PROJECT_OVERVIEW.md — vision, legacy comparison, transformation story; docs: ARCHITECTURE_RATIONALE.md — pros, cons, risk register, on-site scenarios; docs: align all MD docs with 2-DB architecture + Alloy/Kafka images (+6 more)  (9 commits)</t>
         </is>
       </c>
       <c r="J29" s="10" t="inlineStr">
@@ -5074,7 +5074,7 @@
       <c r="H30" s="10" t="inlineStr"/>
       <c r="I30" s="10" t="inlineStr">
         <is>
-          <t>Development activity on THERMYNX — HVAC AI Operations Intelligence (auto-derived from git).</t>
+          <t>THERMYNX [1]: feat: implement full-stack HVAC AI operations platform with multi-agent orchestr  (1 commits)</t>
         </is>
       </c>
       <c r="J30" s="10" t="inlineStr">
@@ -5115,12 +5115,12 @@
       <c r="H31" s="10" t="inlineStr"/>
       <c r="I31" s="10" t="inlineStr">
         <is>
-          <t>Development activity on Nesso — Farm Traceability Platform (auto-derived from git).</t>
+          <t>THERMYNX [12]: feat: add architecture documentation and configure environment-specific Claude s; docs(ai): mark Tier 1/2/3 + Perf T1 + Reliability R1/R4 + Eval Phase 1 as shippe; fix(eval+ui): action-verb regex tolerates articles + vite proxy env-driven (+9 more) · Nesso [5]: docs: add comprehensive developer setup guide and link it in README; docs: initialize README.md with project overview, architecture, and documentatio; docs: add comprehensive project implementation plan and detailed screen inventor (+2 more)  (17 commits)</t>
         </is>
       </c>
       <c r="J31" s="10" t="inlineStr">
         <is>
-          <t>farmer-app</t>
+          <t>thermynx</t>
         </is>
       </c>
       <c r="K31" s="10" t="inlineStr">
@@ -5156,7 +5156,7 @@
       <c r="H32" s="10" t="inlineStr"/>
       <c r="I32" s="10" t="inlineStr">
         <is>
-          <t>Development activity on Nesso — Farm Traceability Platform (auto-derived from git).</t>
+          <t>Nesso [8]: feat: implement activities dashboard and logging interface with API integration; feat(phase-3): crops + activities + catalog (POP + inputs) backend; feat(phase-2): web admin UI for farmers — dashboard shell, list, detail, approva (+5 more)  (8 commits)</t>
         </is>
       </c>
       <c r="J32" s="10" t="inlineStr">
@@ -5197,7 +5197,7 @@
       <c r="H33" s="10" t="inlineStr"/>
       <c r="I33" s="10" t="inlineStr">
         <is>
-          <t>Development activity on Nesso — Farm Traceability Platform (auto-derived from git).</t>
+          <t>Nesso [68]: feat(mobile): real in-app support + live multi-language (no more "coming soon"); fix(mobile/login): bulletproof layout + themed + add missing elements; feat(mobile): app-wide dark mode — light/dark token system + working toggles ✅ (+65 more)  (68 commits)</t>
         </is>
       </c>
       <c r="J33" s="10" t="inlineStr">
@@ -5238,7 +5238,7 @@
       <c r="H34" s="10" t="inlineStr"/>
       <c r="I34" s="10" t="inlineStr">
         <is>
-          <t>Development activity on Nesso — Farm Traceability Platform (auto-derived from git).</t>
+          <t>Nesso [30]: perf(P2): web chart code-split, portal OG metadata, mobile FlatList tuning; fix(mobile): revert moti from dashboard — restore stable plain View KPI cards; docs: mark Phase 6/production ON HOLD until user says (P5 banner) (+27 more)  (30 commits)</t>
         </is>
       </c>
       <c r="J34" s="10" t="inlineStr">
@@ -5279,12 +5279,12 @@
       <c r="H35" s="10" t="inlineStr"/>
       <c r="I35" s="10" t="inlineStr">
         <is>
-          <t>Development activity on Nesso — Farm Traceability Platform (auto-derived from git).</t>
+          <t>OMNYX [40]: presentation: fix file:// security warning — embed logo as data URI; presentation: top-only navigation, no bottom nav, BOM stripped, better highlight; presentation: remove left section sidebar — full-width deck (+37 more) · Nesso [34]: feat(web-vite): MiniMap is now a real map (Leaflet+OSM, open-source, no key); docs: add INTEGRATIONS.md (APIs/CDNs/keys) + migration status; perf(web-vite): swap recharts-&gt;ECharts (tree-shaken) + lazy-load heavy routes (+31 more) · THERMYNX [10]: docs(ai): ADR for per-task LLM right-sizing decision; chore(ollama): bump MAX_LOADED_MODELS=3 + pre-warm hot set on restart; feat(ai): right-size models per task in config defaults (+7 more)  (84 commits)</t>
         </is>
       </c>
       <c r="J35" s="10" t="inlineStr">
         <is>
-          <t>farmer-app</t>
+          <t>omnyx</t>
         </is>
       </c>
       <c r="K35" s="10" t="inlineStr">
@@ -5320,12 +5320,12 @@
       <c r="H36" s="10" t="inlineStr"/>
       <c r="I36" s="10" t="inlineStr">
         <is>
-          <t>Development activity on Nesso — Farm Traceability Platform (auto-derived from git).</t>
+          <t>OMNYX [24]: docs(dev): keep ws-bridge in Docker when running api/web locally; style(frontend): new graphite + Klein palette, WCAG AA tuned for both modes; chore(dev): park Keycloak behind phase2 profile; add local hot-reload dev workfl (+21 more) · THERMYNX [10]: docs(ai): sync AI discovery docs and update README to 2026-06-02 final state; docs: add AI discovery documentation and local development settings; docs(ai): deprioritize Grafana/Prometheus dashboard panels — metrics already emi (+7 more) · Nesso [6]: docs(testing): update roles/logins doc for Vite cutover; feat(web-vite): full shell UI/UX parity with the design; fix(web-vite): Leaflet crash + LoginPage navigate-in-render (+3 more)  (40 commits)</t>
         </is>
       </c>
       <c r="J36" s="10" t="inlineStr">
         <is>
-          <t>farmer-app</t>
+          <t>omnyx</t>
         </is>
       </c>
       <c r="K36" s="10" t="inlineStr">
@@ -5361,12 +5361,12 @@
       <c r="H37" s="10" t="inlineStr"/>
       <c r="I37" s="10" t="inlineStr">
         <is>
-          <t>Development activity on Nesso — Farm Traceability Platform (auto-derived from git).</t>
+          <t>OMNYX [55]: feat(protocols): multi-protocol DAL — MQTT + Modbus + OPC-UA adapters; feat(rag): pgvector knowledge base — ingestion + agent retrieval [Phase 2]; feat(phase2): MinIO data lake + Airflow — working telemetry archive (+52 more) · Nesso [39]: feat(mobile): preflight checker + progress logging + timeouts in dev launcher; feat(web-vite): i18n increment — localize all page titles (en/kn/hi); fix(web-vite): responsive audit — stack field grid + scroll calendar on mobile (+36 more) · TripTrail [5]: Fix RLS infinite recursion: SECURITY DEFINER on policy helper functions; Fix totals trigger infinite recursion (pg_trigger_depth guard); Live: join user for employee_name/department; add re-runnable demo seed (+2 more)  (99 commits)</t>
         </is>
       </c>
       <c r="J37" s="10" t="inlineStr">
         <is>
-          <t>farmer-app</t>
+          <t>omnyx</t>
         </is>
       </c>
       <c r="K37" s="10" t="inlineStr">
@@ -5402,7 +5402,7 @@
       <c r="H38" s="10" t="inlineStr"/>
       <c r="I38" s="10" t="inlineStr">
         <is>
-          <t>Development activity on Current Works in GL — Core Monorepo (auto-derived from git).</t>
+          <t>Current Works in GL [16]: docs: add stress test summary report; docs: add Decision section to 1-page summary report; docs: update comparison and 1-page summary with all scales including 4000x and 5 (+13 more) · OMNYX [13]: docs(openapi): regenerate spec snapshots (adds /api/v1/analysis/correlation); chore: gitignore tsbuildinfo + egg-info build artifacts Co-Authored-By: Claude O; feat(analysis): device signal-correlation page + API (+10 more) · THERMYNX [6]: fix: H6+H7+H8 — forecast backend signal, agent history, is_running cast; feat(ui): work-order approve/dismiss card in agent trace (H3); fix(critical): C1+H1+H2+C3 — thread safety, tool injection, connection leak, mes (+3 more)  (35 commits)</t>
         </is>
       </c>
       <c r="J38" s="10" t="inlineStr">
@@ -5443,7 +5443,7 @@
       <c r="H39" s="10" t="inlineStr"/>
       <c r="I39" s="10" t="inlineStr">
         <is>
-          <t>Development activity on OMNYX — Universal IoT Operations Platform (auto-derived from git).</t>
+          <t>OMNYX [33]: feat: real energy/efficiency KPIs from catalog semantics (Gap 1); docs(site): point onboarding/multi-tenancy/simulator docs at the generator + Mer; chore(console): cut over to Console v2 — promote frontend-next, archive legacy,  (+30 more) · THERMYNX [13]: refactor(ai): consolidate prompts + share JSON parser (P1); bump NL-SQL timeout; feat(predictive): trend-based degradation -&gt; auto-proposed PM work orders; fix(ai): reconcile kW/TR 'fair' threshold drift in prompts (+10 more)  (46 commits)</t>
         </is>
       </c>
       <c r="J39" s="10" t="inlineStr">
@@ -5484,7 +5484,7 @@
       <c r="H40" s="10" t="inlineStr"/>
       <c r="I40" s="10" t="inlineStr">
         <is>
-          <t>Development activity on OMNYX — Universal IoT Operations Platform (auto-derived from git).</t>
+          <t>OMNYX [12]: docs(showcase): sync omnyx.html to delivered work; test(e2e): console v2 + reports persistence + control shadow checks; feat(console): report history/generate + RL control-actions card (+9 more) · THERMYNX [12]: feat(cmms): Phase 1C Alarm -&gt; Work Order management; feat(ems): Phase 1B Energy Management + Cost; feat(ui): THERMYNX sibling theme — real thermal-cyan signature accent (+9 more)  (24 commits)</t>
         </is>
       </c>
       <c r="J40" s="10" t="inlineStr">
@@ -5525,7 +5525,7 @@
       <c r="H41" s="10" t="inlineStr"/>
       <c r="I41" s="10" t="inlineStr">
         <is>
-          <t>Development activity on OMNYX — Universal IoT Operations Platform (auto-derived from git).</t>
+          <t>OMNYX [27]: feat: implement hvac vertical extension with agent-backed telemetry, twin predic; feat: implement initial docker-compose infra, airflow integration, and core serv; fix(security): pin RLS tenant in agentic-ai under the omnyx_svc role (+24 more)  (27 commits)</t>
         </is>
       </c>
       <c r="J41" s="10" t="inlineStr">
@@ -5566,7 +5566,7 @@
       <c r="H42" s="10" t="inlineStr"/>
       <c r="I42" s="10" t="inlineStr">
         <is>
-          <t>Development activity on THERMYNX — HVAC AI Operations Intelligence (auto-derived from git).</t>
+          <t>THERMYNX [14]: chore: add backend runtime logs and IDE settings configuration files; fix(ai): substitute mistral-small3.2 for phi4 — phi4-14B crashes Ollama 0.30.6; feat(ui): readable model roster + modernized 'model in use' toast (+11 more)  (14 commits)</t>
         </is>
       </c>
       <c r="J42" s="10" t="inlineStr">
@@ -5607,12 +5607,12 @@
       <c r="H43" s="10" t="inlineStr"/>
       <c r="I43" s="10" t="inlineStr">
         <is>
-          <t>Development activity on OMNYX — Universal IoT Operations Platform (auto-derived from git).</t>
+          <t>THERMYNX [6]: build(agentic): F0 — OSS agentic runtime + eval/test dependency manifests; docs(agentic): fold model-eval routing, performance must-holds, OSS-software lic; docs(agentic): framework rewrite plan, target architecture, ADR-0002, gap re-aud (+3 more) · OMNYX [1]: docs: add OMNYX project handbook and master documentation index  (7 commits)</t>
         </is>
       </c>
       <c r="J43" s="10" t="inlineStr">
         <is>
-          <t>omnyx</t>
+          <t>thermynx</t>
         </is>
       </c>
       <c r="K43" s="10" t="inlineStr">
@@ -5648,7 +5648,7 @@
       <c r="H44" s="10" t="inlineStr"/>
       <c r="I44" s="10" t="inlineStr">
         <is>
-          <t>Development activity on THERMYNX — HVAC AI Operations Intelligence (auto-derived from git).</t>
+          <t>THERMYNX [40]: feat: add custom environment settings and initial AgentRunner implementation; fix(anomaly): stop 'LLM timeout' on causal cards — warm model + headroom + keep_; chore(claude): expand tool allowlist accumulated this session (+37 more)  (40 commits)</t>
         </is>
       </c>
       <c r="J44" s="10" t="inlineStr">
@@ -5689,12 +5689,12 @@
       <c r="H45" s="10" t="inlineStr"/>
       <c r="I45" s="10" t="inlineStr">
         <is>
-          <t>Development activity on OMNYX — Universal IoT Operations Platform (auto-derived from git).</t>
+          <t>THERMYNX [25]: chore(obs): comment out the langfuse SDK; mark tracing disabled / future-only; chore(frontend): remove orphaned migration-leftover components (zero imports); docs(agentic): F4.9 HITL done; F1.11 durable checkpointer deferred to 48/64GB (+22 more) · OMNYX [1]: docs(ops): flag shared Ollama GPU with THERMYNX (avoid VRAM eviction)  (26 commits)</t>
         </is>
       </c>
       <c r="J45" s="10" t="inlineStr">
         <is>
-          <t>omnyx</t>
+          <t>thermynx</t>
         </is>
       </c>
       <c r="K45" s="10" t="inlineStr">
@@ -5730,7 +5730,7 @@
       <c r="H46" s="10" t="inlineStr"/>
       <c r="I46" s="10" t="inlineStr">
         <is>
-          <t>Development activity on THERMYNX — HVAC AI Operations Intelligence (auto-derived from git).</t>
+          <t>THERMYNX [9]: docs(agentic): Session 3 handoff (2026-06-12); fix(eval): pre-push no longer auto-runs the golden suite (it floods the 20 GB GP; feat(agent): per-node timing traces (lightweight, no Langfuse/infra) (+6 more)  (9 commits)</t>
         </is>
       </c>
       <c r="J46" s="10" t="inlineStr">
@@ -5771,7 +5771,7 @@
       <c r="H47" s="10" t="inlineStr"/>
       <c r="I47" s="10" t="inlineStr">
         <is>
-          <t>Development activity on THERMYNX — HVAC AI Operations Intelligence (auto-derived from git).</t>
+          <t>THERMYNX [6]: docs(agentic): loop-accurate plain-English overview + incidents log + Session-4 ; feat(frontend): Agent Lab workbench - tabbed Run/History/Compare/Tune/Validate +; feat(provider): OpenRouter dev-bridge provider switch (chat roles only; embeddin (+3 more)  (6 commits)</t>
         </is>
       </c>
       <c r="J47" s="10" t="inlineStr">
@@ -5837,12 +5837,12 @@
       <c r="H49" s="10" t="inlineStr"/>
       <c r="I49" s="10" t="inlineStr">
         <is>
-          <t>Development activity on ClimaStream — Real-time HVAC Pipeline (auto-derived from git).</t>
+          <t>THERMYNX [24]: feat: add .claude/settings.json with pre-configured shell execution permissions; feat(security): M9 recursive injection-hardening of tool results; Add architectural handbook for Graylinx LLM platform and initialize Claude proje (+21 more) · ClimaStream [1]: docs: add architecture and agentic flow diagrams to project documentation · Nesso [1]: chore: update lockfile to reflect dependency changes · OMNYX [1]: docs: initialize architecture, security, and roadmap documentation and implement  (27 commits)</t>
         </is>
       </c>
       <c r="J49" s="10" t="inlineStr">
         <is>
-          <t>climastream</t>
+          <t>thermynx</t>
         </is>
       </c>
       <c r="K49" s="10" t="inlineStr">

</xml_diff>

<commit_message>
feat: fill gap days (Lingotran task + RAPL/Examic recruitment interviews) — engagement now 0 needs-fill
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/works.xlsx
+++ b/works.xlsx
@@ -52,7 +52,7 @@
       <color rgb="00ABABAB"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -84,11 +84,6 @@
         <fgColor rgb="00E3E3E3"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E2E2E2"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -116,7 +111,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -151,16 +146,13 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3494,7 +3486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K49"/>
+  <dimension ref="A1:K56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3623,270 +3615,202 @@
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="B3" s="10" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="C3" s="12" t="inlineStr">
         <is>
-          <t>Office</t>
+          <t>WFH</t>
         </is>
       </c>
       <c r="D3" s="10" t="inlineStr">
         <is>
-          <t>Graylinx Office Bangalore</t>
-        </is>
-      </c>
-      <c r="E3" s="10" t="inlineStr">
-        <is>
-          <t>GRS Hotel</t>
-        </is>
-      </c>
-      <c r="F3" s="10" t="inlineStr">
-        <is>
-          <t>9:30 AM</t>
-        </is>
-      </c>
-      <c r="G3" s="10" t="inlineStr">
-        <is>
-          <t>6:30 PM</t>
-        </is>
-      </c>
-      <c r="H3" s="10" t="inlineStr">
-        <is>
-          <t>Mysore to Bangalore</t>
-        </is>
-      </c>
+          <t>Mysore</t>
+        </is>
+      </c>
+      <c r="E3" s="10" t="inlineStr"/>
+      <c r="F3" s="10" t="inlineStr"/>
+      <c r="G3" s="10" t="inlineStr"/>
+      <c r="H3" s="10" t="inlineStr"/>
       <c r="I3" s="10" t="inlineStr">
         <is>
-          <t>Started office deployment and stayed at hotel near office</t>
-        </is>
-      </c>
-      <c r="J3" s="10" t="inlineStr">
-        <is>
-          <t>current-works</t>
-        </is>
-      </c>
+          <t>Lingotran task + recruitment interviews for RAPL and Examic.</t>
+        </is>
+      </c>
+      <c r="J3" s="10" t="inlineStr"/>
       <c r="K3" s="10" t="inlineStr">
         <is>
-          <t>csv</t>
+          <t>manual</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="B4" s="10" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="C4" s="12" t="inlineStr">
         <is>
-          <t>Office</t>
+          <t>WFH</t>
         </is>
       </c>
       <c r="D4" s="10" t="inlineStr">
         <is>
-          <t>Graylinx Office Bangalore</t>
-        </is>
-      </c>
-      <c r="E4" s="10" t="inlineStr">
-        <is>
-          <t>GRS Hotel</t>
-        </is>
-      </c>
-      <c r="F4" s="10" t="inlineStr">
-        <is>
-          <t>9:30 AM</t>
-        </is>
-      </c>
-      <c r="G4" s="10" t="inlineStr">
-        <is>
-          <t>6:30 PM</t>
-        </is>
-      </c>
-      <c r="H4" s="10" t="inlineStr">
-        <is>
-          <t>Stayed in Bangalore</t>
-        </is>
-      </c>
+          <t>Mysore</t>
+        </is>
+      </c>
+      <c r="E4" s="10" t="inlineStr"/>
+      <c r="F4" s="10" t="inlineStr"/>
+      <c r="G4" s="10" t="inlineStr"/>
+      <c r="H4" s="10" t="inlineStr"/>
       <c r="I4" s="10" t="inlineStr">
         <is>
-          <t>Continued office work and architecture discussions</t>
-        </is>
-      </c>
-      <c r="J4" s="10" t="inlineStr">
-        <is>
-          <t>current-works</t>
-        </is>
-      </c>
+          <t>Lingotran task + recruitment interviews for RAPL and Examic.</t>
+        </is>
+      </c>
+      <c r="J4" s="10" t="inlineStr"/>
       <c r="K4" s="10" t="inlineStr">
         <is>
-          <t>csv</t>
+          <t>manual</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B5" s="10" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="C5" s="12" t="inlineStr">
         <is>
-          <t>Office</t>
+          <t>WFH</t>
         </is>
       </c>
       <c r="D5" s="10" t="inlineStr">
         <is>
-          <t>Graylinx Office Bangalore</t>
-        </is>
-      </c>
-      <c r="E5" s="10" t="inlineStr">
-        <is>
-          <t>GRS Hotel</t>
-        </is>
-      </c>
-      <c r="F5" s="10" t="inlineStr">
-        <is>
-          <t>9:30 AM</t>
-        </is>
-      </c>
-      <c r="G5" s="10" t="inlineStr">
-        <is>
-          <t>6:30 PM</t>
-        </is>
-      </c>
-      <c r="H5" s="10" t="inlineStr">
-        <is>
-          <t>Stayed in Bangalore</t>
-        </is>
-      </c>
+          <t>Mysore</t>
+        </is>
+      </c>
+      <c r="E5" s="10" t="inlineStr"/>
+      <c r="F5" s="10" t="inlineStr"/>
+      <c r="G5" s="10" t="inlineStr"/>
+      <c r="H5" s="10" t="inlineStr"/>
       <c r="I5" s="10" t="inlineStr">
         <is>
-          <t>Regular office work and coordination discussions</t>
-        </is>
-      </c>
-      <c r="J5" s="10" t="inlineStr">
-        <is>
-          <t>current-works</t>
-        </is>
-      </c>
+          <t>Lingotran task + recruitment interviews for RAPL and Examic.</t>
+        </is>
+      </c>
+      <c r="J5" s="10" t="inlineStr"/>
       <c r="K5" s="10" t="inlineStr">
         <is>
-          <t>csv</t>
+          <t>manual</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="10" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-04-26</t>
         </is>
       </c>
       <c r="B6" s="10" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="C6" s="12" t="inlineStr">
         <is>
-          <t>Office</t>
+          <t>WFH</t>
         </is>
       </c>
       <c r="D6" s="10" t="inlineStr">
         <is>
-          <t>Graylinx Office Bangalore</t>
-        </is>
-      </c>
-      <c r="E6" s="10" t="inlineStr">
-        <is>
-          <t>GRS Hotel</t>
-        </is>
-      </c>
-      <c r="F6" s="10" t="inlineStr">
-        <is>
-          <t>9:30 AM</t>
-        </is>
-      </c>
-      <c r="G6" s="10" t="inlineStr">
-        <is>
-          <t>6:30 PM</t>
-        </is>
-      </c>
-      <c r="H6" s="10" t="inlineStr">
-        <is>
-          <t>Bangalore to Mysore</t>
-        </is>
-      </c>
+          <t>Mysore</t>
+        </is>
+      </c>
+      <c r="E6" s="10" t="inlineStr"/>
+      <c r="F6" s="10" t="inlineStr"/>
+      <c r="G6" s="10" t="inlineStr"/>
+      <c r="H6" s="10" t="inlineStr"/>
       <c r="I6" s="10" t="inlineStr">
         <is>
-          <t>Returned to Mysore due to Friday leave</t>
+          <t>Lingotran task + recruitment interviews for RAPL and Examic.</t>
         </is>
       </c>
       <c r="J6" s="10" t="inlineStr"/>
       <c r="K6" s="10" t="inlineStr">
         <is>
-          <t>csv</t>
+          <t>manual</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B7" s="10" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="C7" s="13" t="inlineStr">
         <is>
-          <t>Leave</t>
+          <t>Office</t>
         </is>
       </c>
       <c r="D7" s="10" t="inlineStr">
         <is>
-          <t>Mysore</t>
-        </is>
-      </c>
-      <c r="E7" s="10" t="inlineStr"/>
+          <t>Graylinx Office Bangalore</t>
+        </is>
+      </c>
+      <c r="E7" s="10" t="inlineStr">
+        <is>
+          <t>GRS Hotel</t>
+        </is>
+      </c>
       <c r="F7" s="10" t="inlineStr">
         <is>
-          <t>Leave</t>
+          <t>9:30 AM</t>
         </is>
       </c>
       <c r="G7" s="10" t="inlineStr">
         <is>
-          <t>Leave</t>
+          <t>6:30 PM</t>
         </is>
       </c>
       <c r="H7" s="10" t="inlineStr">
         <is>
-          <t>Stayed in Mysore</t>
+          <t>Mysore to Bangalore</t>
         </is>
       </c>
       <c r="I7" s="10" t="inlineStr">
         <is>
-          <t>Friday leave and rest day</t>
-        </is>
-      </c>
-      <c r="J7" s="10" t="inlineStr"/>
+          <t>Started office deployment and stayed at hotel near office</t>
+        </is>
+      </c>
+      <c r="J7" s="10" t="inlineStr">
+        <is>
+          <t>current-works</t>
+        </is>
+      </c>
       <c r="K7" s="10" t="inlineStr">
         <is>
           <t>csv</t>
@@ -3896,48 +3820,52 @@
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B8" s="10" t="inlineStr">
         <is>
-          <t>Monday</t>
-        </is>
-      </c>
-      <c r="C8" s="11" t="inlineStr">
-        <is>
-          <t>Discussion</t>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="C8" s="13" t="inlineStr">
+        <is>
+          <t>Office</t>
         </is>
       </c>
       <c r="D8" s="10" t="inlineStr">
         <is>
-          <t>NA Group Office Mysore</t>
-        </is>
-      </c>
-      <c r="E8" s="10" t="inlineStr"/>
+          <t>Graylinx Office Bangalore</t>
+        </is>
+      </c>
+      <c r="E8" s="10" t="inlineStr">
+        <is>
+          <t>GRS Hotel</t>
+        </is>
+      </c>
       <c r="F8" s="10" t="inlineStr">
         <is>
-          <t>10:00 AM</t>
+          <t>9:30 AM</t>
         </is>
       </c>
       <c r="G8" s="10" t="inlineStr">
         <is>
-          <t>6:00 PM</t>
+          <t>6:30 PM</t>
         </is>
       </c>
       <c r="H8" s="10" t="inlineStr">
         <is>
-          <t>Local travel within Mysore</t>
+          <t>Stayed in Bangalore</t>
         </is>
       </c>
       <c r="I8" s="10" t="inlineStr">
         <is>
-          <t>PRD discussion regarding HVAC systems and architecture modules with Vishnu</t>
+          <t>Continued office work and architecture discussions</t>
         </is>
       </c>
       <c r="J8" s="10" t="inlineStr">
         <is>
-          <t>omnyx</t>
+          <t>current-works</t>
         </is>
       </c>
       <c r="K8" s="10" t="inlineStr">
@@ -3949,48 +3877,52 @@
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B9" s="10" t="inlineStr">
         <is>
-          <t>Tuesday</t>
-        </is>
-      </c>
-      <c r="C9" s="11" t="inlineStr">
-        <is>
-          <t>Discussion</t>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C9" s="13" t="inlineStr">
+        <is>
+          <t>Office</t>
         </is>
       </c>
       <c r="D9" s="10" t="inlineStr">
         <is>
-          <t>NA Group Office Mysore</t>
-        </is>
-      </c>
-      <c r="E9" s="10" t="inlineStr"/>
+          <t>Graylinx Office Bangalore</t>
+        </is>
+      </c>
+      <c r="E9" s="10" t="inlineStr">
+        <is>
+          <t>GRS Hotel</t>
+        </is>
+      </c>
       <c r="F9" s="10" t="inlineStr">
         <is>
-          <t>10:00 AM</t>
+          <t>9:30 AM</t>
         </is>
       </c>
       <c r="G9" s="10" t="inlineStr">
         <is>
-          <t>6:00 PM</t>
+          <t>6:30 PM</t>
         </is>
       </c>
       <c r="H9" s="10" t="inlineStr">
         <is>
-          <t>Local travel within Mysore</t>
+          <t>Stayed in Bangalore</t>
         </is>
       </c>
       <c r="I9" s="10" t="inlineStr">
         <is>
-          <t>Continued PRD planning and module discussions</t>
+          <t>Regular office work and coordination discussions</t>
         </is>
       </c>
       <c r="J9" s="10" t="inlineStr">
         <is>
-          <t>omnyx</t>
+          <t>current-works</t>
         </is>
       </c>
       <c r="K9" s="10" t="inlineStr">
@@ -4002,50 +3934,50 @@
     <row r="10">
       <c r="A10" s="10" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="B10" s="10" t="inlineStr">
         <is>
-          <t>Wednesday</t>
-        </is>
-      </c>
-      <c r="C10" s="11" t="inlineStr">
-        <is>
-          <t>Discussion</t>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="C10" s="13" t="inlineStr">
+        <is>
+          <t>Office</t>
         </is>
       </c>
       <c r="D10" s="10" t="inlineStr">
         <is>
-          <t>NA Group Office Mysore</t>
-        </is>
-      </c>
-      <c r="E10" s="10" t="inlineStr"/>
+          <t>Graylinx Office Bangalore</t>
+        </is>
+      </c>
+      <c r="E10" s="10" t="inlineStr">
+        <is>
+          <t>GRS Hotel</t>
+        </is>
+      </c>
       <c r="F10" s="10" t="inlineStr">
         <is>
-          <t>10:00 AM</t>
+          <t>9:30 AM</t>
         </is>
       </c>
       <c r="G10" s="10" t="inlineStr">
         <is>
-          <t>6:00 PM</t>
+          <t>6:30 PM</t>
         </is>
       </c>
       <c r="H10" s="10" t="inlineStr">
         <is>
-          <t>Local travel within Mysore</t>
+          <t>Bangalore to Mysore</t>
         </is>
       </c>
       <c r="I10" s="10" t="inlineStr">
         <is>
-          <t>Finalized PRD discussions and architecture workflows</t>
-        </is>
-      </c>
-      <c r="J10" s="10" t="inlineStr">
-        <is>
-          <t>omnyx</t>
-        </is>
-      </c>
+          <t>Returned to Mysore due to Friday leave</t>
+        </is>
+      </c>
+      <c r="J10" s="10" t="inlineStr"/>
       <c r="K10" s="10" t="inlineStr">
         <is>
           <t>csv</t>
@@ -4055,7 +3987,7 @@
     <row r="11">
       <c r="A11" s="10" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B11" s="10" t="inlineStr">
@@ -4063,39 +3995,35 @@
           <t>Friday</t>
         </is>
       </c>
-      <c r="C11" s="12" t="inlineStr">
-        <is>
-          <t>Office</t>
+      <c r="C11" s="14" t="inlineStr">
+        <is>
+          <t>Leave</t>
         </is>
       </c>
       <c r="D11" s="10" t="inlineStr">
         <is>
-          <t>Graylinx Office Bangalore</t>
-        </is>
-      </c>
-      <c r="E11" s="10" t="inlineStr">
-        <is>
-          <t>GRS Hotel</t>
-        </is>
-      </c>
+          <t>Mysore</t>
+        </is>
+      </c>
+      <c r="E11" s="10" t="inlineStr"/>
       <c r="F11" s="10" t="inlineStr">
         <is>
-          <t>9:30 AM</t>
+          <t>Leave</t>
         </is>
       </c>
       <c r="G11" s="10" t="inlineStr">
         <is>
-          <t>6:30 PM</t>
+          <t>Leave</t>
         </is>
       </c>
       <c r="H11" s="10" t="inlineStr">
         <is>
-          <t>Mysore to Bangalore</t>
+          <t>Stayed in Mysore</t>
         </is>
       </c>
       <c r="I11" s="10" t="inlineStr">
         <is>
-          <t>Worked with Vishnu before his Australia travel and discussed ongoing tasks</t>
+          <t>Friday leave and rest day</t>
         </is>
       </c>
       <c r="J11" s="10" t="inlineStr"/>
@@ -4108,7 +4036,7 @@
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B12" s="10" t="inlineStr">
@@ -4118,54 +4046,34 @@
       </c>
       <c r="C12" s="12" t="inlineStr">
         <is>
-          <t>Office</t>
+          <t>WFH</t>
         </is>
       </c>
       <c r="D12" s="10" t="inlineStr">
         <is>
-          <t>Graylinx Office Bangalore</t>
-        </is>
-      </c>
-      <c r="E12" s="10" t="inlineStr">
-        <is>
-          <t>GRS Hotel</t>
-        </is>
-      </c>
-      <c r="F12" s="10" t="inlineStr">
-        <is>
-          <t>9:30 AM</t>
-        </is>
-      </c>
-      <c r="G12" s="10" t="inlineStr">
-        <is>
-          <t>6:00 PM</t>
-        </is>
-      </c>
-      <c r="H12" s="10" t="inlineStr">
-        <is>
-          <t>Bangalore to Mysore</t>
-        </is>
-      </c>
+          <t>Mysore</t>
+        </is>
+      </c>
+      <c r="E12" s="10" t="inlineStr"/>
+      <c r="F12" s="10" t="inlineStr"/>
+      <c r="G12" s="10" t="inlineStr"/>
+      <c r="H12" s="10" t="inlineStr"/>
       <c r="I12" s="10" t="inlineStr">
         <is>
-          <t>Returned to Mysore after architecture discussions and AI demonstrations</t>
-        </is>
-      </c>
-      <c r="J12" s="10" t="inlineStr">
-        <is>
-          <t>thermynx</t>
-        </is>
-      </c>
+          <t>Lingotran task + recruitment interviews for RAPL and Examic.</t>
+        </is>
+      </c>
+      <c r="J12" s="10" t="inlineStr"/>
       <c r="K12" s="10" t="inlineStr">
         <is>
-          <t>csv</t>
+          <t>manual</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="10" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B13" s="10" t="inlineStr">
@@ -4173,7 +4081,7 @@
           <t>Sunday</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr">
+      <c r="C13" s="12" t="inlineStr">
         <is>
           <t>WFH</t>
         </is>
@@ -4184,37 +4092,25 @@
         </is>
       </c>
       <c r="E13" s="10" t="inlineStr"/>
-      <c r="F13" s="10" t="inlineStr">
-        <is>
-          <t>10:00 AM</t>
-        </is>
-      </c>
-      <c r="G13" s="10" t="inlineStr">
-        <is>
-          <t>5:00 PM</t>
-        </is>
-      </c>
-      <c r="H13" s="10" t="inlineStr">
-        <is>
-          <t>Worked from Mysore residence</t>
-        </is>
-      </c>
+      <c r="F13" s="10" t="inlineStr"/>
+      <c r="G13" s="10" t="inlineStr"/>
+      <c r="H13" s="10" t="inlineStr"/>
       <c r="I13" s="10" t="inlineStr">
         <is>
-          <t>Continued assigned tasks remotely and coordinated pending work</t>
+          <t>Lingotran task + recruitment interviews for RAPL and Examic.</t>
         </is>
       </c>
       <c r="J13" s="10" t="inlineStr"/>
       <c r="K13" s="10" t="inlineStr">
         <is>
-          <t>csv</t>
+          <t>manual</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="10" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B14" s="10" t="inlineStr">
@@ -4222,14 +4118,14 @@
           <t>Monday</t>
         </is>
       </c>
-      <c r="C14" s="14" t="inlineStr">
-        <is>
-          <t>WFH</t>
+      <c r="C14" s="11" t="inlineStr">
+        <is>
+          <t>Discussion</t>
         </is>
       </c>
       <c r="D14" s="10" t="inlineStr">
         <is>
-          <t>Mysore</t>
+          <t>NA Group Office Mysore</t>
         </is>
       </c>
       <c r="E14" s="10" t="inlineStr"/>
@@ -4245,17 +4141,17 @@
       </c>
       <c r="H14" s="10" t="inlineStr">
         <is>
-          <t>Worked from Mysore residence</t>
+          <t>Local travel within Mysore</t>
         </is>
       </c>
       <c r="I14" s="10" t="inlineStr">
         <is>
-          <t>Existing BACnet simulation flow understanding discussions with team</t>
+          <t>PRD discussion regarding HVAC systems and architecture modules with Vishnu</t>
         </is>
       </c>
       <c r="J14" s="10" t="inlineStr">
         <is>
-          <t>gl-pbs</t>
+          <t>omnyx</t>
         </is>
       </c>
       <c r="K14" s="10" t="inlineStr">
@@ -4267,7 +4163,7 @@
     <row r="15">
       <c r="A15" s="10" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B15" s="10" t="inlineStr">
@@ -4275,14 +4171,14 @@
           <t>Tuesday</t>
         </is>
       </c>
-      <c r="C15" s="14" t="inlineStr">
-        <is>
-          <t>WFH</t>
+      <c r="C15" s="11" t="inlineStr">
+        <is>
+          <t>Discussion</t>
         </is>
       </c>
       <c r="D15" s="10" t="inlineStr">
         <is>
-          <t>Mysore</t>
+          <t>NA Group Office Mysore</t>
         </is>
       </c>
       <c r="E15" s="10" t="inlineStr"/>
@@ -4298,17 +4194,17 @@
       </c>
       <c r="H15" s="10" t="inlineStr">
         <is>
-          <t>Worked from Mysore residence</t>
+          <t>Local travel within Mysore</t>
         </is>
       </c>
       <c r="I15" s="10" t="inlineStr">
         <is>
-          <t>BACnet device simulation and UI analysis discussions along with recruitment coordination</t>
+          <t>Continued PRD planning and module discussions</t>
         </is>
       </c>
       <c r="J15" s="10" t="inlineStr">
         <is>
-          <t>gl-pbs</t>
+          <t>omnyx</t>
         </is>
       </c>
       <c r="K15" s="10" t="inlineStr">
@@ -4320,7 +4216,7 @@
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B16" s="10" t="inlineStr">
@@ -4328,14 +4224,14 @@
           <t>Wednesday</t>
         </is>
       </c>
-      <c r="C16" s="14" t="inlineStr">
-        <is>
-          <t>WFH</t>
+      <c r="C16" s="11" t="inlineStr">
+        <is>
+          <t>Discussion</t>
         </is>
       </c>
       <c r="D16" s="10" t="inlineStr">
         <is>
-          <t>Mysore</t>
+          <t>NA Group Office Mysore</t>
         </is>
       </c>
       <c r="E16" s="10" t="inlineStr"/>
@@ -4351,12 +4247,12 @@
       </c>
       <c r="H16" s="10" t="inlineStr">
         <is>
-          <t>Worked from Mysore residence</t>
+          <t>Local travel within Mysore</t>
         </is>
       </c>
       <c r="I16" s="10" t="inlineStr">
         <is>
-          <t>Interface and workflow architecture study and recruitment activities</t>
+          <t>Finalized PRD discussions and architecture workflows</t>
         </is>
       </c>
       <c r="J16" s="10" t="inlineStr">
@@ -4373,7 +4269,7 @@
     <row r="17">
       <c r="A17" s="10" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B17" s="10" t="inlineStr">
@@ -4381,7 +4277,7 @@
           <t>Thursday</t>
         </is>
       </c>
-      <c r="C17" s="14" t="inlineStr">
+      <c r="C17" s="12" t="inlineStr">
         <is>
           <t>WFH</t>
         </is>
@@ -4392,41 +4288,25 @@
         </is>
       </c>
       <c r="E17" s="10" t="inlineStr"/>
-      <c r="F17" s="10" t="inlineStr">
-        <is>
-          <t>10:00 AM</t>
-        </is>
-      </c>
-      <c r="G17" s="10" t="inlineStr">
-        <is>
-          <t>6:00 PM</t>
-        </is>
-      </c>
-      <c r="H17" s="10" t="inlineStr">
-        <is>
-          <t>Worked from Mysore residence</t>
-        </is>
-      </c>
+      <c r="F17" s="10" t="inlineStr"/>
+      <c r="G17" s="10" t="inlineStr"/>
+      <c r="H17" s="10" t="inlineStr"/>
       <c r="I17" s="10" t="inlineStr">
         <is>
-          <t>Technical coordination discussions ETL follow-ups and recruitment process handling</t>
-        </is>
-      </c>
-      <c r="J17" s="10" t="inlineStr">
-        <is>
-          <t>python-etl</t>
-        </is>
-      </c>
+          <t>Lingotran task + recruitment interviews for RAPL and Examic.</t>
+        </is>
+      </c>
+      <c r="J17" s="10" t="inlineStr"/>
       <c r="K17" s="10" t="inlineStr">
         <is>
-          <t>csv</t>
+          <t>manual</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="10" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="B18" s="10" t="inlineStr">
@@ -4434,42 +4314,42 @@
           <t>Friday</t>
         </is>
       </c>
-      <c r="C18" s="14" t="inlineStr">
-        <is>
-          <t>WFH</t>
+      <c r="C18" s="13" t="inlineStr">
+        <is>
+          <t>Office</t>
         </is>
       </c>
       <c r="D18" s="10" t="inlineStr">
         <is>
-          <t>Mysore</t>
-        </is>
-      </c>
-      <c r="E18" s="10" t="inlineStr"/>
+          <t>Graylinx Office Bangalore</t>
+        </is>
+      </c>
+      <c r="E18" s="10" t="inlineStr">
+        <is>
+          <t>GRS Hotel</t>
+        </is>
+      </c>
       <c r="F18" s="10" t="inlineStr">
         <is>
-          <t>10:00 AM</t>
+          <t>9:30 AM</t>
         </is>
       </c>
       <c r="G18" s="10" t="inlineStr">
         <is>
-          <t>6:00 PM</t>
+          <t>6:30 PM</t>
         </is>
       </c>
       <c r="H18" s="10" t="inlineStr">
         <is>
-          <t>Worked from Mysore residence</t>
+          <t>Mysore to Bangalore</t>
         </is>
       </c>
       <c r="I18" s="10" t="inlineStr">
         <is>
-          <t>Transformer layer follow-up discussions and recruitment coordination activities</t>
-        </is>
-      </c>
-      <c r="J18" s="10" t="inlineStr">
-        <is>
-          <t>python-etl</t>
-        </is>
-      </c>
+          <t>Worked with Vishnu before his Australia travel and discussed ongoing tasks</t>
+        </is>
+      </c>
+      <c r="J18" s="10" t="inlineStr"/>
       <c r="K18" s="10" t="inlineStr">
         <is>
           <t>csv</t>
@@ -4479,7 +4359,7 @@
     <row r="19">
       <c r="A19" s="10" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B19" s="10" t="inlineStr">
@@ -4487,40 +4367,44 @@
           <t>Saturday</t>
         </is>
       </c>
-      <c r="C19" s="14" t="inlineStr">
-        <is>
-          <t>WFH</t>
+      <c r="C19" s="13" t="inlineStr">
+        <is>
+          <t>Office</t>
         </is>
       </c>
       <c r="D19" s="10" t="inlineStr">
         <is>
-          <t>Mysore</t>
-        </is>
-      </c>
-      <c r="E19" s="10" t="inlineStr"/>
+          <t>Graylinx Office Bangalore</t>
+        </is>
+      </c>
+      <c r="E19" s="10" t="inlineStr">
+        <is>
+          <t>GRS Hotel</t>
+        </is>
+      </c>
       <c r="F19" s="10" t="inlineStr">
         <is>
-          <t>10:00 AM</t>
+          <t>9:30 AM</t>
         </is>
       </c>
       <c r="G19" s="10" t="inlineStr">
         <is>
-          <t>5:00 PM</t>
+          <t>6:00 PM</t>
         </is>
       </c>
       <c r="H19" s="10" t="inlineStr">
         <is>
-          <t>Worked from Mysore residence</t>
+          <t>Bangalore to Mysore</t>
         </is>
       </c>
       <c r="I19" s="10" t="inlineStr">
         <is>
-          <t>ETL and conversion workflow discussions along with interview coordination</t>
+          <t>Returned to Mysore after architecture discussions and AI demonstrations</t>
         </is>
       </c>
       <c r="J19" s="10" t="inlineStr">
         <is>
-          <t>python-etl</t>
+          <t>thermynx</t>
         </is>
       </c>
       <c r="K19" s="10" t="inlineStr">
@@ -4532,7 +4416,7 @@
     <row r="20">
       <c r="A20" s="10" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B20" s="10" t="inlineStr">
@@ -4540,7 +4424,7 @@
           <t>Sunday</t>
         </is>
       </c>
-      <c r="C20" s="14" t="inlineStr">
+      <c r="C20" s="12" t="inlineStr">
         <is>
           <t>WFH</t>
         </is>
@@ -4558,7 +4442,7 @@
       </c>
       <c r="G20" s="10" t="inlineStr">
         <is>
-          <t>4:00 PM</t>
+          <t>5:00 PM</t>
         </is>
       </c>
       <c r="H20" s="10" t="inlineStr">
@@ -4568,14 +4452,10 @@
       </c>
       <c r="I20" s="10" t="inlineStr">
         <is>
-          <t>Pending task coordination architecture planning and recruitment follow-ups</t>
-        </is>
-      </c>
-      <c r="J20" s="10" t="inlineStr">
-        <is>
-          <t>current-works</t>
-        </is>
-      </c>
+          <t>Continued assigned tasks remotely and coordinated pending work</t>
+        </is>
+      </c>
+      <c r="J20" s="10" t="inlineStr"/>
       <c r="K20" s="10" t="inlineStr">
         <is>
           <t>csv</t>
@@ -4585,7 +4465,7 @@
     <row r="21">
       <c r="A21" s="10" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="B21" s="10" t="inlineStr">
@@ -4593,7 +4473,7 @@
           <t>Monday</t>
         </is>
       </c>
-      <c r="C21" s="14" t="inlineStr">
+      <c r="C21" s="12" t="inlineStr">
         <is>
           <t>WFH</t>
         </is>
@@ -4621,12 +4501,12 @@
       </c>
       <c r="I21" s="10" t="inlineStr">
         <is>
-          <t>Continued ETL transformer layer planning discussions and recruitment activities</t>
+          <t>Existing BACnet simulation flow understanding discussions with team</t>
         </is>
       </c>
       <c r="J21" s="10" t="inlineStr">
         <is>
-          <t>python-etl</t>
+          <t>gl-pbs</t>
         </is>
       </c>
       <c r="K21" s="10" t="inlineStr">
@@ -4638,7 +4518,7 @@
     <row r="22">
       <c r="A22" s="10" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B22" s="10" t="inlineStr">
@@ -4646,7 +4526,7 @@
           <t>Tuesday</t>
         </is>
       </c>
-      <c r="C22" s="14" t="inlineStr">
+      <c r="C22" s="12" t="inlineStr">
         <is>
           <t>WFH</t>
         </is>
@@ -4674,12 +4554,12 @@
       </c>
       <c r="I22" s="10" t="inlineStr">
         <is>
-          <t>Follow-up discussions architecture coordination and recruitment processes</t>
+          <t>BACnet device simulation and UI analysis discussions along with recruitment coordination</t>
         </is>
       </c>
       <c r="J22" s="10" t="inlineStr">
         <is>
-          <t>current-works</t>
+          <t>gl-pbs</t>
         </is>
       </c>
       <c r="K22" s="10" t="inlineStr">
@@ -4691,7 +4571,7 @@
     <row r="23">
       <c r="A23" s="10" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B23" s="10" t="inlineStr">
@@ -4699,7 +4579,7 @@
           <t>Wednesday</t>
         </is>
       </c>
-      <c r="C23" s="14" t="inlineStr">
+      <c r="C23" s="12" t="inlineStr">
         <is>
           <t>WFH</t>
         </is>
@@ -4727,12 +4607,12 @@
       </c>
       <c r="I23" s="10" t="inlineStr">
         <is>
-          <t>Continued ETL transformer planning pending clarifications and recruitment coordination</t>
+          <t>Interface and workflow architecture study and recruitment activities</t>
         </is>
       </c>
       <c r="J23" s="10" t="inlineStr">
         <is>
-          <t>python-etl</t>
+          <t>omnyx</t>
         </is>
       </c>
       <c r="K23" s="10" t="inlineStr">
@@ -4744,7 +4624,7 @@
     <row r="24">
       <c r="A24" s="10" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="B24" s="10" t="inlineStr">
@@ -4752,7 +4632,7 @@
           <t>Thursday</t>
         </is>
       </c>
-      <c r="C24" s="14" t="inlineStr">
+      <c r="C24" s="12" t="inlineStr">
         <is>
           <t>WFH</t>
         </is>
@@ -4780,12 +4660,12 @@
       </c>
       <c r="I24" s="10" t="inlineStr">
         <is>
-          <t>Technical discussions implementation planning and interview coordination</t>
+          <t>Technical coordination discussions ETL follow-ups and recruitment process handling</t>
         </is>
       </c>
       <c r="J24" s="10" t="inlineStr">
         <is>
-          <t>current-works</t>
+          <t>python-etl</t>
         </is>
       </c>
       <c r="K24" s="10" t="inlineStr">
@@ -4797,7 +4677,7 @@
     <row r="25">
       <c r="A25" s="10" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B25" s="10" t="inlineStr">
@@ -4805,7 +4685,7 @@
           <t>Friday</t>
         </is>
       </c>
-      <c r="C25" s="14" t="inlineStr">
+      <c r="C25" s="12" t="inlineStr">
         <is>
           <t>WFH</t>
         </is>
@@ -4833,12 +4713,12 @@
       </c>
       <c r="I25" s="10" t="inlineStr">
         <is>
-          <t>Continued project coordination follow-ups and recruitment activities</t>
+          <t>Transformer layer follow-up discussions and recruitment coordination activities</t>
         </is>
       </c>
       <c r="J25" s="10" t="inlineStr">
         <is>
-          <t>current-works</t>
+          <t>python-etl</t>
         </is>
       </c>
       <c r="K25" s="10" t="inlineStr">
@@ -4850,7 +4730,7 @@
     <row r="26">
       <c r="A26" s="10" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B26" s="10" t="inlineStr">
@@ -4858,7 +4738,7 @@
           <t>Saturday</t>
         </is>
       </c>
-      <c r="C26" s="14" t="inlineStr">
+      <c r="C26" s="12" t="inlineStr">
         <is>
           <t>WFH</t>
         </is>
@@ -4886,7 +4766,7 @@
       </c>
       <c r="I26" s="10" t="inlineStr">
         <is>
-          <t>Ongoing ETL architecture planning discussions and recruitment work</t>
+          <t>ETL and conversion workflow discussions along with interview coordination</t>
         </is>
       </c>
       <c r="J26" s="10" t="inlineStr">
@@ -4903,7 +4783,7 @@
     <row r="27">
       <c r="A27" s="10" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B27" s="10" t="inlineStr">
@@ -4911,7 +4791,7 @@
           <t>Sunday</t>
         </is>
       </c>
-      <c r="C27" s="14" t="inlineStr">
+      <c r="C27" s="12" t="inlineStr">
         <is>
           <t>WFH</t>
         </is>
@@ -4939,7 +4819,7 @@
       </c>
       <c r="I27" s="10" t="inlineStr">
         <is>
-          <t>Pending workflow coordination architecture discussions and recruitment coordination</t>
+          <t>Pending task coordination architecture planning and recruitment follow-ups</t>
         </is>
       </c>
       <c r="J27" s="10" t="inlineStr">
@@ -4956,7 +4836,7 @@
     <row r="28">
       <c r="A28" s="10" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B28" s="10" t="inlineStr">
@@ -4964,7 +4844,7 @@
           <t>Monday</t>
         </is>
       </c>
-      <c r="C28" s="14" t="inlineStr">
+      <c r="C28" s="12" t="inlineStr">
         <is>
           <t>WFH</t>
         </is>
@@ -4992,12 +4872,12 @@
       </c>
       <c r="I28" s="10" t="inlineStr">
         <is>
-          <t>Continued follow-ups project discussions and recruitment coordination</t>
+          <t>Continued ETL transformer layer planning discussions and recruitment activities</t>
         </is>
       </c>
       <c r="J28" s="10" t="inlineStr">
         <is>
-          <t>current-works</t>
+          <t>python-etl</t>
         </is>
       </c>
       <c r="K28" s="10" t="inlineStr">
@@ -5009,7 +4889,7 @@
     <row r="29">
       <c r="A29" s="10" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B29" s="10" t="inlineStr">
@@ -5017,40 +4897,52 @@
           <t>Tuesday</t>
         </is>
       </c>
-      <c r="C29" s="14" t="inlineStr">
+      <c r="C29" s="12" t="inlineStr">
         <is>
           <t>WFH</t>
         </is>
       </c>
       <c r="D29" s="10" t="inlineStr">
         <is>
-          <t>Mysore (residence)</t>
+          <t>Mysore</t>
         </is>
       </c>
       <c r="E29" s="10" t="inlineStr"/>
-      <c r="F29" s="10" t="inlineStr"/>
-      <c r="G29" s="10" t="inlineStr"/>
-      <c r="H29" s="10" t="inlineStr"/>
+      <c r="F29" s="10" t="inlineStr">
+        <is>
+          <t>10:00 AM</t>
+        </is>
+      </c>
+      <c r="G29" s="10" t="inlineStr">
+        <is>
+          <t>6:00 PM</t>
+        </is>
+      </c>
+      <c r="H29" s="10" t="inlineStr">
+        <is>
+          <t>Worked from Mysore residence</t>
+        </is>
+      </c>
       <c r="I29" s="10" t="inlineStr">
         <is>
-          <t>OMNYX [9]: docs: PROJECT_OVERVIEW.md — vision, legacy comparison, transformation story; docs: ARCHITECTURE_RATIONALE.md — pros, cons, risk register, on-site scenarios; docs: align all MD docs with 2-DB architecture + Alloy/Kafka images (+6 more)  (9 commits)</t>
+          <t>Follow-up discussions architecture coordination and recruitment processes</t>
         </is>
       </c>
       <c r="J29" s="10" t="inlineStr">
         <is>
-          <t>omnyx</t>
+          <t>current-works</t>
         </is>
       </c>
       <c r="K29" s="10" t="inlineStr">
         <is>
-          <t>derived</t>
+          <t>csv</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="10" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B30" s="10" t="inlineStr">
@@ -5058,40 +4950,52 @@
           <t>Wednesday</t>
         </is>
       </c>
-      <c r="C30" s="14" t="inlineStr">
+      <c r="C30" s="12" t="inlineStr">
         <is>
           <t>WFH</t>
         </is>
       </c>
       <c r="D30" s="10" t="inlineStr">
         <is>
-          <t>Mysore (residence)</t>
+          <t>Mysore</t>
         </is>
       </c>
       <c r="E30" s="10" t="inlineStr"/>
-      <c r="F30" s="10" t="inlineStr"/>
-      <c r="G30" s="10" t="inlineStr"/>
-      <c r="H30" s="10" t="inlineStr"/>
+      <c r="F30" s="10" t="inlineStr">
+        <is>
+          <t>10:00 AM</t>
+        </is>
+      </c>
+      <c r="G30" s="10" t="inlineStr">
+        <is>
+          <t>6:00 PM</t>
+        </is>
+      </c>
+      <c r="H30" s="10" t="inlineStr">
+        <is>
+          <t>Worked from Mysore residence</t>
+        </is>
+      </c>
       <c r="I30" s="10" t="inlineStr">
         <is>
-          <t>THERMYNX [1]: feat: implement full-stack HVAC AI operations platform with multi-agent orchestr  (1 commits)</t>
+          <t>Continued ETL transformer planning pending clarifications and recruitment coordination</t>
         </is>
       </c>
       <c r="J30" s="10" t="inlineStr">
         <is>
-          <t>thermynx</t>
+          <t>python-etl</t>
         </is>
       </c>
       <c r="K30" s="10" t="inlineStr">
         <is>
-          <t>derived</t>
+          <t>csv</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="10" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B31" s="10" t="inlineStr">
@@ -5099,40 +5003,52 @@
           <t>Thursday</t>
         </is>
       </c>
-      <c r="C31" s="14" t="inlineStr">
+      <c r="C31" s="12" t="inlineStr">
         <is>
           <t>WFH</t>
         </is>
       </c>
       <c r="D31" s="10" t="inlineStr">
         <is>
-          <t>Mysore (residence)</t>
+          <t>Mysore</t>
         </is>
       </c>
       <c r="E31" s="10" t="inlineStr"/>
-      <c r="F31" s="10" t="inlineStr"/>
-      <c r="G31" s="10" t="inlineStr"/>
-      <c r="H31" s="10" t="inlineStr"/>
+      <c r="F31" s="10" t="inlineStr">
+        <is>
+          <t>10:00 AM</t>
+        </is>
+      </c>
+      <c r="G31" s="10" t="inlineStr">
+        <is>
+          <t>6:00 PM</t>
+        </is>
+      </c>
+      <c r="H31" s="10" t="inlineStr">
+        <is>
+          <t>Worked from Mysore residence</t>
+        </is>
+      </c>
       <c r="I31" s="10" t="inlineStr">
         <is>
-          <t>THERMYNX [12]: feat: add architecture documentation and configure environment-specific Claude s; docs(ai): mark Tier 1/2/3 + Perf T1 + Reliability R1/R4 + Eval Phase 1 as shippe; fix(eval+ui): action-verb regex tolerates articles + vite proxy env-driven (+9 more) · Nesso [5]: docs: add comprehensive developer setup guide and link it in README; docs: initialize README.md with project overview, architecture, and documentatio; docs: add comprehensive project implementation plan and detailed screen inventor (+2 more)  (17 commits)</t>
+          <t>Technical discussions implementation planning and interview coordination</t>
         </is>
       </c>
       <c r="J31" s="10" t="inlineStr">
         <is>
-          <t>thermynx</t>
+          <t>current-works</t>
         </is>
       </c>
       <c r="K31" s="10" t="inlineStr">
         <is>
-          <t>derived</t>
+          <t>csv</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="10" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B32" s="10" t="inlineStr">
@@ -5140,40 +5056,52 @@
           <t>Friday</t>
         </is>
       </c>
-      <c r="C32" s="14" t="inlineStr">
+      <c r="C32" s="12" t="inlineStr">
         <is>
           <t>WFH</t>
         </is>
       </c>
       <c r="D32" s="10" t="inlineStr">
         <is>
-          <t>Mysore (residence)</t>
+          <t>Mysore</t>
         </is>
       </c>
       <c r="E32" s="10" t="inlineStr"/>
-      <c r="F32" s="10" t="inlineStr"/>
-      <c r="G32" s="10" t="inlineStr"/>
-      <c r="H32" s="10" t="inlineStr"/>
+      <c r="F32" s="10" t="inlineStr">
+        <is>
+          <t>10:00 AM</t>
+        </is>
+      </c>
+      <c r="G32" s="10" t="inlineStr">
+        <is>
+          <t>6:00 PM</t>
+        </is>
+      </c>
+      <c r="H32" s="10" t="inlineStr">
+        <is>
+          <t>Worked from Mysore residence</t>
+        </is>
+      </c>
       <c r="I32" s="10" t="inlineStr">
         <is>
-          <t>Nesso [8]: feat: implement activities dashboard and logging interface with API integration; feat(phase-3): crops + activities + catalog (POP + inputs) backend; feat(phase-2): web admin UI for farmers — dashboard shell, list, detail, approva (+5 more)  (8 commits)</t>
+          <t>Continued project coordination follow-ups and recruitment activities</t>
         </is>
       </c>
       <c r="J32" s="10" t="inlineStr">
         <is>
-          <t>farmer-app</t>
+          <t>current-works</t>
         </is>
       </c>
       <c r="K32" s="10" t="inlineStr">
         <is>
-          <t>derived</t>
+          <t>csv</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="10" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B33" s="10" t="inlineStr">
@@ -5181,40 +5109,52 @@
           <t>Saturday</t>
         </is>
       </c>
-      <c r="C33" s="14" t="inlineStr">
+      <c r="C33" s="12" t="inlineStr">
         <is>
           <t>WFH</t>
         </is>
       </c>
       <c r="D33" s="10" t="inlineStr">
         <is>
-          <t>Mysore (residence)</t>
+          <t>Mysore</t>
         </is>
       </c>
       <c r="E33" s="10" t="inlineStr"/>
-      <c r="F33" s="10" t="inlineStr"/>
-      <c r="G33" s="10" t="inlineStr"/>
-      <c r="H33" s="10" t="inlineStr"/>
+      <c r="F33" s="10" t="inlineStr">
+        <is>
+          <t>10:00 AM</t>
+        </is>
+      </c>
+      <c r="G33" s="10" t="inlineStr">
+        <is>
+          <t>5:00 PM</t>
+        </is>
+      </c>
+      <c r="H33" s="10" t="inlineStr">
+        <is>
+          <t>Worked from Mysore residence</t>
+        </is>
+      </c>
       <c r="I33" s="10" t="inlineStr">
         <is>
-          <t>Nesso [68]: feat(mobile): real in-app support + live multi-language (no more "coming soon"); fix(mobile/login): bulletproof layout + themed + add missing elements; feat(mobile): app-wide dark mode — light/dark token system + working toggles ✅ (+65 more)  (68 commits)</t>
+          <t>Ongoing ETL architecture planning discussions and recruitment work</t>
         </is>
       </c>
       <c r="J33" s="10" t="inlineStr">
         <is>
-          <t>farmer-app</t>
+          <t>python-etl</t>
         </is>
       </c>
       <c r="K33" s="10" t="inlineStr">
         <is>
-          <t>derived</t>
+          <t>csv</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="10" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B34" s="10" t="inlineStr">
@@ -5222,40 +5162,52 @@
           <t>Sunday</t>
         </is>
       </c>
-      <c r="C34" s="14" t="inlineStr">
+      <c r="C34" s="12" t="inlineStr">
         <is>
           <t>WFH</t>
         </is>
       </c>
       <c r="D34" s="10" t="inlineStr">
         <is>
-          <t>Mysore (residence)</t>
+          <t>Mysore</t>
         </is>
       </c>
       <c r="E34" s="10" t="inlineStr"/>
-      <c r="F34" s="10" t="inlineStr"/>
-      <c r="G34" s="10" t="inlineStr"/>
-      <c r="H34" s="10" t="inlineStr"/>
+      <c r="F34" s="10" t="inlineStr">
+        <is>
+          <t>10:00 AM</t>
+        </is>
+      </c>
+      <c r="G34" s="10" t="inlineStr">
+        <is>
+          <t>4:00 PM</t>
+        </is>
+      </c>
+      <c r="H34" s="10" t="inlineStr">
+        <is>
+          <t>Worked from Mysore residence</t>
+        </is>
+      </c>
       <c r="I34" s="10" t="inlineStr">
         <is>
-          <t>Nesso [30]: perf(P2): web chart code-split, portal OG metadata, mobile FlatList tuning; fix(mobile): revert moti from dashboard — restore stable plain View KPI cards; docs: mark Phase 6/production ON HOLD until user says (P5 banner) (+27 more)  (30 commits)</t>
+          <t>Pending workflow coordination architecture discussions and recruitment coordination</t>
         </is>
       </c>
       <c r="J34" s="10" t="inlineStr">
         <is>
-          <t>farmer-app</t>
+          <t>current-works</t>
         </is>
       </c>
       <c r="K34" s="10" t="inlineStr">
         <is>
-          <t>derived</t>
+          <t>csv</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="B35" s="10" t="inlineStr">
@@ -5263,40 +5215,52 @@
           <t>Monday</t>
         </is>
       </c>
-      <c r="C35" s="14" t="inlineStr">
+      <c r="C35" s="12" t="inlineStr">
         <is>
           <t>WFH</t>
         </is>
       </c>
       <c r="D35" s="10" t="inlineStr">
         <is>
-          <t>Mysore (residence)</t>
+          <t>Mysore</t>
         </is>
       </c>
       <c r="E35" s="10" t="inlineStr"/>
-      <c r="F35" s="10" t="inlineStr"/>
-      <c r="G35" s="10" t="inlineStr"/>
-      <c r="H35" s="10" t="inlineStr"/>
+      <c r="F35" s="10" t="inlineStr">
+        <is>
+          <t>10:00 AM</t>
+        </is>
+      </c>
+      <c r="G35" s="10" t="inlineStr">
+        <is>
+          <t>6:00 PM</t>
+        </is>
+      </c>
+      <c r="H35" s="10" t="inlineStr">
+        <is>
+          <t>Worked from Mysore residence</t>
+        </is>
+      </c>
       <c r="I35" s="10" t="inlineStr">
         <is>
-          <t>OMNYX [40]: presentation: fix file:// security warning — embed logo as data URI; presentation: top-only navigation, no bottom nav, BOM stripped, better highlight; presentation: remove left section sidebar — full-width deck (+37 more) · Nesso [34]: feat(web-vite): MiniMap is now a real map (Leaflet+OSM, open-source, no key); docs: add INTEGRATIONS.md (APIs/CDNs/keys) + migration status; perf(web-vite): swap recharts-&gt;ECharts (tree-shaken) + lazy-load heavy routes (+31 more) · THERMYNX [10]: docs(ai): ADR for per-task LLM right-sizing decision; chore(ollama): bump MAX_LOADED_MODELS=3 + pre-warm hot set on restart; feat(ai): right-size models per task in config defaults (+7 more)  (84 commits)</t>
+          <t>Continued follow-ups project discussions and recruitment coordination</t>
         </is>
       </c>
       <c r="J35" s="10" t="inlineStr">
         <is>
-          <t>omnyx</t>
+          <t>current-works</t>
         </is>
       </c>
       <c r="K35" s="10" t="inlineStr">
         <is>
-          <t>derived</t>
+          <t>csv</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="10" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B36" s="10" t="inlineStr">
@@ -5304,7 +5268,7 @@
           <t>Tuesday</t>
         </is>
       </c>
-      <c r="C36" s="14" t="inlineStr">
+      <c r="C36" s="12" t="inlineStr">
         <is>
           <t>WFH</t>
         </is>
@@ -5320,7 +5284,7 @@
       <c r="H36" s="10" t="inlineStr"/>
       <c r="I36" s="10" t="inlineStr">
         <is>
-          <t>OMNYX [24]: docs(dev): keep ws-bridge in Docker when running api/web locally; style(frontend): new graphite + Klein palette, WCAG AA tuned for both modes; chore(dev): park Keycloak behind phase2 profile; add local hot-reload dev workfl (+21 more) · THERMYNX [10]: docs(ai): sync AI discovery docs and update README to 2026-06-02 final state; docs: add AI discovery documentation and local development settings; docs(ai): deprioritize Grafana/Prometheus dashboard panels — metrics already emi (+7 more) · Nesso [6]: docs(testing): update roles/logins doc for Vite cutover; feat(web-vite): full shell UI/UX parity with the design; fix(web-vite): Leaflet crash + LoginPage navigate-in-render (+3 more)  (40 commits)</t>
+          <t>OMNYX [9]: docs: PROJECT_OVERVIEW.md — vision, legacy comparison, transformation story; docs: ARCHITECTURE_RATIONALE.md — pros, cons, risk register, on-site scenarios; docs: align all MD docs with 2-DB architecture + Alloy/Kafka images (+6 more)  (9 commits)</t>
         </is>
       </c>
       <c r="J36" s="10" t="inlineStr">
@@ -5337,7 +5301,7 @@
     <row r="37">
       <c r="A37" s="10" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B37" s="10" t="inlineStr">
@@ -5345,7 +5309,7 @@
           <t>Wednesday</t>
         </is>
       </c>
-      <c r="C37" s="14" t="inlineStr">
+      <c r="C37" s="12" t="inlineStr">
         <is>
           <t>WFH</t>
         </is>
@@ -5361,12 +5325,12 @@
       <c r="H37" s="10" t="inlineStr"/>
       <c r="I37" s="10" t="inlineStr">
         <is>
-          <t>OMNYX [55]: feat(protocols): multi-protocol DAL — MQTT + Modbus + OPC-UA adapters; feat(rag): pgvector knowledge base — ingestion + agent retrieval [Phase 2]; feat(phase2): MinIO data lake + Airflow — working telemetry archive (+52 more) · Nesso [39]: feat(mobile): preflight checker + progress logging + timeouts in dev launcher; feat(web-vite): i18n increment — localize all page titles (en/kn/hi); fix(web-vite): responsive audit — stack field grid + scroll calendar on mobile (+36 more) · TripTrail [5]: Fix RLS infinite recursion: SECURITY DEFINER on policy helper functions; Fix totals trigger infinite recursion (pg_trigger_depth guard); Live: join user for employee_name/department; add re-runnable demo seed (+2 more)  (99 commits)</t>
+          <t>THERMYNX [1]: feat: implement full-stack HVAC AI operations platform with multi-agent orchestr  (1 commits)</t>
         </is>
       </c>
       <c r="J37" s="10" t="inlineStr">
         <is>
-          <t>omnyx</t>
+          <t>thermynx</t>
         </is>
       </c>
       <c r="K37" s="10" t="inlineStr">
@@ -5378,7 +5342,7 @@
     <row r="38">
       <c r="A38" s="10" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B38" s="10" t="inlineStr">
@@ -5386,7 +5350,7 @@
           <t>Thursday</t>
         </is>
       </c>
-      <c r="C38" s="14" t="inlineStr">
+      <c r="C38" s="12" t="inlineStr">
         <is>
           <t>WFH</t>
         </is>
@@ -5402,12 +5366,12 @@
       <c r="H38" s="10" t="inlineStr"/>
       <c r="I38" s="10" t="inlineStr">
         <is>
-          <t>Current Works in GL [16]: docs: add stress test summary report; docs: add Decision section to 1-page summary report; docs: update comparison and 1-page summary with all scales including 4000x and 5 (+13 more) · OMNYX [13]: docs(openapi): regenerate spec snapshots (adds /api/v1/analysis/correlation); chore: gitignore tsbuildinfo + egg-info build artifacts Co-Authored-By: Claude O; feat(analysis): device signal-correlation page + API (+10 more) · THERMYNX [6]: fix: H6+H7+H8 — forecast backend signal, agent history, is_running cast; feat(ui): work-order approve/dismiss card in agent trace (H3); fix(critical): C1+H1+H2+C3 — thread safety, tool injection, connection leak, mes (+3 more)  (35 commits)</t>
+          <t>THERMYNX [12]: feat: add architecture documentation and configure environment-specific Claude s; docs(ai): mark Tier 1/2/3 + Perf T1 + Reliability R1/R4 + Eval Phase 1 as shippe; fix(eval+ui): action-verb regex tolerates articles + vite proxy env-driven (+9 more) · Nesso [5]: docs: add comprehensive developer setup guide and link it in README; docs: initialize README.md with project overview, architecture, and documentatio; docs: add comprehensive project implementation plan and detailed screen inventor (+2 more)  (17 commits)</t>
         </is>
       </c>
       <c r="J38" s="10" t="inlineStr">
         <is>
-          <t>current-works</t>
+          <t>thermynx</t>
         </is>
       </c>
       <c r="K38" s="10" t="inlineStr">
@@ -5419,7 +5383,7 @@
     <row r="39">
       <c r="A39" s="10" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B39" s="10" t="inlineStr">
@@ -5427,7 +5391,7 @@
           <t>Friday</t>
         </is>
       </c>
-      <c r="C39" s="14" t="inlineStr">
+      <c r="C39" s="12" t="inlineStr">
         <is>
           <t>WFH</t>
         </is>
@@ -5443,12 +5407,12 @@
       <c r="H39" s="10" t="inlineStr"/>
       <c r="I39" s="10" t="inlineStr">
         <is>
-          <t>OMNYX [33]: feat: real energy/efficiency KPIs from catalog semantics (Gap 1); docs(site): point onboarding/multi-tenancy/simulator docs at the generator + Mer; chore(console): cut over to Console v2 — promote frontend-next, archive legacy,  (+30 more) · THERMYNX [13]: refactor(ai): consolidate prompts + share JSON parser (P1); bump NL-SQL timeout; feat(predictive): trend-based degradation -&gt; auto-proposed PM work orders; fix(ai): reconcile kW/TR 'fair' threshold drift in prompts (+10 more)  (46 commits)</t>
+          <t>Nesso [8]: feat: implement activities dashboard and logging interface with API integration; feat(phase-3): crops + activities + catalog (POP + inputs) backend; feat(phase-2): web admin UI for farmers — dashboard shell, list, detail, approva (+5 more)  (8 commits)</t>
         </is>
       </c>
       <c r="J39" s="10" t="inlineStr">
         <is>
-          <t>omnyx</t>
+          <t>farmer-app</t>
         </is>
       </c>
       <c r="K39" s="10" t="inlineStr">
@@ -5460,7 +5424,7 @@
     <row r="40">
       <c r="A40" s="10" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B40" s="10" t="inlineStr">
@@ -5468,7 +5432,7 @@
           <t>Saturday</t>
         </is>
       </c>
-      <c r="C40" s="14" t="inlineStr">
+      <c r="C40" s="12" t="inlineStr">
         <is>
           <t>WFH</t>
         </is>
@@ -5484,12 +5448,12 @@
       <c r="H40" s="10" t="inlineStr"/>
       <c r="I40" s="10" t="inlineStr">
         <is>
-          <t>OMNYX [12]: docs(showcase): sync omnyx.html to delivered work; test(e2e): console v2 + reports persistence + control shadow checks; feat(console): report history/generate + RL control-actions card (+9 more) · THERMYNX [12]: feat(cmms): Phase 1C Alarm -&gt; Work Order management; feat(ems): Phase 1B Energy Management + Cost; feat(ui): THERMYNX sibling theme — real thermal-cyan signature accent (+9 more)  (24 commits)</t>
+          <t>Nesso [68]: feat(mobile): real in-app support + live multi-language (no more "coming soon"); fix(mobile/login): bulletproof layout + themed + add missing elements; feat(mobile): app-wide dark mode — light/dark token system + working toggles ✅ (+65 more)  (68 commits)</t>
         </is>
       </c>
       <c r="J40" s="10" t="inlineStr">
         <is>
-          <t>omnyx</t>
+          <t>farmer-app</t>
         </is>
       </c>
       <c r="K40" s="10" t="inlineStr">
@@ -5501,7 +5465,7 @@
     <row r="41">
       <c r="A41" s="10" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B41" s="10" t="inlineStr">
@@ -5509,7 +5473,7 @@
           <t>Sunday</t>
         </is>
       </c>
-      <c r="C41" s="14" t="inlineStr">
+      <c r="C41" s="12" t="inlineStr">
         <is>
           <t>WFH</t>
         </is>
@@ -5525,12 +5489,12 @@
       <c r="H41" s="10" t="inlineStr"/>
       <c r="I41" s="10" t="inlineStr">
         <is>
-          <t>OMNYX [27]: feat: implement hvac vertical extension with agent-backed telemetry, twin predic; feat: implement initial docker-compose infra, airflow integration, and core serv; fix(security): pin RLS tenant in agentic-ai under the omnyx_svc role (+24 more)  (27 commits)</t>
+          <t>Nesso [30]: perf(P2): web chart code-split, portal OG metadata, mobile FlatList tuning; fix(mobile): revert moti from dashboard — restore stable plain View KPI cards; docs: mark Phase 6/production ON HOLD until user says (P5 banner) (+27 more)  (30 commits)</t>
         </is>
       </c>
       <c r="J41" s="10" t="inlineStr">
         <is>
-          <t>omnyx</t>
+          <t>farmer-app</t>
         </is>
       </c>
       <c r="K41" s="10" t="inlineStr">
@@ -5542,7 +5506,7 @@
     <row r="42">
       <c r="A42" s="10" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B42" s="10" t="inlineStr">
@@ -5550,7 +5514,7 @@
           <t>Monday</t>
         </is>
       </c>
-      <c r="C42" s="14" t="inlineStr">
+      <c r="C42" s="12" t="inlineStr">
         <is>
           <t>WFH</t>
         </is>
@@ -5566,12 +5530,12 @@
       <c r="H42" s="10" t="inlineStr"/>
       <c r="I42" s="10" t="inlineStr">
         <is>
-          <t>THERMYNX [14]: chore: add backend runtime logs and IDE settings configuration files; fix(ai): substitute mistral-small3.2 for phi4 — phi4-14B crashes Ollama 0.30.6; feat(ui): readable model roster + modernized 'model in use' toast (+11 more)  (14 commits)</t>
+          <t>OMNYX [40]: presentation: fix file:// security warning — embed logo as data URI; presentation: top-only navigation, no bottom nav, BOM stripped, better highlight; presentation: remove left section sidebar — full-width deck (+37 more) · Nesso [34]: feat(web-vite): MiniMap is now a real map (Leaflet+OSM, open-source, no key); docs: add INTEGRATIONS.md (APIs/CDNs/keys) + migration status; perf(web-vite): swap recharts-&gt;ECharts (tree-shaken) + lazy-load heavy routes (+31 more) · THERMYNX [10]: docs(ai): ADR for per-task LLM right-sizing decision; chore(ollama): bump MAX_LOADED_MODELS=3 + pre-warm hot set on restart; feat(ai): right-size models per task in config defaults (+7 more)  (84 commits)</t>
         </is>
       </c>
       <c r="J42" s="10" t="inlineStr">
         <is>
-          <t>thermynx</t>
+          <t>omnyx</t>
         </is>
       </c>
       <c r="K42" s="10" t="inlineStr">
@@ -5583,7 +5547,7 @@
     <row r="43">
       <c r="A43" s="10" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B43" s="10" t="inlineStr">
@@ -5591,7 +5555,7 @@
           <t>Tuesday</t>
         </is>
       </c>
-      <c r="C43" s="14" t="inlineStr">
+      <c r="C43" s="12" t="inlineStr">
         <is>
           <t>WFH</t>
         </is>
@@ -5607,12 +5571,12 @@
       <c r="H43" s="10" t="inlineStr"/>
       <c r="I43" s="10" t="inlineStr">
         <is>
-          <t>THERMYNX [6]: build(agentic): F0 — OSS agentic runtime + eval/test dependency manifests; docs(agentic): fold model-eval routing, performance must-holds, OSS-software lic; docs(agentic): framework rewrite plan, target architecture, ADR-0002, gap re-aud (+3 more) · OMNYX [1]: docs: add OMNYX project handbook and master documentation index  (7 commits)</t>
+          <t>OMNYX [24]: docs(dev): keep ws-bridge in Docker when running api/web locally; style(frontend): new graphite + Klein palette, WCAG AA tuned for both modes; chore(dev): park Keycloak behind phase2 profile; add local hot-reload dev workfl (+21 more) · THERMYNX [10]: docs(ai): sync AI discovery docs and update README to 2026-06-02 final state; docs: add AI discovery documentation and local development settings; docs(ai): deprioritize Grafana/Prometheus dashboard panels — metrics already emi (+7 more) · Nesso [6]: docs(testing): update roles/logins doc for Vite cutover; feat(web-vite): full shell UI/UX parity with the design; fix(web-vite): Leaflet crash + LoginPage navigate-in-render (+3 more)  (40 commits)</t>
         </is>
       </c>
       <c r="J43" s="10" t="inlineStr">
         <is>
-          <t>thermynx</t>
+          <t>omnyx</t>
         </is>
       </c>
       <c r="K43" s="10" t="inlineStr">
@@ -5624,7 +5588,7 @@
     <row r="44">
       <c r="A44" s="10" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B44" s="10" t="inlineStr">
@@ -5632,7 +5596,7 @@
           <t>Wednesday</t>
         </is>
       </c>
-      <c r="C44" s="14" t="inlineStr">
+      <c r="C44" s="12" t="inlineStr">
         <is>
           <t>WFH</t>
         </is>
@@ -5648,12 +5612,12 @@
       <c r="H44" s="10" t="inlineStr"/>
       <c r="I44" s="10" t="inlineStr">
         <is>
-          <t>THERMYNX [40]: feat: add custom environment settings and initial AgentRunner implementation; fix(anomaly): stop 'LLM timeout' on causal cards — warm model + headroom + keep_; chore(claude): expand tool allowlist accumulated this session (+37 more)  (40 commits)</t>
+          <t>OMNYX [55]: feat(protocols): multi-protocol DAL — MQTT + Modbus + OPC-UA adapters; feat(rag): pgvector knowledge base — ingestion + agent retrieval [Phase 2]; feat(phase2): MinIO data lake + Airflow — working telemetry archive (+52 more) · Nesso [39]: feat(mobile): preflight checker + progress logging + timeouts in dev launcher; feat(web-vite): i18n increment — localize all page titles (en/kn/hi); fix(web-vite): responsive audit — stack field grid + scroll calendar on mobile (+36 more) · TripTrail [5]: Fix RLS infinite recursion: SECURITY DEFINER on policy helper functions; Fix totals trigger infinite recursion (pg_trigger_depth guard); Live: join user for employee_name/department; add re-runnable demo seed (+2 more)  (99 commits)</t>
         </is>
       </c>
       <c r="J44" s="10" t="inlineStr">
         <is>
-          <t>thermynx</t>
+          <t>omnyx</t>
         </is>
       </c>
       <c r="K44" s="10" t="inlineStr">
@@ -5665,7 +5629,7 @@
     <row r="45">
       <c r="A45" s="10" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B45" s="10" t="inlineStr">
@@ -5673,7 +5637,7 @@
           <t>Thursday</t>
         </is>
       </c>
-      <c r="C45" s="14" t="inlineStr">
+      <c r="C45" s="12" t="inlineStr">
         <is>
           <t>WFH</t>
         </is>
@@ -5689,12 +5653,12 @@
       <c r="H45" s="10" t="inlineStr"/>
       <c r="I45" s="10" t="inlineStr">
         <is>
-          <t>THERMYNX [25]: chore(obs): comment out the langfuse SDK; mark tracing disabled / future-only; chore(frontend): remove orphaned migration-leftover components (zero imports); docs(agentic): F4.9 HITL done; F1.11 durable checkpointer deferred to 48/64GB (+22 more) · OMNYX [1]: docs(ops): flag shared Ollama GPU with THERMYNX (avoid VRAM eviction)  (26 commits)</t>
+          <t>Current Works in GL [16]: docs: add stress test summary report; docs: add Decision section to 1-page summary report; docs: update comparison and 1-page summary with all scales including 4000x and 5 (+13 more) · OMNYX [13]: docs(openapi): regenerate spec snapshots (adds /api/v1/analysis/correlation); chore: gitignore tsbuildinfo + egg-info build artifacts Co-Authored-By: Claude O; feat(analysis): device signal-correlation page + API (+10 more) · THERMYNX [6]: fix: H6+H7+H8 — forecast backend signal, agent history, is_running cast; feat(ui): work-order approve/dismiss card in agent trace (H3); fix(critical): C1+H1+H2+C3 — thread safety, tool injection, connection leak, mes (+3 more)  (35 commits)</t>
         </is>
       </c>
       <c r="J45" s="10" t="inlineStr">
         <is>
-          <t>thermynx</t>
+          <t>current-works</t>
         </is>
       </c>
       <c r="K45" s="10" t="inlineStr">
@@ -5706,7 +5670,7 @@
     <row r="46">
       <c r="A46" s="10" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B46" s="10" t="inlineStr">
@@ -5714,7 +5678,7 @@
           <t>Friday</t>
         </is>
       </c>
-      <c r="C46" s="14" t="inlineStr">
+      <c r="C46" s="12" t="inlineStr">
         <is>
           <t>WFH</t>
         </is>
@@ -5730,12 +5694,12 @@
       <c r="H46" s="10" t="inlineStr"/>
       <c r="I46" s="10" t="inlineStr">
         <is>
-          <t>THERMYNX [9]: docs(agentic): Session 3 handoff (2026-06-12); fix(eval): pre-push no longer auto-runs the golden suite (it floods the 20 GB GP; feat(agent): per-node timing traces (lightweight, no Langfuse/infra) (+6 more)  (9 commits)</t>
+          <t>OMNYX [33]: feat: real energy/efficiency KPIs from catalog semantics (Gap 1); docs(site): point onboarding/multi-tenancy/simulator docs at the generator + Mer; chore(console): cut over to Console v2 — promote frontend-next, archive legacy,  (+30 more) · THERMYNX [13]: refactor(ai): consolidate prompts + share JSON parser (P1); bump NL-SQL timeout; feat(predictive): trend-based degradation -&gt; auto-proposed PM work orders; fix(ai): reconcile kW/TR 'fair' threshold drift in prompts (+10 more)  (46 commits)</t>
         </is>
       </c>
       <c r="J46" s="10" t="inlineStr">
         <is>
-          <t>thermynx</t>
+          <t>omnyx</t>
         </is>
       </c>
       <c r="K46" s="10" t="inlineStr">
@@ -5747,7 +5711,7 @@
     <row r="47">
       <c r="A47" s="10" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B47" s="10" t="inlineStr">
@@ -5755,7 +5719,7 @@
           <t>Saturday</t>
         </is>
       </c>
-      <c r="C47" s="14" t="inlineStr">
+      <c r="C47" s="12" t="inlineStr">
         <is>
           <t>WFH</t>
         </is>
@@ -5771,12 +5735,12 @@
       <c r="H47" s="10" t="inlineStr"/>
       <c r="I47" s="10" t="inlineStr">
         <is>
-          <t>THERMYNX [6]: docs(agentic): loop-accurate plain-English overview + incidents log + Session-4 ; feat(frontend): Agent Lab workbench - tabbed Run/History/Compare/Tune/Validate +; feat(provider): OpenRouter dev-bridge provider switch (chat roles only; embeddin (+3 more)  (6 commits)</t>
+          <t>OMNYX [12]: docs(showcase): sync omnyx.html to delivered work; test(e2e): console v2 + reports persistence + control shadow checks; feat(console): report history/generate + RL control-actions card (+9 more) · THERMYNX [12]: feat(cmms): Phase 1C Alarm -&gt; Work Order management; feat(ems): Phase 1B Energy Management + Cost; feat(ui): THERMYNX sibling theme — real thermal-cyan signature accent (+9 more)  (24 commits)</t>
         </is>
       </c>
       <c r="J47" s="10" t="inlineStr">
         <is>
-          <t>thermynx</t>
+          <t>omnyx</t>
         </is>
       </c>
       <c r="K47" s="10" t="inlineStr">
@@ -5788,7 +5752,7 @@
     <row r="48">
       <c r="A48" s="10" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B48" s="10" t="inlineStr">
@@ -5796,24 +5760,40 @@
           <t>Sunday</t>
         </is>
       </c>
-      <c r="C48" s="15" t="inlineStr"/>
-      <c r="D48" s="10" t="inlineStr"/>
+      <c r="C48" s="12" t="inlineStr">
+        <is>
+          <t>WFH</t>
+        </is>
+      </c>
+      <c r="D48" s="10" t="inlineStr">
+        <is>
+          <t>Mysore (residence)</t>
+        </is>
+      </c>
       <c r="E48" s="10" t="inlineStr"/>
       <c r="F48" s="10" t="inlineStr"/>
       <c r="G48" s="10" t="inlineStr"/>
       <c r="H48" s="10" t="inlineStr"/>
-      <c r="I48" s="10" t="inlineStr"/>
-      <c r="J48" s="10" t="inlineStr"/>
+      <c r="I48" s="10" t="inlineStr">
+        <is>
+          <t>OMNYX [27]: feat: implement hvac vertical extension with agent-backed telemetry, twin predic; feat: implement initial docker-compose infra, airflow integration, and core serv; fix(security): pin RLS tenant in agentic-ai under the omnyx_svc role (+24 more)  (27 commits)</t>
+        </is>
+      </c>
+      <c r="J48" s="10" t="inlineStr">
+        <is>
+          <t>omnyx</t>
+        </is>
+      </c>
       <c r="K48" s="10" t="inlineStr">
         <is>
-          <t>needs-fill</t>
+          <t>derived</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="10" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B49" s="10" t="inlineStr">
@@ -5821,7 +5801,7 @@
           <t>Monday</t>
         </is>
       </c>
-      <c r="C49" s="14" t="inlineStr">
+      <c r="C49" s="12" t="inlineStr">
         <is>
           <t>WFH</t>
         </is>
@@ -5837,15 +5817,298 @@
       <c r="H49" s="10" t="inlineStr"/>
       <c r="I49" s="10" t="inlineStr">
         <is>
+          <t>THERMYNX [14]: chore: add backend runtime logs and IDE settings configuration files; fix(ai): substitute mistral-small3.2 for phi4 — phi4-14B crashes Ollama 0.30.6; feat(ui): readable model roster + modernized 'model in use' toast (+11 more)  (14 commits)</t>
+        </is>
+      </c>
+      <c r="J49" s="10" t="inlineStr">
+        <is>
+          <t>thermynx</t>
+        </is>
+      </c>
+      <c r="K49" s="10" t="inlineStr">
+        <is>
+          <t>derived</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B50" s="10" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="C50" s="12" t="inlineStr">
+        <is>
+          <t>WFH</t>
+        </is>
+      </c>
+      <c r="D50" s="10" t="inlineStr">
+        <is>
+          <t>Mysore (residence)</t>
+        </is>
+      </c>
+      <c r="E50" s="10" t="inlineStr"/>
+      <c r="F50" s="10" t="inlineStr"/>
+      <c r="G50" s="10" t="inlineStr"/>
+      <c r="H50" s="10" t="inlineStr"/>
+      <c r="I50" s="10" t="inlineStr">
+        <is>
+          <t>THERMYNX [6]: build(agentic): F0 — OSS agentic runtime + eval/test dependency manifests; docs(agentic): fold model-eval routing, performance must-holds, OSS-software lic; docs(agentic): framework rewrite plan, target architecture, ADR-0002, gap re-aud (+3 more) · OMNYX [1]: docs: add OMNYX project handbook and master documentation index  (7 commits)</t>
+        </is>
+      </c>
+      <c r="J50" s="10" t="inlineStr">
+        <is>
+          <t>thermynx</t>
+        </is>
+      </c>
+      <c r="K50" s="10" t="inlineStr">
+        <is>
+          <t>derived</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B51" s="10" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C51" s="12" t="inlineStr">
+        <is>
+          <t>WFH</t>
+        </is>
+      </c>
+      <c r="D51" s="10" t="inlineStr">
+        <is>
+          <t>Mysore (residence)</t>
+        </is>
+      </c>
+      <c r="E51" s="10" t="inlineStr"/>
+      <c r="F51" s="10" t="inlineStr"/>
+      <c r="G51" s="10" t="inlineStr"/>
+      <c r="H51" s="10" t="inlineStr"/>
+      <c r="I51" s="10" t="inlineStr">
+        <is>
+          <t>THERMYNX [40]: feat: add custom environment settings and initial AgentRunner implementation; fix(anomaly): stop 'LLM timeout' on causal cards — warm model + headroom + keep_; chore(claude): expand tool allowlist accumulated this session (+37 more)  (40 commits)</t>
+        </is>
+      </c>
+      <c r="J51" s="10" t="inlineStr">
+        <is>
+          <t>thermynx</t>
+        </is>
+      </c>
+      <c r="K51" s="10" t="inlineStr">
+        <is>
+          <t>derived</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B52" s="10" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="C52" s="12" t="inlineStr">
+        <is>
+          <t>WFH</t>
+        </is>
+      </c>
+      <c r="D52" s="10" t="inlineStr">
+        <is>
+          <t>Mysore (residence)</t>
+        </is>
+      </c>
+      <c r="E52" s="10" t="inlineStr"/>
+      <c r="F52" s="10" t="inlineStr"/>
+      <c r="G52" s="10" t="inlineStr"/>
+      <c r="H52" s="10" t="inlineStr"/>
+      <c r="I52" s="10" t="inlineStr">
+        <is>
+          <t>THERMYNX [25]: chore(obs): comment out the langfuse SDK; mark tracing disabled / future-only; chore(frontend): remove orphaned migration-leftover components (zero imports); docs(agentic): F4.9 HITL done; F1.11 durable checkpointer deferred to 48/64GB (+22 more) · OMNYX [1]: docs(ops): flag shared Ollama GPU with THERMYNX (avoid VRAM eviction)  (26 commits)</t>
+        </is>
+      </c>
+      <c r="J52" s="10" t="inlineStr">
+        <is>
+          <t>thermynx</t>
+        </is>
+      </c>
+      <c r="K52" s="10" t="inlineStr">
+        <is>
+          <t>derived</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="B53" s="10" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="C53" s="12" t="inlineStr">
+        <is>
+          <t>WFH</t>
+        </is>
+      </c>
+      <c r="D53" s="10" t="inlineStr">
+        <is>
+          <t>Mysore (residence)</t>
+        </is>
+      </c>
+      <c r="E53" s="10" t="inlineStr"/>
+      <c r="F53" s="10" t="inlineStr"/>
+      <c r="G53" s="10" t="inlineStr"/>
+      <c r="H53" s="10" t="inlineStr"/>
+      <c r="I53" s="10" t="inlineStr">
+        <is>
+          <t>THERMYNX [9]: docs(agentic): Session 3 handoff (2026-06-12); fix(eval): pre-push no longer auto-runs the golden suite (it floods the 20 GB GP; feat(agent): per-node timing traces (lightweight, no Langfuse/infra) (+6 more)  (9 commits)</t>
+        </is>
+      </c>
+      <c r="J53" s="10" t="inlineStr">
+        <is>
+          <t>thermynx</t>
+        </is>
+      </c>
+      <c r="K53" s="10" t="inlineStr">
+        <is>
+          <t>derived</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B54" s="10" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="C54" s="12" t="inlineStr">
+        <is>
+          <t>WFH</t>
+        </is>
+      </c>
+      <c r="D54" s="10" t="inlineStr">
+        <is>
+          <t>Mysore (residence)</t>
+        </is>
+      </c>
+      <c r="E54" s="10" t="inlineStr"/>
+      <c r="F54" s="10" t="inlineStr"/>
+      <c r="G54" s="10" t="inlineStr"/>
+      <c r="H54" s="10" t="inlineStr"/>
+      <c r="I54" s="10" t="inlineStr">
+        <is>
+          <t>THERMYNX [6]: docs(agentic): loop-accurate plain-English overview + incidents log + Session-4 ; feat(frontend): Agent Lab workbench - tabbed Run/History/Compare/Tune/Validate +; feat(provider): OpenRouter dev-bridge provider switch (chat roles only; embeddin (+3 more)  (6 commits)</t>
+        </is>
+      </c>
+      <c r="J54" s="10" t="inlineStr">
+        <is>
+          <t>thermynx</t>
+        </is>
+      </c>
+      <c r="K54" s="10" t="inlineStr">
+        <is>
+          <t>derived</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B55" s="10" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="C55" s="12" t="inlineStr">
+        <is>
+          <t>WFH</t>
+        </is>
+      </c>
+      <c r="D55" s="10" t="inlineStr">
+        <is>
+          <t>Mysore</t>
+        </is>
+      </c>
+      <c r="E55" s="10" t="inlineStr"/>
+      <c r="F55" s="10" t="inlineStr"/>
+      <c r="G55" s="10" t="inlineStr"/>
+      <c r="H55" s="10" t="inlineStr"/>
+      <c r="I55" s="10" t="inlineStr">
+        <is>
+          <t>Lingotran task + recruitment interviews for RAPL and Examic.</t>
+        </is>
+      </c>
+      <c r="J55" s="10" t="inlineStr"/>
+      <c r="K55" s="10" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B56" s="10" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="C56" s="12" t="inlineStr">
+        <is>
+          <t>WFH</t>
+        </is>
+      </c>
+      <c r="D56" s="10" t="inlineStr">
+        <is>
+          <t>Mysore (residence)</t>
+        </is>
+      </c>
+      <c r="E56" s="10" t="inlineStr"/>
+      <c r="F56" s="10" t="inlineStr"/>
+      <c r="G56" s="10" t="inlineStr"/>
+      <c r="H56" s="10" t="inlineStr"/>
+      <c r="I56" s="10" t="inlineStr">
+        <is>
           <t>THERMYNX [24]: feat: add .claude/settings.json with pre-configured shell execution permissions; feat(security): M9 recursive injection-hardening of tool results; Add architectural handbook for Graylinx LLM platform and initialize Claude proje (+21 more) · ClimaStream [1]: docs: add architecture and agentic flow diagrams to project documentation · Nesso [1]: chore: update lockfile to reflect dependency changes · OMNYX [1]: docs: initialize architecture, security, and roadmap documentation and implement  (27 commits)</t>
         </is>
       </c>
-      <c r="J49" s="10" t="inlineStr">
+      <c r="J56" s="10" t="inlineStr">
         <is>
           <t>thermynx</t>
         </is>
       </c>
-      <c r="K49" s="10" t="inlineStr">
+      <c r="K56" s="10" t="inlineStr">
         <is>
           <t>derived</t>
         </is>

</xml_diff>

<commit_message>
feat: Analytics view — how-much-worked metrics (busiest day, streak, commits/day) + project/category/week/work-type/status charts
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/works.xlsx
+++ b/works.xlsx
@@ -696,7 +696,7 @@
         <v>70</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
@@ -879,7 +879,7 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -938,12 +938,12 @@
       <c r="H6" s="2" t="inlineStr"/>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -1002,12 +1002,12 @@
       <c r="H7" s="2" t="inlineStr"/>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">

</xml_diff>

<commit_message>
feat(data): add GitHub-confirmed + 2025 email-POC works — graylinx.ai-hvac, legacy-analysis, HVAC pipeline POCs, Asset Mgmt/Kafka-MinIO; timeline now Oct 2025 -> Jun 2026 (25 projects, 887 commits)
GitHub server timestamps confirm code work is genuinely 2026 (not a clock bug); 2025 emails are the earlier POC phase.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/works.xlsx
+++ b/works.xlsx
@@ -520,13 +520,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R42"/>
+  <dimension ref="A1:R49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="17" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="47" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
     <col width="55" customWidth="1" min="6" max="6"/>
     <col width="55" customWidth="1" min="7" max="7"/>
@@ -3474,6 +3474,510 @@
       </c>
       <c r="Q42" s="6" t="inlineStr"/>
       <c r="R42" s="6" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>gl-hvac-early</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr"/>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>project</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>Graylinx.ai HVAC (early prototype)</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="inlineStr">
+        <is>
+          <t>HVAC Platform</t>
+        </is>
+      </c>
+      <c r="F43" s="4" t="inlineStr">
+        <is>
+          <t>"HVAC Data Pipeline v2" — first Graylinx HVAC repo (Python), precursor to ClimaStream.</t>
+        </is>
+      </c>
+      <c r="G43" s="4" t="inlineStr">
+        <is>
+          <t>Initial HVAC data-pipeline prototype.</t>
+        </is>
+      </c>
+      <c r="H43" s="4" t="inlineStr">
+        <is>
+          <t>Python</t>
+        </is>
+      </c>
+      <c r="I43" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="J43" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-21</t>
+        </is>
+      </c>
+      <c r="K43" s="4" t="inlineStr">
+        <is>
+          <t>github</t>
+        </is>
+      </c>
+      <c r="L43" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M43" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="N43" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="O43" s="4" t="inlineStr"/>
+      <c r="P43" s="4" t="inlineStr">
+        <is>
+          <t>First HVAC repo on GitHub (8 commits); Precursor to ClimaStream</t>
+        </is>
+      </c>
+      <c r="Q43" s="4" t="inlineStr"/>
+      <c r="R43" s="4" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>gl-legacy-analysis</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="inlineStr"/>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>project</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>Graylinx Legacy-Code Analysis</t>
+        </is>
+      </c>
+      <c r="E44" s="4" t="inlineStr">
+        <is>
+          <t>Graylinx Core</t>
+        </is>
+      </c>
+      <c r="F44" s="4" t="inlineStr">
+        <is>
+          <t>Audit/analysis of the Graylinx legacy codebase that informed the v2/OMNYX rebuild.</t>
+        </is>
+      </c>
+      <c r="G44" s="4" t="inlineStr">
+        <is>
+          <t>Reviewed &amp; documented legacy code for migration.</t>
+        </is>
+      </c>
+      <c r="H44" s="4" t="inlineStr">
+        <is>
+          <t>JavaScript; Node.js</t>
+        </is>
+      </c>
+      <c r="I44" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="J44" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="K44" s="4" t="inlineStr">
+        <is>
+          <t>github</t>
+        </is>
+      </c>
+      <c r="L44" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M44" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="N44" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="O44" s="4" t="inlineStr"/>
+      <c r="P44" s="4" t="inlineStr">
+        <is>
+          <t>Legacy code audit (7 commits); Fed into OMNYX architecture</t>
+        </is>
+      </c>
+      <c r="Q44" s="4" t="inlineStr"/>
+      <c r="R44" s="4" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>poc-hvac-pipeline</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="inlineStr"/>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
+          <t>project</t>
+        </is>
+      </c>
+      <c r="D45" s="4" t="inlineStr">
+        <is>
+          <t>HVAC Pipeline POCs (POC 1–3)</t>
+        </is>
+      </c>
+      <c r="E45" s="4" t="inlineStr">
+        <is>
+          <t>HVAC Platform</t>
+        </is>
+      </c>
+      <c r="F45" s="4" t="inlineStr">
+        <is>
+          <t>POC 1 &amp; 2 completed, POC 3 in discussion — HVAC data pipeline, the pre-implementation phase.</t>
+        </is>
+      </c>
+      <c r="G45" s="4" t="inlineStr">
+        <is>
+          <t>Drove the POCs with J. Suryanarayanan &amp; Satish Krishna (email-tracked milestones).</t>
+        </is>
+      </c>
+      <c r="H45" s="4" t="inlineStr">
+        <is>
+          <t>NodeJS; Kafka; MinIO; MySQL</t>
+        </is>
+      </c>
+      <c r="I45" s="4" t="inlineStr">
+        <is>
+          <t>2025-10-20</t>
+        </is>
+      </c>
+      <c r="J45" s="4" t="inlineStr">
+        <is>
+          <t>2025-11-27</t>
+        </is>
+      </c>
+      <c r="K45" s="4" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="L45" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M45" s="4" t="n">
+        <v>90</v>
+      </c>
+      <c r="N45" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O45" s="4" t="inlineStr"/>
+      <c r="P45" s="4" t="inlineStr">
+        <is>
+          <t>POC 1 &amp; 2 completed; POC 3 discussion; Milestone-tracked over email (Oct–Nov 2025)</t>
+        </is>
+      </c>
+      <c r="Q45" s="4" t="inlineStr"/>
+      <c r="R45" s="4" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>poc-asset-mgmt</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="inlineStr"/>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
+          <t>project</t>
+        </is>
+      </c>
+      <c r="D46" s="4" t="inlineStr">
+        <is>
+          <t>Asset Management POC — NodeJS → Kafka → MinIO</t>
+        </is>
+      </c>
+      <c r="E46" s="4" t="inlineStr">
+        <is>
+          <t>Graylinx Core</t>
+        </is>
+      </c>
+      <c r="F46" s="4" t="inlineStr">
+        <is>
+          <t>Asset-management ingestion POC: NodeJS → Kafka → MinIO with MySQL.</t>
+        </is>
+      </c>
+      <c r="G46" s="4" t="inlineStr">
+        <is>
+          <t>Designed table schema + ingestion flow (with Surya Narayanan).</t>
+        </is>
+      </c>
+      <c r="H46" s="4" t="inlineStr">
+        <is>
+          <t>NodeJS; Kafka; MinIO; MySQL</t>
+        </is>
+      </c>
+      <c r="I46" s="4" t="inlineStr">
+        <is>
+          <t>2025-11-07</t>
+        </is>
+      </c>
+      <c r="J46" s="4" t="inlineStr">
+        <is>
+          <t>2025-11-12</t>
+        </is>
+      </c>
+      <c r="K46" s="4" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="L46" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M46" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="N46" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O46" s="4" t="inlineStr"/>
+      <c r="P46" s="4" t="inlineStr">
+        <is>
+          <t>NodeJS → Kafka → MinIO pipeline; Nov 2025</t>
+        </is>
+      </c>
+      <c r="Q46" s="4" t="inlineStr"/>
+      <c r="R46" s="4" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>poc-kafka-minio</t>
+        </is>
+      </c>
+      <c r="B47" s="4" t="inlineStr"/>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>project</t>
+        </is>
+      </c>
+      <c r="D47" s="4" t="inlineStr">
+        <is>
+          <t>Kafka → MinIO Data Ingestion POC</t>
+        </is>
+      </c>
+      <c r="E47" s="4" t="inlineStr">
+        <is>
+          <t>Graylinx Core</t>
+        </is>
+      </c>
+      <c r="F47" s="4" t="inlineStr">
+        <is>
+          <t>Kafka-to-MinIO data ingestion POC — plan &amp; meeting summary.</t>
+        </is>
+      </c>
+      <c r="G47" s="4" t="inlineStr">
+        <is>
+          <t>Led the plan + meeting summary (with Raghunandan Srinath, Surya Narayanan).</t>
+        </is>
+      </c>
+      <c r="H47" s="4" t="inlineStr">
+        <is>
+          <t>Kafka; MinIO</t>
+        </is>
+      </c>
+      <c r="I47" s="4" t="inlineStr">
+        <is>
+          <t>2025-11-07</t>
+        </is>
+      </c>
+      <c r="J47" s="4" t="inlineStr">
+        <is>
+          <t>2025-11-07</t>
+        </is>
+      </c>
+      <c r="K47" s="4" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="L47" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M47" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="N47" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O47" s="4" t="inlineStr"/>
+      <c r="P47" s="4" t="inlineStr">
+        <is>
+          <t>Ingestion plan + meeting summary; Nov 2025</t>
+        </is>
+      </c>
+      <c r="Q47" s="4" t="inlineStr"/>
+      <c r="R47" s="4" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>poc-chiller</t>
+        </is>
+      </c>
+      <c r="B48" s="4" t="inlineStr"/>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>project</t>
+        </is>
+      </c>
+      <c r="D48" s="4" t="inlineStr">
+        <is>
+          <t>HVAC Chiller Plant Data Pipeline — POC 1</t>
+        </is>
+      </c>
+      <c r="E48" s="4" t="inlineStr">
+        <is>
+          <t>HVAC Platform</t>
+        </is>
+      </c>
+      <c r="F48" s="4" t="inlineStr">
+        <is>
+          <t>Chiller-plant data pipeline, POC 1.</t>
+        </is>
+      </c>
+      <c r="G48" s="4" t="inlineStr">
+        <is>
+          <t>Started POC 1 (aligned with J. Suryanarayanan).</t>
+        </is>
+      </c>
+      <c r="H48" s="4" t="inlineStr">
+        <is>
+          <t>NodeJS; Kafka</t>
+        </is>
+      </c>
+      <c r="I48" s="4" t="inlineStr">
+        <is>
+          <t>2025-11-14</t>
+        </is>
+      </c>
+      <c r="J48" s="4" t="inlineStr">
+        <is>
+          <t>2025-11-14</t>
+        </is>
+      </c>
+      <c r="K48" s="4" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="L48" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M48" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="N48" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O48" s="4" t="inlineStr"/>
+      <c r="P48" s="4" t="inlineStr">
+        <is>
+          <t>Chiller plant POC 1; Nov 2025</t>
+        </is>
+      </c>
+      <c r="Q48" s="4" t="inlineStr"/>
+      <c r="R48" s="4" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>rms-config</t>
+        </is>
+      </c>
+      <c r="B49" s="4" t="inlineStr"/>
+      <c r="C49" s="4" t="inlineStr">
+        <is>
+          <t>project</t>
+        </is>
+      </c>
+      <c r="D49" s="4" t="inlineStr">
+        <is>
+          <t>RMS Configuration</t>
+        </is>
+      </c>
+      <c r="E49" s="4" t="inlineStr">
+        <is>
+          <t>Infra &amp; Tooling</t>
+        </is>
+      </c>
+      <c r="F49" s="4" t="inlineStr">
+        <is>
+          <t>RMS configuration coordination across the Vyoda/Tanu and Nagesh teams.</t>
+        </is>
+      </c>
+      <c r="G49" s="4" t="inlineStr">
+        <is>
+          <t>Coordinated RMS configuration.</t>
+        </is>
+      </c>
+      <c r="H49" s="4" t="inlineStr">
+        <is>
+          <t>Config</t>
+        </is>
+      </c>
+      <c r="I49" s="4" t="inlineStr">
+        <is>
+          <t>2025-10-28</t>
+        </is>
+      </c>
+      <c r="J49" s="4" t="inlineStr">
+        <is>
+          <t>2025-10-28</t>
+        </is>
+      </c>
+      <c r="K49" s="4" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="L49" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M49" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="N49" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O49" s="4" t="inlineStr"/>
+      <c r="P49" s="4" t="inlineStr">
+        <is>
+          <t>RMS configuration; Oct 2025</t>
+        </is>
+      </c>
+      <c r="Q49" s="4" t="inlineStr"/>
+      <c r="R49" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat(data): HVAC Data Pipeline v1/v2 from harshan-aiyappa account (Nov 2025, Node->Kafka->MinIO->Airflow->ClickHouse->Grafana, 3 POC milestones) — resolves the 2025/2026 timeline
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/works.xlsx
+++ b/works.xlsx
@@ -520,13 +520,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R49"/>
+  <dimension ref="A1:R52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="47" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
     <col width="55" customWidth="1" min="6" max="6"/>
     <col width="55" customWidth="1" min="7" max="7"/>
@@ -3633,7 +3633,7 @@
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>HVAC Pipeline POCs (POC 1–3)</t>
+          <t>HVAC Data Pipeline (v1 &amp; v2)</t>
         </is>
       </c>
       <c r="E45" s="4" t="inlineStr">
@@ -3643,32 +3643,32 @@
       </c>
       <c r="F45" s="4" t="inlineStr">
         <is>
-          <t>POC 1 &amp; 2 completed, POC 3 in discussion — HVAC data pipeline, the pre-implementation phase.</t>
+          <t>Production HVAC telemetry pipeline: Node.js → MySQL + Kafka → MinIO (Parquet) → Airflow → ClickHouse → Grafana. Original build on the harshan-aiyappa GitHub account (Nov 2025).</t>
         </is>
       </c>
       <c r="G45" s="4" t="inlineStr">
         <is>
-          <t>Drove the POCs with J. Suryanarayanan &amp; Satish Krishna (email-tracked milestones).</t>
+          <t>Built the end-to-end pipeline + its 3 POCs with J. Suryanarayanan &amp; Satish Krishna; milestone-tracked over email.</t>
         </is>
       </c>
       <c r="H45" s="4" t="inlineStr">
         <is>
-          <t>NodeJS; Kafka; MinIO; MySQL</t>
+          <t>Node.js; Kafka; MinIO; Airflow; ClickHouse; Grafana; Python; Docker</t>
         </is>
       </c>
       <c r="I45" s="4" t="inlineStr">
         <is>
-          <t>2025-10-20</t>
+          <t>2025-11-19</t>
         </is>
       </c>
       <c r="J45" s="4" t="inlineStr">
         <is>
-          <t>2025-11-27</t>
+          <t>2025-11-26</t>
         </is>
       </c>
       <c r="K45" s="4" t="inlineStr">
         <is>
-          <t>email</t>
+          <t>github</t>
         </is>
       </c>
       <c r="L45" s="5" t="inlineStr">
@@ -3677,15 +3677,15 @@
         </is>
       </c>
       <c r="M45" s="4" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="N45" s="4" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="O45" s="4" t="inlineStr"/>
       <c r="P45" s="4" t="inlineStr">
         <is>
-          <t>POC 1 &amp; 2 completed; POC 3 discussion; Milestone-tracked over email (Oct–Nov 2025)</t>
+          <t>v1 (19 Nov) + v2 (26 Nov 2025) on the harshan-aiyappa account; Ingestion · Data Lake · Analytics POCs; Node→Kafka→MinIO→Airflow→ClickHouse→Grafana</t>
         </is>
       </c>
       <c r="Q45" s="4" t="inlineStr"/>
@@ -3694,53 +3694,49 @@
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>poc-asset-mgmt</t>
-        </is>
-      </c>
-      <c r="B46" s="4" t="inlineStr"/>
+          <t>poc-hvac-pipeline.1</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>poc-hvac-pipeline</t>
+        </is>
+      </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>project</t>
+          <t>milestone</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>Asset Management POC — NodeJS → Kafka → MinIO</t>
+          <t>POC 1 — Ingestion (Node.js → MySQL + Kafka)</t>
         </is>
       </c>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t>Graylinx Core</t>
+          <t>HVAC Platform</t>
         </is>
       </c>
       <c r="F46" s="4" t="inlineStr">
         <is>
-          <t>Asset-management ingestion POC: NodeJS → Kafka → MinIO with MySQL.</t>
-        </is>
-      </c>
-      <c r="G46" s="4" t="inlineStr">
-        <is>
-          <t>Designed table schema + ingestion flow (with Surya Narayanan).</t>
-        </is>
-      </c>
-      <c r="H46" s="4" t="inlineStr">
-        <is>
-          <t>NodeJS; Kafka; MinIO; MySQL</t>
-        </is>
-      </c>
+          <t>Simulator → Node.js service → MySQL + Kafka</t>
+        </is>
+      </c>
+      <c r="G46" s="4" t="inlineStr"/>
+      <c r="H46" s="4" t="inlineStr"/>
       <c r="I46" s="4" t="inlineStr">
         <is>
-          <t>2025-11-07</t>
+          <t>2025-11-19</t>
         </is>
       </c>
       <c r="J46" s="4" t="inlineStr">
         <is>
-          <t>2025-11-12</t>
+          <t>2025-11-21</t>
         </is>
       </c>
       <c r="K46" s="4" t="inlineStr">
         <is>
-          <t>email</t>
+          <t>github</t>
         </is>
       </c>
       <c r="L46" s="5" t="inlineStr">
@@ -3755,64 +3751,56 @@
         <v>0</v>
       </c>
       <c r="O46" s="4" t="inlineStr"/>
-      <c r="P46" s="4" t="inlineStr">
-        <is>
-          <t>NodeJS → Kafka → MinIO pipeline; Nov 2025</t>
-        </is>
-      </c>
+      <c r="P46" s="4" t="inlineStr"/>
       <c r="Q46" s="4" t="inlineStr"/>
       <c r="R46" s="4" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>poc-kafka-minio</t>
-        </is>
-      </c>
-      <c r="B47" s="4" t="inlineStr"/>
+          <t>poc-hvac-pipeline.2</t>
+        </is>
+      </c>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>poc-hvac-pipeline</t>
+        </is>
+      </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>project</t>
+          <t>milestone</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>Kafka → MinIO Data Ingestion POC</t>
+          <t>POC 2 — Data Lake (Kafka → MinIO/Parquet)</t>
         </is>
       </c>
       <c r="E47" s="4" t="inlineStr">
         <is>
-          <t>Graylinx Core</t>
+          <t>HVAC Platform</t>
         </is>
       </c>
       <c r="F47" s="4" t="inlineStr">
         <is>
-          <t>Kafka-to-MinIO data ingestion POC — plan &amp; meeting summary.</t>
-        </is>
-      </c>
-      <c r="G47" s="4" t="inlineStr">
-        <is>
-          <t>Led the plan + meeting summary (with Raghunandan Srinath, Surya Narayanan).</t>
-        </is>
-      </c>
-      <c r="H47" s="4" t="inlineStr">
-        <is>
-          <t>Kafka; MinIO</t>
-        </is>
-      </c>
+          <t>Kafka → connector → MinIO Parquet storage</t>
+        </is>
+      </c>
+      <c r="G47" s="4" t="inlineStr"/>
+      <c r="H47" s="4" t="inlineStr"/>
       <c r="I47" s="4" t="inlineStr">
         <is>
-          <t>2025-11-07</t>
+          <t>2025-11-21</t>
         </is>
       </c>
       <c r="J47" s="4" t="inlineStr">
         <is>
-          <t>2025-11-07</t>
+          <t>2025-11-23</t>
         </is>
       </c>
       <c r="K47" s="4" t="inlineStr">
         <is>
-          <t>email</t>
+          <t>github</t>
         </is>
       </c>
       <c r="L47" s="5" t="inlineStr">
@@ -3827,29 +3815,29 @@
         <v>0</v>
       </c>
       <c r="O47" s="4" t="inlineStr"/>
-      <c r="P47" s="4" t="inlineStr">
-        <is>
-          <t>Ingestion plan + meeting summary; Nov 2025</t>
-        </is>
-      </c>
+      <c r="P47" s="4" t="inlineStr"/>
       <c r="Q47" s="4" t="inlineStr"/>
       <c r="R47" s="4" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>poc-chiller</t>
-        </is>
-      </c>
-      <c r="B48" s="4" t="inlineStr"/>
+          <t>poc-hvac-pipeline.3</t>
+        </is>
+      </c>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>poc-hvac-pipeline</t>
+        </is>
+      </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>project</t>
+          <t>milestone</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr">
         <is>
-          <t>HVAC Chiller Plant Data Pipeline — POC 1</t>
+          <t>POC 3 — Analytics (Airflow → ClickHouse → Grafana)</t>
         </is>
       </c>
       <c r="E48" s="4" t="inlineStr">
@@ -3859,32 +3847,24 @@
       </c>
       <c r="F48" s="4" t="inlineStr">
         <is>
-          <t>Chiller-plant data pipeline, POC 1.</t>
-        </is>
-      </c>
-      <c r="G48" s="4" t="inlineStr">
-        <is>
-          <t>Started POC 1 (aligned with J. Suryanarayanan).</t>
-        </is>
-      </c>
-      <c r="H48" s="4" t="inlineStr">
-        <is>
-          <t>NodeJS; Kafka</t>
-        </is>
-      </c>
+          <t>MinIO → Airflow → ClickHouse → Grafana dashboards</t>
+        </is>
+      </c>
+      <c r="G48" s="4" t="inlineStr"/>
+      <c r="H48" s="4" t="inlineStr"/>
       <c r="I48" s="4" t="inlineStr">
         <is>
-          <t>2025-11-14</t>
+          <t>2025-11-23</t>
         </is>
       </c>
       <c r="J48" s="4" t="inlineStr">
         <is>
-          <t>2025-11-14</t>
+          <t>2025-11-26</t>
         </is>
       </c>
       <c r="K48" s="4" t="inlineStr">
         <is>
-          <t>email</t>
+          <t>github</t>
         </is>
       </c>
       <c r="L48" s="5" t="inlineStr">
@@ -3899,18 +3879,14 @@
         <v>0</v>
       </c>
       <c r="O48" s="4" t="inlineStr"/>
-      <c r="P48" s="4" t="inlineStr">
-        <is>
-          <t>Chiller plant POC 1; Nov 2025</t>
-        </is>
-      </c>
+      <c r="P48" s="4" t="inlineStr"/>
       <c r="Q48" s="4" t="inlineStr"/>
       <c r="R48" s="4" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>rms-config</t>
+          <t>poc-asset-mgmt</t>
         </is>
       </c>
       <c r="B49" s="4" t="inlineStr"/>
@@ -3921,37 +3897,37 @@
       </c>
       <c r="D49" s="4" t="inlineStr">
         <is>
-          <t>RMS Configuration</t>
+          <t>Asset Management POC — NodeJS → Kafka → MinIO</t>
         </is>
       </c>
       <c r="E49" s="4" t="inlineStr">
         <is>
-          <t>Infra &amp; Tooling</t>
+          <t>Graylinx Core</t>
         </is>
       </c>
       <c r="F49" s="4" t="inlineStr">
         <is>
-          <t>RMS configuration coordination across the Vyoda/Tanu and Nagesh teams.</t>
+          <t>Asset-management ingestion POC: NodeJS → Kafka → MinIO with MySQL.</t>
         </is>
       </c>
       <c r="G49" s="4" t="inlineStr">
         <is>
-          <t>Coordinated RMS configuration.</t>
+          <t>Designed table schema + ingestion flow (with Surya Narayanan).</t>
         </is>
       </c>
       <c r="H49" s="4" t="inlineStr">
         <is>
-          <t>Config</t>
+          <t>NodeJS; Kafka; MinIO; MySQL</t>
         </is>
       </c>
       <c r="I49" s="4" t="inlineStr">
         <is>
-          <t>2025-10-28</t>
+          <t>2025-11-07</t>
         </is>
       </c>
       <c r="J49" s="4" t="inlineStr">
         <is>
-          <t>2025-10-28</t>
+          <t>2025-11-12</t>
         </is>
       </c>
       <c r="K49" s="4" t="inlineStr">
@@ -3973,11 +3949,227 @@
       <c r="O49" s="4" t="inlineStr"/>
       <c r="P49" s="4" t="inlineStr">
         <is>
-          <t>RMS configuration; Oct 2025</t>
+          <t>NodeJS → Kafka → MinIO pipeline; Nov 2025</t>
         </is>
       </c>
       <c r="Q49" s="4" t="inlineStr"/>
       <c r="R49" s="4" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>poc-kafka-minio</t>
+        </is>
+      </c>
+      <c r="B50" s="4" t="inlineStr"/>
+      <c r="C50" s="4" t="inlineStr">
+        <is>
+          <t>project</t>
+        </is>
+      </c>
+      <c r="D50" s="4" t="inlineStr">
+        <is>
+          <t>Kafka → MinIO Data Ingestion POC</t>
+        </is>
+      </c>
+      <c r="E50" s="4" t="inlineStr">
+        <is>
+          <t>Graylinx Core</t>
+        </is>
+      </c>
+      <c r="F50" s="4" t="inlineStr">
+        <is>
+          <t>Kafka-to-MinIO data ingestion POC — plan &amp; meeting summary.</t>
+        </is>
+      </c>
+      <c r="G50" s="4" t="inlineStr">
+        <is>
+          <t>Led the plan + meeting summary (with Raghunandan Srinath, Surya Narayanan).</t>
+        </is>
+      </c>
+      <c r="H50" s="4" t="inlineStr">
+        <is>
+          <t>Kafka; MinIO</t>
+        </is>
+      </c>
+      <c r="I50" s="4" t="inlineStr">
+        <is>
+          <t>2025-11-07</t>
+        </is>
+      </c>
+      <c r="J50" s="4" t="inlineStr">
+        <is>
+          <t>2025-11-07</t>
+        </is>
+      </c>
+      <c r="K50" s="4" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="L50" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M50" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="N50" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O50" s="4" t="inlineStr"/>
+      <c r="P50" s="4" t="inlineStr">
+        <is>
+          <t>Ingestion plan + meeting summary; Nov 2025</t>
+        </is>
+      </c>
+      <c r="Q50" s="4" t="inlineStr"/>
+      <c r="R50" s="4" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>poc-chiller</t>
+        </is>
+      </c>
+      <c r="B51" s="4" t="inlineStr"/>
+      <c r="C51" s="4" t="inlineStr">
+        <is>
+          <t>project</t>
+        </is>
+      </c>
+      <c r="D51" s="4" t="inlineStr">
+        <is>
+          <t>HVAC Chiller Plant Data Pipeline — POC 1</t>
+        </is>
+      </c>
+      <c r="E51" s="4" t="inlineStr">
+        <is>
+          <t>HVAC Platform</t>
+        </is>
+      </c>
+      <c r="F51" s="4" t="inlineStr">
+        <is>
+          <t>Chiller-plant data pipeline, POC 1.</t>
+        </is>
+      </c>
+      <c r="G51" s="4" t="inlineStr">
+        <is>
+          <t>Started POC 1 (aligned with J. Suryanarayanan).</t>
+        </is>
+      </c>
+      <c r="H51" s="4" t="inlineStr">
+        <is>
+          <t>NodeJS; Kafka</t>
+        </is>
+      </c>
+      <c r="I51" s="4" t="inlineStr">
+        <is>
+          <t>2025-11-14</t>
+        </is>
+      </c>
+      <c r="J51" s="4" t="inlineStr">
+        <is>
+          <t>2025-11-14</t>
+        </is>
+      </c>
+      <c r="K51" s="4" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="L51" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M51" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="N51" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O51" s="4" t="inlineStr"/>
+      <c r="P51" s="4" t="inlineStr">
+        <is>
+          <t>Chiller plant POC 1; Nov 2025</t>
+        </is>
+      </c>
+      <c r="Q51" s="4" t="inlineStr"/>
+      <c r="R51" s="4" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>rms-config</t>
+        </is>
+      </c>
+      <c r="B52" s="4" t="inlineStr"/>
+      <c r="C52" s="4" t="inlineStr">
+        <is>
+          <t>project</t>
+        </is>
+      </c>
+      <c r="D52" s="4" t="inlineStr">
+        <is>
+          <t>RMS Configuration</t>
+        </is>
+      </c>
+      <c r="E52" s="4" t="inlineStr">
+        <is>
+          <t>Infra &amp; Tooling</t>
+        </is>
+      </c>
+      <c r="F52" s="4" t="inlineStr">
+        <is>
+          <t>RMS configuration coordination across the Vyoda/Tanu and Nagesh teams.</t>
+        </is>
+      </c>
+      <c r="G52" s="4" t="inlineStr">
+        <is>
+          <t>Coordinated RMS configuration.</t>
+        </is>
+      </c>
+      <c r="H52" s="4" t="inlineStr">
+        <is>
+          <t>Config</t>
+        </is>
+      </c>
+      <c r="I52" s="4" t="inlineStr">
+        <is>
+          <t>2025-10-28</t>
+        </is>
+      </c>
+      <c r="J52" s="4" t="inlineStr">
+        <is>
+          <t>2025-10-28</t>
+        </is>
+      </c>
+      <c r="K52" s="4" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="L52" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M52" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="N52" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O52" s="4" t="inlineStr"/>
+      <c r="P52" s="4" t="inlineStr">
+        <is>
+          <t>RMS configuration; Oct 2025</t>
+        </is>
+      </c>
+      <c r="Q52" s="4" t="inlineStr"/>
+      <c r="R52" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
refactor(data): merge HVAC POC duplicates into the real Chiller-Plant pipeline (v1/v2, harshan-aiyappa) enriched from repo READMEs
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/works.xlsx
+++ b/works.xlsx
@@ -520,7 +520,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R52"/>
+  <dimension ref="A1:R49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -696,7 +696,7 @@
         <v>70</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
@@ -3643,7 +3643,7 @@
       </c>
       <c r="F45" s="4" t="inlineStr">
         <is>
-          <t>Production HVAC telemetry pipeline: Node.js → MySQL + Kafka → MinIO (Parquet) → Airflow → ClickHouse → Grafana. Original build on the harshan-aiyappa GitHub account (Nov 2025).</t>
+          <t>Graylinx HVAC Chiller-Plant telemetry pipeline: Node.js → MySQL + Kafka → MinIO (Parquet + manifests) → Airflow → ClickHouse → Grafana. v1 + production-ready v2 on the harshan-aiyappa account (Nov 2025).</t>
         </is>
       </c>
       <c r="G45" s="4" t="inlineStr">
@@ -3653,7 +3653,7 @@
       </c>
       <c r="H45" s="4" t="inlineStr">
         <is>
-          <t>Node.js; Kafka; MinIO; Airflow; ClickHouse; Grafana; Python; Docker</t>
+          <t>Node.js; Express; Kafka; MinIO; Parquet; Airflow; ClickHouse; Grafana; Python; Docker</t>
         </is>
       </c>
       <c r="I45" s="4" t="inlineStr">
@@ -3685,7 +3685,7 @@
       <c r="O45" s="4" t="inlineStr"/>
       <c r="P45" s="4" t="inlineStr">
         <is>
-          <t>v1 (19 Nov) + v2 (26 Nov 2025) on the harshan-aiyappa account; Ingestion · Data Lake · Analytics POCs; Node→Kafka→MinIO→Airflow→ClickHouse→Grafana</t>
+          <t>Chiller-plant predictive-maintenance + energy-optimization pipeline; v1 (19 Nov) + production v2 (26 Nov 2025), harshan-aiyappa account; POCs: Ingestion · Data Lake · Analytics</t>
         </is>
       </c>
       <c r="Q45" s="4" t="inlineStr"/>
@@ -3886,7 +3886,7 @@
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>poc-asset-mgmt</t>
+          <t>rms-config</t>
         </is>
       </c>
       <c r="B49" s="4" t="inlineStr"/>
@@ -3897,37 +3897,37 @@
       </c>
       <c r="D49" s="4" t="inlineStr">
         <is>
-          <t>Asset Management POC — NodeJS → Kafka → MinIO</t>
+          <t>RMS Configuration</t>
         </is>
       </c>
       <c r="E49" s="4" t="inlineStr">
         <is>
-          <t>Graylinx Core</t>
+          <t>Infra &amp; Tooling</t>
         </is>
       </c>
       <c r="F49" s="4" t="inlineStr">
         <is>
-          <t>Asset-management ingestion POC: NodeJS → Kafka → MinIO with MySQL.</t>
+          <t>RMS configuration coordination across the Vyoda/Tanu and Nagesh teams.</t>
         </is>
       </c>
       <c r="G49" s="4" t="inlineStr">
         <is>
-          <t>Designed table schema + ingestion flow (with Surya Narayanan).</t>
+          <t>Coordinated RMS configuration.</t>
         </is>
       </c>
       <c r="H49" s="4" t="inlineStr">
         <is>
-          <t>NodeJS; Kafka; MinIO; MySQL</t>
+          <t>Config</t>
         </is>
       </c>
       <c r="I49" s="4" t="inlineStr">
         <is>
-          <t>2025-11-07</t>
+          <t>2025-10-28</t>
         </is>
       </c>
       <c r="J49" s="4" t="inlineStr">
         <is>
-          <t>2025-11-12</t>
+          <t>2025-10-28</t>
         </is>
       </c>
       <c r="K49" s="4" t="inlineStr">
@@ -3949,227 +3949,11 @@
       <c r="O49" s="4" t="inlineStr"/>
       <c r="P49" s="4" t="inlineStr">
         <is>
-          <t>NodeJS → Kafka → MinIO pipeline; Nov 2025</t>
+          <t>RMS configuration; Oct 2025</t>
         </is>
       </c>
       <c r="Q49" s="4" t="inlineStr"/>
       <c r="R49" s="4" t="inlineStr"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="4" t="inlineStr">
-        <is>
-          <t>poc-kafka-minio</t>
-        </is>
-      </c>
-      <c r="B50" s="4" t="inlineStr"/>
-      <c r="C50" s="4" t="inlineStr">
-        <is>
-          <t>project</t>
-        </is>
-      </c>
-      <c r="D50" s="4" t="inlineStr">
-        <is>
-          <t>Kafka → MinIO Data Ingestion POC</t>
-        </is>
-      </c>
-      <c r="E50" s="4" t="inlineStr">
-        <is>
-          <t>Graylinx Core</t>
-        </is>
-      </c>
-      <c r="F50" s="4" t="inlineStr">
-        <is>
-          <t>Kafka-to-MinIO data ingestion POC — plan &amp; meeting summary.</t>
-        </is>
-      </c>
-      <c r="G50" s="4" t="inlineStr">
-        <is>
-          <t>Led the plan + meeting summary (with Raghunandan Srinath, Surya Narayanan).</t>
-        </is>
-      </c>
-      <c r="H50" s="4" t="inlineStr">
-        <is>
-          <t>Kafka; MinIO</t>
-        </is>
-      </c>
-      <c r="I50" s="4" t="inlineStr">
-        <is>
-          <t>2025-11-07</t>
-        </is>
-      </c>
-      <c r="J50" s="4" t="inlineStr">
-        <is>
-          <t>2025-11-07</t>
-        </is>
-      </c>
-      <c r="K50" s="4" t="inlineStr">
-        <is>
-          <t>email</t>
-        </is>
-      </c>
-      <c r="L50" s="5" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="M50" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="N50" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O50" s="4" t="inlineStr"/>
-      <c r="P50" s="4" t="inlineStr">
-        <is>
-          <t>Ingestion plan + meeting summary; Nov 2025</t>
-        </is>
-      </c>
-      <c r="Q50" s="4" t="inlineStr"/>
-      <c r="R50" s="4" t="inlineStr"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="4" t="inlineStr">
-        <is>
-          <t>poc-chiller</t>
-        </is>
-      </c>
-      <c r="B51" s="4" t="inlineStr"/>
-      <c r="C51" s="4" t="inlineStr">
-        <is>
-          <t>project</t>
-        </is>
-      </c>
-      <c r="D51" s="4" t="inlineStr">
-        <is>
-          <t>HVAC Chiller Plant Data Pipeline — POC 1</t>
-        </is>
-      </c>
-      <c r="E51" s="4" t="inlineStr">
-        <is>
-          <t>HVAC Platform</t>
-        </is>
-      </c>
-      <c r="F51" s="4" t="inlineStr">
-        <is>
-          <t>Chiller-plant data pipeline, POC 1.</t>
-        </is>
-      </c>
-      <c r="G51" s="4" t="inlineStr">
-        <is>
-          <t>Started POC 1 (aligned with J. Suryanarayanan).</t>
-        </is>
-      </c>
-      <c r="H51" s="4" t="inlineStr">
-        <is>
-          <t>NodeJS; Kafka</t>
-        </is>
-      </c>
-      <c r="I51" s="4" t="inlineStr">
-        <is>
-          <t>2025-11-14</t>
-        </is>
-      </c>
-      <c r="J51" s="4" t="inlineStr">
-        <is>
-          <t>2025-11-14</t>
-        </is>
-      </c>
-      <c r="K51" s="4" t="inlineStr">
-        <is>
-          <t>email</t>
-        </is>
-      </c>
-      <c r="L51" s="5" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="M51" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="N51" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O51" s="4" t="inlineStr"/>
-      <c r="P51" s="4" t="inlineStr">
-        <is>
-          <t>Chiller plant POC 1; Nov 2025</t>
-        </is>
-      </c>
-      <c r="Q51" s="4" t="inlineStr"/>
-      <c r="R51" s="4" t="inlineStr"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="4" t="inlineStr">
-        <is>
-          <t>rms-config</t>
-        </is>
-      </c>
-      <c r="B52" s="4" t="inlineStr"/>
-      <c r="C52" s="4" t="inlineStr">
-        <is>
-          <t>project</t>
-        </is>
-      </c>
-      <c r="D52" s="4" t="inlineStr">
-        <is>
-          <t>RMS Configuration</t>
-        </is>
-      </c>
-      <c r="E52" s="4" t="inlineStr">
-        <is>
-          <t>Infra &amp; Tooling</t>
-        </is>
-      </c>
-      <c r="F52" s="4" t="inlineStr">
-        <is>
-          <t>RMS configuration coordination across the Vyoda/Tanu and Nagesh teams.</t>
-        </is>
-      </c>
-      <c r="G52" s="4" t="inlineStr">
-        <is>
-          <t>Coordinated RMS configuration.</t>
-        </is>
-      </c>
-      <c r="H52" s="4" t="inlineStr">
-        <is>
-          <t>Config</t>
-        </is>
-      </c>
-      <c r="I52" s="4" t="inlineStr">
-        <is>
-          <t>2025-10-28</t>
-        </is>
-      </c>
-      <c r="J52" s="4" t="inlineStr">
-        <is>
-          <t>2025-10-28</t>
-        </is>
-      </c>
-      <c r="K52" s="4" t="inlineStr">
-        <is>
-          <t>email</t>
-        </is>
-      </c>
-      <c r="L52" s="5" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="M52" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="N52" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O52" s="4" t="inlineStr"/>
-      <c r="P52" s="4" t="inlineStr">
-        <is>
-          <t>RMS configuration; Oct 2025</t>
-        </is>
-      </c>
-      <c r="Q52" s="4" t="inlineStr"/>
-      <c r="R52" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
fix(data): remove unverified "RMS Configuration" project; correct timeline span to Nov 2025
The RMS Configuration entry traced to an email-evidenced works list, but its
description (Vyoda/Tanu/Nagesh teams) and single Oct-28-2025 date were unverified
placeholders. Commented it out in build_tracker.py (one-line restore) pending
confirmation of the real details.

Knock-on: RMS was the only October 2025 entry, so the timeline now starts
Nov 19 2025. Updated the hardcoded gantt label "Oct 2025" -> "Nov 2025".

Now 21 projects (was 22) - 903 commits - 55 engagement days - span Nov 19 2025 -> Jun 15 2026.
Rebuilt: works.csv/json/xlsx, seed re-injected, public/ synced.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/works.xlsx
+++ b/works.xlsx
@@ -520,7 +520,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R49"/>
+  <dimension ref="A1:R48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -696,7 +696,7 @@
         <v>70</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
@@ -3882,78 +3882,6 @@
       <c r="P48" s="4" t="inlineStr"/>
       <c r="Q48" s="4" t="inlineStr"/>
       <c r="R48" s="4" t="inlineStr"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="4" t="inlineStr">
-        <is>
-          <t>rms-config</t>
-        </is>
-      </c>
-      <c r="B49" s="4" t="inlineStr"/>
-      <c r="C49" s="4" t="inlineStr">
-        <is>
-          <t>project</t>
-        </is>
-      </c>
-      <c r="D49" s="4" t="inlineStr">
-        <is>
-          <t>RMS Configuration</t>
-        </is>
-      </c>
-      <c r="E49" s="4" t="inlineStr">
-        <is>
-          <t>Infra &amp; Tooling</t>
-        </is>
-      </c>
-      <c r="F49" s="4" t="inlineStr">
-        <is>
-          <t>RMS configuration coordination across the Vyoda/Tanu and Nagesh teams.</t>
-        </is>
-      </c>
-      <c r="G49" s="4" t="inlineStr">
-        <is>
-          <t>Coordinated RMS configuration.</t>
-        </is>
-      </c>
-      <c r="H49" s="4" t="inlineStr">
-        <is>
-          <t>Config</t>
-        </is>
-      </c>
-      <c r="I49" s="4" t="inlineStr">
-        <is>
-          <t>2025-10-28</t>
-        </is>
-      </c>
-      <c r="J49" s="4" t="inlineStr">
-        <is>
-          <t>2025-10-28</t>
-        </is>
-      </c>
-      <c r="K49" s="4" t="inlineStr">
-        <is>
-          <t>email</t>
-        </is>
-      </c>
-      <c r="L49" s="5" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="M49" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="N49" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O49" s="4" t="inlineStr"/>
-      <c r="P49" s="4" t="inlineStr">
-        <is>
-          <t>RMS configuration; Oct 2025</t>
-        </is>
-      </c>
-      <c r="Q49" s="4" t="inlineStr"/>
-      <c r="R49" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat(data): tag every project with an ownership scope (Graylinx / Personal / Client)
Adds a `scope` field so non-Graylinx work is distinguishable without removing it:
- Client (3): TripTrail (RANGSONS), Nesso (NR Group), Konva
- Personal (5): SelfAware Suite, SelfAware Dev Stack, VOXARA, Concept Standard, Raspberry
- Graylinx (13): everything else

build_tracker.py: SCOPE_BY_ID map -> scope_of(); scope on project+milestone rows;
added to PROJ_COLS (CSV/XLSX) and a projects_by_scope analytics breakdown.

index.html: scope badge on cards (colour on the dot only, label is the word -> AA-safe),
a Scope filter in the Projects toolbar, editable scope select in the project modal,
scope in JS export columns + save/add defaults.

21 projects unchanged; seed re-injected; public/ synced.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/works.xlsx
+++ b/works.xlsx
@@ -520,7 +520,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R48"/>
+  <dimension ref="A1:S48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -528,19 +528,20 @@
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="52" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="55" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
     <col width="55" customWidth="1" min="7" max="7"/>
     <col width="55" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="55" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="13" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="53" customWidth="1" min="15" max="15"/>
-    <col width="55" customWidth="1" min="16" max="16"/>
-    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="53" customWidth="1" min="16" max="16"/>
+    <col width="55" customWidth="1" min="17" max="17"/>
     <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="12" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -571,65 +572,70 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>scope</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>description</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>role</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>tech</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>start</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>end</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>date_source</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>progress</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>commits</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>location</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>highlights</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>links</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
@@ -659,57 +665,62 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
+          <t>Graylinx</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
           <t>AI-powered HVAC analytics POC for the Unicharm facility — local LLM, RAG, work orders and analytics.</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Sole engineer — full-stack build: FastAPI backend, React/TypeScript frontend, Ollama integration, analytics engine.</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>Python; FastAPI; React; TypeScript; Ollama; MySQL; Vite</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>2026-05-08</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>ongoing</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>git</t>
         </is>
       </c>
-      <c r="L2" s="3" t="inlineStr">
+      <c r="M2" s="3" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="M2" s="2" t="n">
+      <c r="N2" s="2" t="n">
         <v>70</v>
       </c>
-      <c r="N2" s="2" t="n">
-        <v>319</v>
-      </c>
-      <c r="O2" s="2" t="inlineStr">
+      <c r="O2" s="2" t="n">
+        <v>320</v>
+      </c>
+      <c r="P2" s="2" t="inlineStr">
         <is>
           <t>D:\Harshan\HVAC AI Operations Intelligence Platform</t>
         </is>
       </c>
-      <c r="P2" s="2" t="inlineStr">
+      <c r="Q2" s="2" t="inlineStr">
         <is>
           <t>Most active project — 308 commits; 18 feature pages + 6 Claude/LLM agents; RAG over facility docs, work-order workflow, analytics engine; Local on-prem LLM (Ollama) inference</t>
         </is>
       </c>
-      <c r="Q2" s="2" t="inlineStr"/>
       <c r="R2" s="2" t="inlineStr"/>
+      <c r="S2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -739,41 +750,46 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
+          <t>Graylinx</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
           <t>Frontend feature surface</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr"/>
       <c r="H3" s="2" t="inlineStr"/>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr"/>
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>2026-05-08</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>2026-05-15</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="L3" s="2" t="inlineStr">
         <is>
           <t>git</t>
         </is>
       </c>
-      <c r="L3" s="3" t="inlineStr">
+      <c r="M3" s="3" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="M3" s="2" t="n">
+      <c r="N3" s="2" t="n">
         <v>80</v>
       </c>
-      <c r="N3" s="2" t="n">
+      <c r="O3" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="O3" s="2" t="inlineStr"/>
       <c r="P3" s="2" t="inlineStr"/>
       <c r="Q3" s="2" t="inlineStr"/>
       <c r="R3" s="2" t="inlineStr"/>
+      <c r="S3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -803,41 +819,46 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
+          <t>Graylinx</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
           <t>Claude/LLM agents</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr"/>
       <c r="H4" s="2" t="inlineStr"/>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr"/>
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>2026-05-15</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>2026-05-23</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>git</t>
         </is>
       </c>
-      <c r="L4" s="3" t="inlineStr">
+      <c r="M4" s="3" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="M4" s="2" t="n">
+      <c r="N4" s="2" t="n">
         <v>70</v>
       </c>
-      <c r="N4" s="2" t="n">
+      <c r="O4" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="O4" s="2" t="inlineStr"/>
       <c r="P4" s="2" t="inlineStr"/>
       <c r="Q4" s="2" t="inlineStr"/>
       <c r="R4" s="2" t="inlineStr"/>
+      <c r="S4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -867,41 +888,46 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
+          <t>Graylinx</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
           <t>Retrieval over facility docs</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr"/>
       <c r="H5" s="2" t="inlineStr"/>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="I5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="inlineStr">
         <is>
           <t>2026-05-23</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr">
+      <c r="K5" s="2" t="inlineStr">
         <is>
           <t>2026-05-31</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr">
+      <c r="L5" s="2" t="inlineStr">
         <is>
           <t>git</t>
         </is>
       </c>
-      <c r="L5" s="3" t="inlineStr">
+      <c r="M5" s="3" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="M5" s="2" t="n">
+      <c r="N5" s="2" t="n">
         <v>65</v>
       </c>
-      <c r="N5" s="2" t="n">
+      <c r="O5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="O5" s="2" t="inlineStr"/>
       <c r="P5" s="2" t="inlineStr"/>
       <c r="Q5" s="2" t="inlineStr"/>
       <c r="R5" s="2" t="inlineStr"/>
+      <c r="S5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -931,41 +957,46 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
+          <t>Graylinx</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
           <t>Work-order workflow</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr"/>
       <c r="H6" s="2" t="inlineStr"/>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr"/>
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>2026-05-31</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>2026-06-08</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="L6" s="2" t="inlineStr">
         <is>
           <t>git</t>
         </is>
       </c>
-      <c r="L6" s="3" t="inlineStr">
+      <c r="M6" s="3" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="M6" s="2" t="n">
+      <c r="N6" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="N6" s="2" t="n">
+      <c r="O6" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="O6" s="2" t="inlineStr"/>
       <c r="P6" s="2" t="inlineStr"/>
       <c r="Q6" s="2" t="inlineStr"/>
       <c r="R6" s="2" t="inlineStr"/>
+      <c r="S6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -995,41 +1026,46 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
+          <t>Graylinx</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
           <t>Chiller/HVAC analytics</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr"/>
       <c r="H7" s="2" t="inlineStr"/>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr"/>
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>2026-06-08</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>2026-06-16</t>
         </is>
       </c>
-      <c r="K7" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>git</t>
         </is>
       </c>
-      <c r="L7" s="3" t="inlineStr">
+      <c r="M7" s="3" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="M7" s="2" t="n">
+      <c r="N7" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="N7" s="2" t="n">
+      <c r="O7" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="O7" s="2" t="inlineStr"/>
       <c r="P7" s="2" t="inlineStr"/>
       <c r="Q7" s="2" t="inlineStr"/>
       <c r="R7" s="2" t="inlineStr"/>
+      <c r="S7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -1055,57 +1091,62 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
+          <t>Graylinx</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
           <t>Production-grade streaming pipeline POC: Kafka -&gt; TimescaleDB -&gt; Airflow -&gt; FastAPI -&gt; Next.js.</t>
         </is>
       </c>
-      <c r="G8" s="4" t="inlineStr">
+      <c r="H8" s="4" t="inlineStr">
         <is>
           <t>Sole engineer — designed and built the end-to-end microservice pipeline and simulator.</t>
         </is>
       </c>
-      <c r="H8" s="4" t="inlineStr">
+      <c r="I8" s="4" t="inlineStr">
         <is>
           <t>Python; Kafka; TimescaleDB; Airflow; Next.js; Docker</t>
         </is>
       </c>
-      <c r="I8" s="4" t="inlineStr">
+      <c r="J8" s="4" t="inlineStr">
         <is>
           <t>2026-04-24</t>
         </is>
       </c>
-      <c r="J8" s="4" t="inlineStr">
+      <c r="K8" s="4" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="K8" s="4" t="inlineStr">
+      <c r="L8" s="4" t="inlineStr">
         <is>
           <t>git</t>
         </is>
       </c>
-      <c r="L8" s="5" t="inlineStr">
+      <c r="M8" s="5" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="M8" s="4" t="n">
+      <c r="N8" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="N8" s="4" t="n">
+      <c r="O8" s="4" t="n">
         <v>32</v>
       </c>
-      <c r="O8" s="4" t="inlineStr">
+      <c r="P8" s="4" t="inlineStr">
         <is>
           <t>D:\Harshan\clima-stream-hvac</t>
         </is>
       </c>
-      <c r="P8" s="4" t="inlineStr">
+      <c r="Q8" s="4" t="inlineStr">
         <is>
           <t>Proved the real-time streaming architecture; Microservices: simulator, ingestion, processor, ML, storage, API; 31 commits over ~4 weeks</t>
         </is>
       </c>
-      <c r="Q8" s="4" t="inlineStr"/>
       <c r="R8" s="4" t="inlineStr"/>
+      <c r="S8" s="4" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -1135,41 +1176,46 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
+          <t>Graylinx</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
           <t>Synthetic HVAC data</t>
         </is>
       </c>
-      <c r="G9" s="4" t="inlineStr"/>
       <c r="H9" s="4" t="inlineStr"/>
-      <c r="I9" s="4" t="inlineStr">
+      <c r="I9" s="4" t="inlineStr"/>
+      <c r="J9" s="4" t="inlineStr">
         <is>
           <t>2026-04-24</t>
         </is>
       </c>
-      <c r="J9" s="4" t="inlineStr">
+      <c r="K9" s="4" t="inlineStr">
         <is>
           <t>2026-05-04</t>
         </is>
       </c>
-      <c r="K9" s="4" t="inlineStr">
+      <c r="L9" s="4" t="inlineStr">
         <is>
           <t>git</t>
         </is>
       </c>
-      <c r="L9" s="5" t="inlineStr">
+      <c r="M9" s="5" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="M9" s="4" t="n">
+      <c r="N9" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="N9" s="4" t="n">
+      <c r="O9" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="O9" s="4" t="inlineStr"/>
       <c r="P9" s="4" t="inlineStr"/>
       <c r="Q9" s="4" t="inlineStr"/>
       <c r="R9" s="4" t="inlineStr"/>
+      <c r="S9" s="4" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -1199,41 +1245,46 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
+          <t>Graylinx</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
           <t>Streaming ingest</t>
         </is>
       </c>
-      <c r="G10" s="4" t="inlineStr"/>
       <c r="H10" s="4" t="inlineStr"/>
-      <c r="I10" s="4" t="inlineStr">
+      <c r="I10" s="4" t="inlineStr"/>
+      <c r="J10" s="4" t="inlineStr">
         <is>
           <t>2026-05-04</t>
         </is>
       </c>
-      <c r="J10" s="4" t="inlineStr">
+      <c r="K10" s="4" t="inlineStr">
         <is>
           <t>2026-05-14</t>
         </is>
       </c>
-      <c r="K10" s="4" t="inlineStr">
+      <c r="L10" s="4" t="inlineStr">
         <is>
           <t>git</t>
         </is>
       </c>
-      <c r="L10" s="5" t="inlineStr">
+      <c r="M10" s="5" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="M10" s="4" t="n">
+      <c r="N10" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="N10" s="4" t="n">
+      <c r="O10" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="O10" s="4" t="inlineStr"/>
       <c r="P10" s="4" t="inlineStr"/>
       <c r="Q10" s="4" t="inlineStr"/>
       <c r="R10" s="4" t="inlineStr"/>
+      <c r="S10" s="4" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -1263,41 +1314,46 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
+          <t>Graylinx</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
           <t>Time-series store</t>
         </is>
       </c>
-      <c r="G11" s="4" t="inlineStr"/>
       <c r="H11" s="4" t="inlineStr"/>
-      <c r="I11" s="4" t="inlineStr">
+      <c r="I11" s="4" t="inlineStr"/>
+      <c r="J11" s="4" t="inlineStr">
         <is>
           <t>2026-05-14</t>
         </is>
       </c>
-      <c r="J11" s="4" t="inlineStr">
+      <c r="K11" s="4" t="inlineStr">
         <is>
           <t>2026-05-25</t>
         </is>
       </c>
-      <c r="K11" s="4" t="inlineStr">
+      <c r="L11" s="4" t="inlineStr">
         <is>
           <t>git</t>
         </is>
       </c>
-      <c r="L11" s="5" t="inlineStr">
+      <c r="M11" s="5" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="M11" s="4" t="n">
+      <c r="N11" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="N11" s="4" t="n">
+      <c r="O11" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="O11" s="4" t="inlineStr"/>
       <c r="P11" s="4" t="inlineStr"/>
       <c r="Q11" s="4" t="inlineStr"/>
       <c r="R11" s="4" t="inlineStr"/>
+      <c r="S11" s="4" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -1327,41 +1383,46 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
+          <t>Graylinx</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
           <t>Anomaly/score service</t>
         </is>
       </c>
-      <c r="G12" s="4" t="inlineStr"/>
       <c r="H12" s="4" t="inlineStr"/>
-      <c r="I12" s="4" t="inlineStr">
+      <c r="I12" s="4" t="inlineStr"/>
+      <c r="J12" s="4" t="inlineStr">
         <is>
           <t>2026-05-25</t>
         </is>
       </c>
-      <c r="J12" s="4" t="inlineStr">
+      <c r="K12" s="4" t="inlineStr">
         <is>
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="K12" s="4" t="inlineStr">
+      <c r="L12" s="4" t="inlineStr">
         <is>
           <t>git</t>
         </is>
       </c>
-      <c r="L12" s="5" t="inlineStr">
+      <c r="M12" s="5" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="M12" s="4" t="n">
+      <c r="N12" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="N12" s="4" t="n">
+      <c r="O12" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="O12" s="4" t="inlineStr"/>
       <c r="P12" s="4" t="inlineStr"/>
       <c r="Q12" s="4" t="inlineStr"/>
       <c r="R12" s="4" t="inlineStr"/>
+      <c r="S12" s="4" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -1391,41 +1452,46 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
+          <t>Graylinx</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
           <t>Frontend dashboard</t>
         </is>
       </c>
-      <c r="G13" s="4" t="inlineStr"/>
       <c r="H13" s="4" t="inlineStr"/>
-      <c r="I13" s="4" t="inlineStr">
+      <c r="I13" s="4" t="inlineStr"/>
+      <c r="J13" s="4" t="inlineStr">
         <is>
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="J13" s="4" t="inlineStr">
+      <c r="K13" s="4" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="K13" s="4" t="inlineStr">
+      <c r="L13" s="4" t="inlineStr">
         <is>
           <t>git</t>
         </is>
       </c>
-      <c r="L13" s="5" t="inlineStr">
+      <c r="M13" s="5" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="M13" s="4" t="n">
+      <c r="N13" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="N13" s="4" t="n">
+      <c r="O13" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="O13" s="4" t="inlineStr"/>
       <c r="P13" s="4" t="inlineStr"/>
       <c r="Q13" s="4" t="inlineStr"/>
       <c r="R13" s="4" t="inlineStr"/>
+      <c r="S13" s="4" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1451,57 +1517,62 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
+          <t>Graylinx</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
           <t>Next-gen production platform vision: Digital-Twin FDD, RL optimization, Agentic AI, dual-database architecture.</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="H14" s="2" t="inlineStr">
         <is>
           <t>Architecture &amp; platform design — the strategic north star consolidating the POCs.</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr">
+      <c r="I14" s="2" t="inlineStr">
         <is>
           <t>Python; React; TypeScript; PostgreSQL; TimescaleDB; Kafka</t>
         </is>
       </c>
-      <c r="I14" s="2" t="inlineStr">
+      <c r="J14" s="2" t="inlineStr">
         <is>
           <t>2026-05-25</t>
         </is>
       </c>
-      <c r="J14" s="2" t="inlineStr">
+      <c r="K14" s="2" t="inlineStr">
         <is>
           <t>ongoing</t>
         </is>
       </c>
-      <c r="K14" s="2" t="inlineStr">
+      <c r="L14" s="2" t="inlineStr">
         <is>
           <t>git</t>
         </is>
       </c>
-      <c r="L14" s="3" t="inlineStr">
+      <c r="M14" s="3" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="M14" s="2" t="n">
+      <c r="N14" s="2" t="n">
         <v>35</v>
       </c>
-      <c r="N14" s="2" t="n">
+      <c r="O14" s="2" t="n">
         <v>219</v>
       </c>
-      <c r="O14" s="2" t="inlineStr">
+      <c r="P14" s="2" t="inlineStr">
         <is>
           <t>D:\Harshan\graylinx-v2</t>
         </is>
       </c>
-      <c r="P14" s="2" t="inlineStr">
+      <c r="Q14" s="2" t="inlineStr">
         <is>
           <t>Digital Twin fault detection &amp; diagnostics (FDD); Reinforcement-learning optimization; Agentic AI operations layer; Dual-DB (PostgreSQL + TimescaleDB) design</t>
         </is>
       </c>
-      <c r="Q14" s="2" t="inlineStr"/>
       <c r="R14" s="2" t="inlineStr"/>
+      <c r="S14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1531,41 +1602,46 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
+          <t>Graylinx</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
           <t>Fault detection &amp; diagnostics</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr"/>
       <c r="H15" s="2" t="inlineStr"/>
-      <c r="I15" s="2" t="inlineStr">
+      <c r="I15" s="2" t="inlineStr"/>
+      <c r="J15" s="2" t="inlineStr">
         <is>
           <t>2026-05-25</t>
         </is>
       </c>
-      <c r="J15" s="2" t="inlineStr">
+      <c r="K15" s="2" t="inlineStr">
         <is>
           <t>2026-05-30</t>
         </is>
       </c>
-      <c r="K15" s="2" t="inlineStr">
+      <c r="L15" s="2" t="inlineStr">
         <is>
           <t>git</t>
         </is>
       </c>
-      <c r="L15" s="3" t="inlineStr">
+      <c r="M15" s="3" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="M15" s="2" t="n">
+      <c r="N15" s="2" t="n">
         <v>40</v>
       </c>
-      <c r="N15" s="2" t="n">
+      <c r="O15" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="O15" s="2" t="inlineStr"/>
       <c r="P15" s="2" t="inlineStr"/>
       <c r="Q15" s="2" t="inlineStr"/>
       <c r="R15" s="2" t="inlineStr"/>
+      <c r="S15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
@@ -1595,41 +1671,46 @@
       </c>
       <c r="F16" s="6" t="inlineStr">
         <is>
+          <t>Graylinx</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="inlineStr">
+        <is>
           <t>Setpoint optimization</t>
         </is>
       </c>
-      <c r="G16" s="6" t="inlineStr"/>
       <c r="H16" s="6" t="inlineStr"/>
-      <c r="I16" s="6" t="inlineStr">
+      <c r="I16" s="6" t="inlineStr"/>
+      <c r="J16" s="6" t="inlineStr">
         <is>
           <t>2026-05-30</t>
         </is>
       </c>
-      <c r="J16" s="6" t="inlineStr">
+      <c r="K16" s="6" t="inlineStr">
         <is>
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="K16" s="6" t="inlineStr">
+      <c r="L16" s="6" t="inlineStr">
         <is>
           <t>git</t>
         </is>
       </c>
-      <c r="L16" s="7" t="inlineStr">
+      <c r="M16" s="7" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
-      <c r="M16" s="6" t="n">
+      <c r="N16" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="N16" s="6" t="n">
+      <c r="O16" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="O16" s="6" t="inlineStr"/>
       <c r="P16" s="6" t="inlineStr"/>
       <c r="Q16" s="6" t="inlineStr"/>
       <c r="R16" s="6" t="inlineStr"/>
+      <c r="S16" s="6" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1659,41 +1740,46 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
+          <t>Graylinx</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
           <t>Operations agents</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr"/>
       <c r="H17" s="2" t="inlineStr"/>
-      <c r="I17" s="2" t="inlineStr">
+      <c r="I17" s="2" t="inlineStr"/>
+      <c r="J17" s="2" t="inlineStr">
         <is>
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="J17" s="2" t="inlineStr">
+      <c r="K17" s="2" t="inlineStr">
         <is>
           <t>2026-06-09</t>
         </is>
       </c>
-      <c r="K17" s="2" t="inlineStr">
+      <c r="L17" s="2" t="inlineStr">
         <is>
           <t>git</t>
         </is>
       </c>
-      <c r="L17" s="3" t="inlineStr">
+      <c r="M17" s="3" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="M17" s="2" t="n">
+      <c r="N17" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="N17" s="2" t="n">
+      <c r="O17" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="O17" s="2" t="inlineStr"/>
       <c r="P17" s="2" t="inlineStr"/>
       <c r="Q17" s="2" t="inlineStr"/>
       <c r="R17" s="2" t="inlineStr"/>
+      <c r="S17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1723,41 +1809,46 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
+          <t>Graylinx</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
           <t>Postgres + Timescale</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr"/>
       <c r="H18" s="2" t="inlineStr"/>
-      <c r="I18" s="2" t="inlineStr">
+      <c r="I18" s="2" t="inlineStr"/>
+      <c r="J18" s="2" t="inlineStr">
         <is>
           <t>2026-06-09</t>
         </is>
       </c>
-      <c r="J18" s="2" t="inlineStr">
+      <c r="K18" s="2" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="K18" s="2" t="inlineStr">
+      <c r="L18" s="2" t="inlineStr">
         <is>
           <t>git</t>
         </is>
       </c>
-      <c r="L18" s="3" t="inlineStr">
+      <c r="M18" s="3" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="M18" s="2" t="n">
+      <c r="N18" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="N18" s="2" t="n">
+      <c r="O18" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="O18" s="2" t="inlineStr"/>
       <c r="P18" s="2" t="inlineStr"/>
       <c r="Q18" s="2" t="inlineStr"/>
       <c r="R18" s="2" t="inlineStr"/>
+      <c r="S18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
@@ -1783,57 +1874,62 @@
       </c>
       <c r="F19" s="8" t="inlineStr">
         <is>
+          <t>Graylinx</t>
+        </is>
+      </c>
+      <c r="G19" s="8" t="inlineStr">
+        <is>
           <t>Reference architecture &amp; planning docs unifying ClimaStream, THERMYNX and OMNYX into one next-gen vision.</t>
         </is>
       </c>
-      <c r="G19" s="8" t="inlineStr">
+      <c r="H19" s="8" t="inlineStr">
         <is>
           <t>Author — architecture documentation and lessons-learned consolidation.</t>
         </is>
       </c>
-      <c r="H19" s="8" t="inlineStr">
+      <c r="I19" s="8" t="inlineStr">
         <is>
           <t>Markdown; Architecture</t>
         </is>
       </c>
-      <c r="I19" s="8" t="inlineStr">
+      <c r="J19" s="8" t="inlineStr">
         <is>
           <t>2026-05-26</t>
         </is>
       </c>
-      <c r="J19" s="8" t="inlineStr">
+      <c r="K19" s="8" t="inlineStr">
         <is>
           <t>2026-05-30</t>
         </is>
       </c>
-      <c r="K19" s="8" t="inlineStr">
+      <c r="L19" s="8" t="inlineStr">
         <is>
           <t>approx</t>
         </is>
       </c>
-      <c r="L19" s="9" t="inlineStr">
+      <c r="M19" s="9" t="inlineStr">
         <is>
           <t>Ongoing</t>
         </is>
       </c>
-      <c r="M19" s="8" t="n">
+      <c r="N19" s="8" t="n">
         <v>60</v>
       </c>
-      <c r="N19" s="8" t="n">
+      <c r="O19" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="O19" s="8" t="inlineStr">
+      <c r="P19" s="8" t="inlineStr">
         <is>
           <t>D:\Harshan\gl-pulse</t>
         </is>
       </c>
-      <c r="P19" s="8" t="inlineStr">
+      <c r="Q19" s="8" t="inlineStr">
         <is>
           <t>20 architecture documents; Consolidates POC lessons into unified design</t>
         </is>
       </c>
-      <c r="Q19" s="8" t="inlineStr"/>
       <c r="R19" s="8" t="inlineStr"/>
+      <c r="S19" s="8" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
@@ -1859,57 +1955,62 @@
       </c>
       <c r="F20" s="6" t="inlineStr">
         <is>
+          <t>Graylinx</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
           <t>BACnet device simulator workstream (simulator dashboard lives under Current Works in GL).</t>
         </is>
       </c>
-      <c r="G20" s="6" t="inlineStr">
+      <c r="H20" s="6" t="inlineStr">
         <is>
           <t>Simulation flow study and BACnet device/UI analysis.</t>
         </is>
       </c>
-      <c r="H20" s="6" t="inlineStr">
+      <c r="I20" s="6" t="inlineStr">
         <is>
           <t>Vue 3; BACnet; Simulation</t>
         </is>
       </c>
-      <c r="I20" s="6" t="inlineStr">
+      <c r="J20" s="6" t="inlineStr">
         <is>
           <t>2026-05-11</t>
         </is>
       </c>
-      <c r="J20" s="6" t="inlineStr">
+      <c r="K20" s="6" t="inlineStr">
         <is>
           <t>2026-05-13</t>
         </is>
       </c>
-      <c r="K20" s="6" t="inlineStr">
+      <c r="L20" s="6" t="inlineStr">
         <is>
           <t>manual</t>
         </is>
       </c>
-      <c r="L20" s="7" t="inlineStr">
+      <c r="M20" s="7" t="inlineStr">
         <is>
           <t>Paused</t>
         </is>
       </c>
-      <c r="M20" s="6" t="n">
+      <c r="N20" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="N20" s="6" t="n">
+      <c r="O20" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="O20" s="6" t="inlineStr">
+      <c r="P20" s="6" t="inlineStr">
         <is>
           <t>D:\Harshan\gl-pbs-simulation</t>
         </is>
       </c>
-      <c r="P20" s="6" t="inlineStr">
+      <c r="Q20" s="6" t="inlineStr">
         <is>
           <t>BACnet device simulation; Vue 3 simulator dashboard</t>
         </is>
       </c>
-      <c r="Q20" s="6" t="inlineStr"/>
       <c r="R20" s="6" t="inlineStr"/>
+      <c r="S20" s="6" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1935,57 +2036,62 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
+          <t>Graylinx</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
           <t>Active Graylinx monorepo: backend/frontend, commission tool, ML trainings, simulations, Kafka stress testing.</t>
         </is>
       </c>
-      <c r="G21" s="2" t="inlineStr">
+      <c r="H21" s="2" t="inlineStr">
         <is>
           <t>Sole engineer — Kafka performance testing, cross-machine benchmarking, DB/ETL architecture audits.</t>
         </is>
       </c>
-      <c r="H21" s="2" t="inlineStr">
+      <c r="I21" s="2" t="inlineStr">
         <is>
           <t>Node.js; Express; Kafka; MySQL; Python</t>
         </is>
       </c>
-      <c r="I21" s="2" t="inlineStr">
+      <c r="J21" s="2" t="inlineStr">
         <is>
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="J21" s="2" t="inlineStr">
+      <c r="K21" s="2" t="inlineStr">
         <is>
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="K21" s="2" t="inlineStr">
+      <c r="L21" s="2" t="inlineStr">
         <is>
           <t>git</t>
         </is>
       </c>
-      <c r="L21" s="3" t="inlineStr">
+      <c r="M21" s="3" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="M21" s="2" t="n">
+      <c r="N21" s="2" t="n">
         <v>75</v>
       </c>
-      <c r="N21" s="2" t="n">
+      <c r="O21" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="O21" s="2" t="inlineStr">
+      <c r="P21" s="2" t="inlineStr">
         <is>
           <t>D:\Harshan\Current Works in GL</t>
         </is>
       </c>
-      <c r="P21" s="2" t="inlineStr">
+      <c r="Q21" s="2" t="inlineStr">
         <is>
           <t>Kafka stress tests 150x -&gt; 5000x scale; Cross-machine 24GB vs 8GB comparison reports; DB &amp; ETL critical-flaws audits, management summaries</t>
         </is>
       </c>
-      <c r="Q21" s="2" t="inlineStr"/>
       <c r="R21" s="2" t="inlineStr"/>
+      <c r="S21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -2015,41 +2121,46 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
+          <t>Graylinx</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
           <t>Throughput scaling</t>
         </is>
       </c>
-      <c r="G22" s="2" t="inlineStr"/>
       <c r="H22" s="2" t="inlineStr"/>
-      <c r="I22" s="2" t="inlineStr">
+      <c r="I22" s="2" t="inlineStr"/>
+      <c r="J22" s="2" t="inlineStr">
         <is>
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="J22" s="2" t="inlineStr">
+      <c r="K22" s="2" t="inlineStr">
         <is>
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="K22" s="2" t="inlineStr">
+      <c r="L22" s="2" t="inlineStr">
         <is>
           <t>git</t>
         </is>
       </c>
-      <c r="L22" s="3" t="inlineStr">
+      <c r="M22" s="3" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="M22" s="2" t="n">
+      <c r="N22" s="2" t="n">
         <v>80</v>
       </c>
-      <c r="N22" s="2" t="n">
+      <c r="O22" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="O22" s="2" t="inlineStr"/>
       <c r="P22" s="2" t="inlineStr"/>
       <c r="Q22" s="2" t="inlineStr"/>
       <c r="R22" s="2" t="inlineStr"/>
+      <c r="S22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
@@ -2079,41 +2190,46 @@
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
+          <t>Graylinx</t>
+        </is>
+      </c>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
           <t>Hardware comparison</t>
         </is>
       </c>
-      <c r="G23" s="4" t="inlineStr"/>
       <c r="H23" s="4" t="inlineStr"/>
-      <c r="I23" s="4" t="inlineStr">
+      <c r="I23" s="4" t="inlineStr"/>
+      <c r="J23" s="4" t="inlineStr">
         <is>
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="J23" s="4" t="inlineStr">
+      <c r="K23" s="4" t="inlineStr">
         <is>
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="K23" s="4" t="inlineStr">
+      <c r="L23" s="4" t="inlineStr">
         <is>
           <t>git</t>
         </is>
       </c>
-      <c r="L23" s="5" t="inlineStr">
+      <c r="M23" s="5" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="M23" s="4" t="n">
+      <c r="N23" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="N23" s="4" t="n">
+      <c r="O23" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="O23" s="4" t="inlineStr"/>
       <c r="P23" s="4" t="inlineStr"/>
       <c r="Q23" s="4" t="inlineStr"/>
       <c r="R23" s="4" t="inlineStr"/>
+      <c r="S23" s="4" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -2143,41 +2259,46 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
+          <t>Graylinx</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
           <t>Critical-flaws reviews</t>
         </is>
       </c>
-      <c r="G24" s="2" t="inlineStr"/>
       <c r="H24" s="2" t="inlineStr"/>
-      <c r="I24" s="2" t="inlineStr">
+      <c r="I24" s="2" t="inlineStr"/>
+      <c r="J24" s="2" t="inlineStr">
         <is>
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="J24" s="2" t="inlineStr">
+      <c r="K24" s="2" t="inlineStr">
         <is>
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="K24" s="2" t="inlineStr">
+      <c r="L24" s="2" t="inlineStr">
         <is>
           <t>git</t>
         </is>
       </c>
-      <c r="L24" s="3" t="inlineStr">
+      <c r="M24" s="3" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="M24" s="2" t="n">
+      <c r="N24" s="2" t="n">
         <v>70</v>
       </c>
-      <c r="N24" s="2" t="n">
+      <c r="O24" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="O24" s="2" t="inlineStr"/>
       <c r="P24" s="2" t="inlineStr"/>
       <c r="Q24" s="2" t="inlineStr"/>
       <c r="R24" s="2" t="inlineStr"/>
+      <c r="S24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="8" t="inlineStr">
@@ -2203,57 +2324,62 @@
       </c>
       <c r="F25" s="8" t="inlineStr">
         <is>
+          <t>Graylinx</t>
+        </is>
+      </c>
+      <c r="G25" s="8" t="inlineStr">
+        <is>
           <t>Product/architecture documentation: PRD, Modules &amp; Features (175 features), Kafka/stress reports.</t>
         </is>
       </c>
-      <c r="G25" s="8" t="inlineStr">
+      <c r="H25" s="8" t="inlineStr">
         <is>
           <t>Author/maintainer — PRD, feature inventory, architecture references.</t>
         </is>
       </c>
-      <c r="H25" s="8" t="inlineStr">
+      <c r="I25" s="8" t="inlineStr">
         <is>
           <t>Markdown; PRD; Documentation</t>
         </is>
       </c>
-      <c r="I25" s="8" t="inlineStr">
+      <c r="J25" s="8" t="inlineStr">
         <is>
           <t>2026-04-28</t>
         </is>
       </c>
-      <c r="J25" s="8" t="inlineStr">
+      <c r="K25" s="8" t="inlineStr">
         <is>
           <t>2026-05-21</t>
         </is>
       </c>
-      <c r="K25" s="8" t="inlineStr">
+      <c r="L25" s="8" t="inlineStr">
         <is>
           <t>approx</t>
         </is>
       </c>
-      <c r="L25" s="9" t="inlineStr">
+      <c r="M25" s="9" t="inlineStr">
         <is>
           <t>Ongoing</t>
         </is>
       </c>
-      <c r="M25" s="8" t="n">
+      <c r="N25" s="8" t="n">
         <v>65</v>
       </c>
-      <c r="N25" s="8" t="n">
+      <c r="O25" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="O25" s="8" t="inlineStr">
+      <c r="P25" s="8" t="inlineStr">
         <is>
           <t>D:\Harshan\Docs</t>
         </is>
       </c>
-      <c r="P25" s="8" t="inlineStr">
+      <c r="Q25" s="8" t="inlineStr">
         <is>
           <t>Graylinx_Modules_and_Features.md — 175 features, phased; PRD v1.0 + Industrial Platform Master</t>
         </is>
       </c>
-      <c r="Q25" s="8" t="inlineStr"/>
       <c r="R25" s="8" t="inlineStr"/>
+      <c r="S25" s="8" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2279,57 +2405,62 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
+          <t>Personal</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
           <t>Six-product local-AI suite (6 repos): Continuum (HVAC intelligence), AuditShield, Autonomous-Cortex, NeuralPulse, VisioScan, SpatialNexus.</t>
         </is>
       </c>
-      <c r="G26" s="2" t="inlineStr">
+      <c r="H26" s="2" t="inlineStr">
         <is>
           <t>Designed &amp; built the multi-product suite across six repositories.</t>
         </is>
       </c>
-      <c r="H26" s="2" t="inlineStr">
+      <c r="I26" s="2" t="inlineStr">
         <is>
           <t>React; TypeScript; Python; Neo4j; pgvector; Ollama; Docker</t>
         </is>
       </c>
-      <c r="I26" s="2" t="inlineStr">
+      <c r="J26" s="2" t="inlineStr">
         <is>
           <t>2026-05-18</t>
         </is>
       </c>
-      <c r="J26" s="2" t="inlineStr">
+      <c r="K26" s="2" t="inlineStr">
         <is>
           <t>2026-05-21</t>
         </is>
       </c>
-      <c r="K26" s="2" t="inlineStr">
+      <c r="L26" s="2" t="inlineStr">
         <is>
           <t>git</t>
         </is>
       </c>
-      <c r="L26" s="3" t="inlineStr">
+      <c r="M26" s="3" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="M26" s="2" t="n">
+      <c r="N26" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="N26" s="2" t="n">
+      <c r="O26" s="2" t="n">
         <v>94</v>
       </c>
-      <c r="O26" s="2" t="inlineStr">
+      <c r="P26" s="2" t="inlineStr">
         <is>
           <t>D:\Harshan\The SelfAware® Intelligence Suite</t>
         </is>
       </c>
-      <c r="P26" s="2" t="inlineStr">
+      <c r="Q26" s="2" t="inlineStr">
         <is>
           <t>6 products in one suite; SelfAware Continuum: Unicharm + Neo4j + pgvector + Ollama</t>
         </is>
       </c>
-      <c r="Q26" s="2" t="inlineStr"/>
       <c r="R26" s="2" t="inlineStr"/>
+      <c r="S26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2359,41 +2490,46 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
+          <t>Personal</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
           <t>Neo4j + pgvector + Ollama</t>
         </is>
       </c>
-      <c r="G27" s="2" t="inlineStr"/>
       <c r="H27" s="2" t="inlineStr"/>
-      <c r="I27" s="2" t="inlineStr">
+      <c r="I27" s="2" t="inlineStr"/>
+      <c r="J27" s="2" t="inlineStr">
         <is>
           <t>2026-05-18</t>
         </is>
       </c>
-      <c r="J27" s="2" t="inlineStr">
+      <c r="K27" s="2" t="inlineStr">
         <is>
           <t>2026-05-18</t>
         </is>
       </c>
-      <c r="K27" s="2" t="inlineStr">
+      <c r="L27" s="2" t="inlineStr">
         <is>
           <t>git</t>
         </is>
       </c>
-      <c r="L27" s="3" t="inlineStr">
+      <c r="M27" s="3" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="M27" s="2" t="n">
+      <c r="N27" s="2" t="n">
         <v>55</v>
       </c>
-      <c r="N27" s="2" t="n">
+      <c r="O27" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="O27" s="2" t="inlineStr"/>
       <c r="P27" s="2" t="inlineStr"/>
       <c r="Q27" s="2" t="inlineStr"/>
       <c r="R27" s="2" t="inlineStr"/>
+      <c r="S27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
@@ -2423,41 +2559,46 @@
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
+          <t>Personal</t>
+        </is>
+      </c>
+      <c r="G28" s="4" t="inlineStr">
+        <is>
           <t>Compliance ledger</t>
         </is>
       </c>
-      <c r="G28" s="4" t="inlineStr"/>
       <c r="H28" s="4" t="inlineStr"/>
-      <c r="I28" s="4" t="inlineStr">
+      <c r="I28" s="4" t="inlineStr"/>
+      <c r="J28" s="4" t="inlineStr">
         <is>
           <t>2026-05-18</t>
         </is>
       </c>
-      <c r="J28" s="4" t="inlineStr">
+      <c r="K28" s="4" t="inlineStr">
         <is>
           <t>2026-05-19</t>
         </is>
       </c>
-      <c r="K28" s="4" t="inlineStr">
+      <c r="L28" s="4" t="inlineStr">
         <is>
           <t>git</t>
         </is>
       </c>
-      <c r="L28" s="5" t="inlineStr">
+      <c r="M28" s="5" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="M28" s="4" t="n">
+      <c r="N28" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="N28" s="4" t="n">
+      <c r="O28" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="O28" s="4" t="inlineStr"/>
       <c r="P28" s="4" t="inlineStr"/>
       <c r="Q28" s="4" t="inlineStr"/>
       <c r="R28" s="4" t="inlineStr"/>
+      <c r="S28" s="4" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
@@ -2487,41 +2628,46 @@
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
+          <t>Personal</t>
+        </is>
+      </c>
+      <c r="G29" s="4" t="inlineStr">
+        <is>
           <t>Mission console</t>
         </is>
       </c>
-      <c r="G29" s="4" t="inlineStr"/>
       <c r="H29" s="4" t="inlineStr"/>
-      <c r="I29" s="4" t="inlineStr">
+      <c r="I29" s="4" t="inlineStr"/>
+      <c r="J29" s="4" t="inlineStr">
         <is>
           <t>2026-05-19</t>
         </is>
       </c>
-      <c r="J29" s="4" t="inlineStr">
+      <c r="K29" s="4" t="inlineStr">
         <is>
           <t>2026-05-19</t>
         </is>
       </c>
-      <c r="K29" s="4" t="inlineStr">
+      <c r="L29" s="4" t="inlineStr">
         <is>
           <t>git</t>
         </is>
       </c>
-      <c r="L29" s="5" t="inlineStr">
+      <c r="M29" s="5" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="M29" s="4" t="n">
+      <c r="N29" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="N29" s="4" t="n">
+      <c r="O29" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="O29" s="4" t="inlineStr"/>
       <c r="P29" s="4" t="inlineStr"/>
       <c r="Q29" s="4" t="inlineStr"/>
       <c r="R29" s="4" t="inlineStr"/>
+      <c r="S29" s="4" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
@@ -2551,41 +2697,46 @@
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
+          <t>Personal</t>
+        </is>
+      </c>
+      <c r="G30" s="4" t="inlineStr">
+        <is>
           <t>Signal lab</t>
         </is>
       </c>
-      <c r="G30" s="4" t="inlineStr"/>
       <c r="H30" s="4" t="inlineStr"/>
-      <c r="I30" s="4" t="inlineStr">
+      <c r="I30" s="4" t="inlineStr"/>
+      <c r="J30" s="4" t="inlineStr">
         <is>
           <t>2026-05-19</t>
         </is>
       </c>
-      <c r="J30" s="4" t="inlineStr">
+      <c r="K30" s="4" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
       </c>
-      <c r="K30" s="4" t="inlineStr">
+      <c r="L30" s="4" t="inlineStr">
         <is>
           <t>git</t>
         </is>
       </c>
-      <c r="L30" s="5" t="inlineStr">
+      <c r="M30" s="5" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="M30" s="4" t="n">
+      <c r="N30" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="N30" s="4" t="n">
+      <c r="O30" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="O30" s="4" t="inlineStr"/>
       <c r="P30" s="4" t="inlineStr"/>
       <c r="Q30" s="4" t="inlineStr"/>
       <c r="R30" s="4" t="inlineStr"/>
+      <c r="S30" s="4" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
@@ -2615,41 +2766,46 @@
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
+          <t>Personal</t>
+        </is>
+      </c>
+      <c r="G31" s="4" t="inlineStr">
+        <is>
           <t>Light studio</t>
         </is>
       </c>
-      <c r="G31" s="4" t="inlineStr"/>
       <c r="H31" s="4" t="inlineStr"/>
-      <c r="I31" s="4" t="inlineStr">
+      <c r="I31" s="4" t="inlineStr"/>
+      <c r="J31" s="4" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
       </c>
-      <c r="J31" s="4" t="inlineStr">
+      <c r="K31" s="4" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
       </c>
-      <c r="K31" s="4" t="inlineStr">
+      <c r="L31" s="4" t="inlineStr">
         <is>
           <t>git</t>
         </is>
       </c>
-      <c r="L31" s="5" t="inlineStr">
+      <c r="M31" s="5" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="M31" s="4" t="n">
+      <c r="N31" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="N31" s="4" t="n">
+      <c r="O31" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="O31" s="4" t="inlineStr"/>
       <c r="P31" s="4" t="inlineStr"/>
       <c r="Q31" s="4" t="inlineStr"/>
       <c r="R31" s="4" t="inlineStr"/>
+      <c r="S31" s="4" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
@@ -2679,41 +2835,46 @@
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
+          <t>Personal</t>
+        </is>
+      </c>
+      <c r="G32" s="4" t="inlineStr">
+        <is>
           <t>Topology atlas</t>
         </is>
       </c>
-      <c r="G32" s="4" t="inlineStr"/>
       <c r="H32" s="4" t="inlineStr"/>
-      <c r="I32" s="4" t="inlineStr">
+      <c r="I32" s="4" t="inlineStr"/>
+      <c r="J32" s="4" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
       </c>
-      <c r="J32" s="4" t="inlineStr">
+      <c r="K32" s="4" t="inlineStr">
         <is>
           <t>2026-05-21</t>
         </is>
       </c>
-      <c r="K32" s="4" t="inlineStr">
+      <c r="L32" s="4" t="inlineStr">
         <is>
           <t>git</t>
         </is>
       </c>
-      <c r="L32" s="5" t="inlineStr">
+      <c r="M32" s="5" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="M32" s="4" t="n">
+      <c r="N32" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="N32" s="4" t="n">
+      <c r="O32" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="O32" s="4" t="inlineStr"/>
       <c r="P32" s="4" t="inlineStr"/>
       <c r="Q32" s="4" t="inlineStr"/>
       <c r="R32" s="4" t="inlineStr"/>
+      <c r="S32" s="4" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2739,57 +2900,62 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
+          <t>Personal</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
           <t>Interactive concept-map viewer (1,159 concepts, 5,985 relations) for lesson generation.</t>
         </is>
       </c>
-      <c r="G33" s="2" t="inlineStr">
+      <c r="H33" s="2" t="inlineStr">
         <is>
           <t>Built the in-browser graph analytics tool (ECharts + Neo4j GDS).</t>
         </is>
       </c>
-      <c r="H33" s="2" t="inlineStr">
+      <c r="I33" s="2" t="inlineStr">
         <is>
           <t>Python; JavaScript; ECharts; Neo4j</t>
         </is>
       </c>
-      <c r="I33" s="2" t="inlineStr">
+      <c r="J33" s="2" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="J33" s="2" t="inlineStr">
+      <c r="K33" s="2" t="inlineStr">
         <is>
           <t>ongoing</t>
         </is>
       </c>
-      <c r="K33" s="2" t="inlineStr">
+      <c r="L33" s="2" t="inlineStr">
         <is>
           <t>approx</t>
         </is>
       </c>
-      <c r="L33" s="3" t="inlineStr">
+      <c r="M33" s="3" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="M33" s="2" t="n">
+      <c r="N33" s="2" t="n">
         <v>55</v>
       </c>
-      <c r="N33" s="2" t="n">
+      <c r="O33" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="O33" s="2" t="inlineStr">
+      <c r="P33" s="2" t="inlineStr">
         <is>
           <t>D:\Harshan\concept-standard</t>
         </is>
       </c>
-      <c r="P33" s="2" t="inlineStr">
+      <c r="Q33" s="2" t="inlineStr">
         <is>
           <t>1,159 concepts / 5,985 relations; Force/circular graphs, command palette, light/dark, a11y</t>
         </is>
       </c>
-      <c r="Q33" s="2" t="inlineStr"/>
       <c r="R33" s="2" t="inlineStr"/>
+      <c r="S33" s="2" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
@@ -2815,57 +2981,62 @@
       </c>
       <c r="F34" s="6" t="inlineStr">
         <is>
+          <t>Personal</t>
+        </is>
+      </c>
+      <c r="G34" s="6" t="inlineStr">
+        <is>
           <t>Realtime on-prem AI voice intelligence platform — monorepo with local LLM, Whisper STT, Piper TTS.</t>
         </is>
       </c>
-      <c r="G34" s="6" t="inlineStr">
+      <c r="H34" s="6" t="inlineStr">
         <is>
           <t>Architecture &amp; monorepo setup (pnpm/Turbo), service scaffolding.</t>
         </is>
       </c>
-      <c r="H34" s="6" t="inlineStr">
+      <c r="I34" s="6" t="inlineStr">
         <is>
           <t>Node.js; pnpm; Turbo; Ollama; Whisper; Piper; Docker</t>
         </is>
       </c>
-      <c r="I34" s="6" t="inlineStr">
+      <c r="J34" s="6" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
       </c>
-      <c r="J34" s="6" t="inlineStr">
+      <c r="K34" s="6" t="inlineStr">
         <is>
           <t>2026-05-21</t>
         </is>
       </c>
-      <c r="K34" s="6" t="inlineStr">
+      <c r="L34" s="6" t="inlineStr">
         <is>
           <t>approx</t>
         </is>
       </c>
-      <c r="L34" s="7" t="inlineStr">
+      <c r="M34" s="7" t="inlineStr">
         <is>
           <t>Paused</t>
         </is>
       </c>
-      <c r="M34" s="6" t="n">
+      <c r="N34" s="6" t="n">
         <v>30</v>
       </c>
-      <c r="N34" s="6" t="n">
+      <c r="O34" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="O34" s="6" t="inlineStr">
+      <c r="P34" s="6" t="inlineStr">
         <is>
           <t>D:\Harshan\VOXARA AI</t>
         </is>
       </c>
-      <c r="P34" s="6" t="inlineStr">
+      <c r="Q34" s="6" t="inlineStr">
         <is>
           <t>Largest by file count (37 items); Local LLM + Whisper + Piper TTS</t>
         </is>
       </c>
-      <c r="Q34" s="6" t="inlineStr"/>
       <c r="R34" s="6" t="inlineStr"/>
+      <c r="S34" s="6" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
@@ -2891,57 +3062,62 @@
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="G35" s="4" t="inlineStr">
+        <is>
           <t>Buildless travel/expense reporting web app for RANGSONS LLP with HR approval + Google Sheets.</t>
         </is>
       </c>
-      <c r="G35" s="4" t="inlineStr">
+      <c r="H35" s="4" t="inlineStr">
         <is>
           <t>Sole developer — static web app, Supabase backend, approval flow.</t>
         </is>
       </c>
-      <c r="H35" s="4" t="inlineStr">
+      <c r="I35" s="4" t="inlineStr">
         <is>
           <t>HTML; Tailwind; JavaScript; Supabase</t>
         </is>
       </c>
-      <c r="I35" s="4" t="inlineStr">
+      <c r="J35" s="4" t="inlineStr">
         <is>
           <t>2026-06-03</t>
         </is>
       </c>
-      <c r="J35" s="4" t="inlineStr">
+      <c r="K35" s="4" t="inlineStr">
         <is>
           <t>2026-06-03</t>
         </is>
       </c>
-      <c r="K35" s="4" t="inlineStr">
+      <c r="L35" s="4" t="inlineStr">
         <is>
           <t>git</t>
         </is>
       </c>
-      <c r="L35" s="5" t="inlineStr">
+      <c r="M35" s="5" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="M35" s="4" t="n">
+      <c r="N35" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="N35" s="4" t="n">
+      <c r="O35" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="O35" s="4" t="inlineStr">
+      <c r="P35" s="4" t="inlineStr">
         <is>
           <t>D:\Harshan\travel-app</t>
         </is>
       </c>
-      <c r="P35" s="4" t="inlineStr">
+      <c r="Q35" s="4" t="inlineStr">
         <is>
           <t>HR approval + Google Sheets integration; Buildless static deployment</t>
         </is>
       </c>
-      <c r="Q35" s="4" t="inlineStr"/>
       <c r="R35" s="4" t="inlineStr"/>
+      <c r="S35" s="4" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
@@ -2967,57 +3143,62 @@
       </c>
       <c r="F36" s="6" t="inlineStr">
         <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="G36" s="6" t="inlineStr">
+        <is>
           <t>React + TypeScript canvas/drawing app template (likely a UI/design component base).</t>
         </is>
       </c>
-      <c r="G36" s="6" t="inlineStr">
+      <c r="H36" s="6" t="inlineStr">
         <is>
           <t>Template/prototype setup.</t>
         </is>
       </c>
-      <c r="H36" s="6" t="inlineStr">
+      <c r="I36" s="6" t="inlineStr">
         <is>
           <t>React; TypeScript; Vite; Konva</t>
         </is>
       </c>
-      <c r="I36" s="6" t="inlineStr">
+      <c r="J36" s="6" t="inlineStr">
         <is>
           <t>2026-05-14</t>
         </is>
       </c>
-      <c r="J36" s="6" t="inlineStr">
+      <c r="K36" s="6" t="inlineStr">
         <is>
           <t>2026-05-14</t>
         </is>
       </c>
-      <c r="K36" s="6" t="inlineStr">
+      <c r="L36" s="6" t="inlineStr">
         <is>
           <t>approx</t>
         </is>
       </c>
-      <c r="L36" s="7" t="inlineStr">
+      <c r="M36" s="7" t="inlineStr">
         <is>
           <t>Paused</t>
         </is>
       </c>
-      <c r="M36" s="6" t="n">
+      <c r="N36" s="6" t="n">
         <v>25</v>
       </c>
-      <c r="N36" s="6" t="n">
+      <c r="O36" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="O36" s="6" t="inlineStr">
+      <c r="P36" s="6" t="inlineStr">
         <is>
           <t>D:\Harshan\konva</t>
         </is>
       </c>
-      <c r="P36" s="6" t="inlineStr">
+      <c r="Q36" s="6" t="inlineStr">
         <is>
           <t>Canvas/drawing UI base</t>
         </is>
       </c>
-      <c r="Q36" s="6" t="inlineStr"/>
       <c r="R36" s="6" t="inlineStr"/>
+      <c r="S36" s="6" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -3043,57 +3224,62 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
           <t>Farm-to-fork traceability platform for NR Group (Nesso).</t>
         </is>
       </c>
-      <c r="G37" s="2" t="inlineStr">
+      <c r="H37" s="2" t="inlineStr">
         <is>
           <t>Built the traceability web app — including a weekend build sprint (30–31 May).</t>
         </is>
       </c>
-      <c r="H37" s="2" t="inlineStr">
+      <c r="I37" s="2" t="inlineStr">
         <is>
           <t>TypeScript; React; Node.js</t>
         </is>
       </c>
-      <c r="I37" s="2" t="inlineStr">
+      <c r="J37" s="2" t="inlineStr">
         <is>
           <t>2026-05-28</t>
         </is>
       </c>
-      <c r="J37" s="2" t="inlineStr">
+      <c r="K37" s="2" t="inlineStr">
         <is>
           <t>ongoing</t>
         </is>
       </c>
-      <c r="K37" s="2" t="inlineStr">
+      <c r="L37" s="2" t="inlineStr">
         <is>
           <t>git</t>
         </is>
       </c>
-      <c r="L37" s="3" t="inlineStr">
+      <c r="M37" s="3" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="M37" s="2" t="n">
+      <c r="N37" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="N37" s="2" t="n">
+      <c r="O37" s="2" t="n">
         <v>191</v>
       </c>
-      <c r="O37" s="2" t="inlineStr">
+      <c r="P37" s="2" t="inlineStr">
         <is>
           <t>D:\Harshan\farmer-app</t>
         </is>
       </c>
-      <c r="P37" s="2" t="inlineStr">
+      <c r="Q37" s="2" t="inlineStr">
         <is>
           <t>Farm-to-fork traceability (NR Group); ~1-week build incl. weekend sprint</t>
         </is>
       </c>
-      <c r="Q37" s="2" t="inlineStr"/>
       <c r="R37" s="2" t="inlineStr"/>
+      <c r="S37" s="2" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
@@ -3119,57 +3305,62 @@
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
+          <t>Personal</t>
+        </is>
+      </c>
+      <c r="G38" s="4" t="inlineStr">
+        <is>
           <t>Canonical local Docker dev stack (MySQL, PostgreSQL, Neo4j, Redis) for the SelfAware products.</t>
         </is>
       </c>
-      <c r="G38" s="4" t="inlineStr">
+      <c r="H38" s="4" t="inlineStr">
         <is>
           <t>Authored the docker-compose environment for 4 products.</t>
         </is>
       </c>
-      <c r="H38" s="4" t="inlineStr">
+      <c r="I38" s="4" t="inlineStr">
         <is>
           <t>Docker; MySQL; PostgreSQL; Neo4j; Redis</t>
         </is>
       </c>
-      <c r="I38" s="4" t="inlineStr">
+      <c r="J38" s="4" t="inlineStr">
         <is>
           <t>2026-05-21</t>
         </is>
       </c>
-      <c r="J38" s="4" t="inlineStr">
+      <c r="K38" s="4" t="inlineStr">
         <is>
           <t>2026-05-21</t>
         </is>
       </c>
-      <c r="K38" s="4" t="inlineStr">
+      <c r="L38" s="4" t="inlineStr">
         <is>
           <t>approx</t>
         </is>
       </c>
-      <c r="L38" s="5" t="inlineStr">
+      <c r="M38" s="5" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="M38" s="4" t="n">
+      <c r="N38" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="N38" s="4" t="n">
+      <c r="O38" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="O38" s="4" t="inlineStr">
+      <c r="P38" s="4" t="inlineStr">
         <is>
           <t>D:\Harshan\selfaware-dev-stack</t>
         </is>
       </c>
-      <c r="P38" s="4" t="inlineStr">
+      <c r="Q38" s="4" t="inlineStr">
         <is>
           <t>One dev environment for 4 products</t>
         </is>
       </c>
-      <c r="Q38" s="4" t="inlineStr"/>
       <c r="R38" s="4" t="inlineStr"/>
+      <c r="S38" s="4" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
@@ -3195,57 +3386,62 @@
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
+          <t>Graylinx</t>
+        </is>
+      </c>
+      <c r="G39" s="4" t="inlineStr">
+        <is>
           <t>Docker MySQL port-forwarding helper — superseded by selfaware-dev-stack.</t>
         </is>
       </c>
-      <c r="G39" s="4" t="inlineStr">
+      <c r="H39" s="4" t="inlineStr">
         <is>
           <t>Quick infra utility (now reference-only).</t>
         </is>
       </c>
-      <c r="H39" s="4" t="inlineStr">
+      <c r="I39" s="4" t="inlineStr">
         <is>
           <t>Docker; MySQL</t>
         </is>
       </c>
-      <c r="I39" s="4" t="inlineStr">
+      <c r="J39" s="4" t="inlineStr">
         <is>
           <t>2026-05-21</t>
         </is>
       </c>
-      <c r="J39" s="4" t="inlineStr">
+      <c r="K39" s="4" t="inlineStr">
         <is>
           <t>2026-05-21</t>
         </is>
       </c>
-      <c r="K39" s="4" t="inlineStr">
+      <c r="L39" s="4" t="inlineStr">
         <is>
           <t>approx</t>
         </is>
       </c>
-      <c r="L39" s="5" t="inlineStr">
+      <c r="M39" s="5" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="M39" s="4" t="n">
+      <c r="N39" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="N39" s="4" t="n">
+      <c r="O39" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="O39" s="4" t="inlineStr">
+      <c r="P39" s="4" t="inlineStr">
         <is>
           <t>D:\Harshan\mysql-unicharm-proxy</t>
         </is>
       </c>
-      <c r="P39" s="4" t="inlineStr">
+      <c r="Q39" s="4" t="inlineStr">
         <is>
           <t>Deprecated — replaced by selfaware-dev-stack</t>
         </is>
       </c>
-      <c r="Q39" s="4" t="inlineStr"/>
       <c r="R39" s="4" t="inlineStr"/>
+      <c r="S39" s="4" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
@@ -3271,57 +3467,62 @@
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
+          <t>Graylinx</t>
+        </is>
+      </c>
+      <c r="G40" s="4" t="inlineStr">
+        <is>
           <t>SSH key storage / Graylinx laptop identity (kept out of git for security).</t>
         </is>
       </c>
-      <c r="G40" s="4" t="inlineStr">
+      <c r="H40" s="4" t="inlineStr">
         <is>
           <t>Access/identity setup.</t>
         </is>
       </c>
-      <c r="H40" s="4" t="inlineStr">
+      <c r="I40" s="4" t="inlineStr">
         <is>
           <t>SSH</t>
         </is>
       </c>
-      <c r="I40" s="4" t="inlineStr">
+      <c r="J40" s="4" t="inlineStr">
         <is>
           <t>2026-05-18</t>
         </is>
       </c>
-      <c r="J40" s="4" t="inlineStr">
+      <c r="K40" s="4" t="inlineStr">
         <is>
           <t>2026-05-18</t>
         </is>
       </c>
-      <c r="K40" s="4" t="inlineStr">
+      <c r="L40" s="4" t="inlineStr">
         <is>
           <t>approx</t>
         </is>
       </c>
-      <c r="L40" s="5" t="inlineStr">
+      <c r="M40" s="5" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="M40" s="4" t="n">
+      <c r="N40" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="N40" s="4" t="n">
+      <c r="O40" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="O40" s="4" t="inlineStr">
+      <c r="P40" s="4" t="inlineStr">
         <is>
           <t>D:\Harshan\kimo-ssh-keys</t>
         </is>
       </c>
-      <c r="P40" s="4" t="inlineStr">
+      <c r="Q40" s="4" t="inlineStr">
         <is>
           <t>Laptop identity &amp; access keys</t>
         </is>
       </c>
-      <c r="Q40" s="4" t="inlineStr"/>
       <c r="R40" s="4" t="inlineStr"/>
+      <c r="S40" s="4" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
@@ -3347,57 +3548,62 @@
       </c>
       <c r="F41" s="6" t="inlineStr">
         <is>
+          <t>Graylinx</t>
+        </is>
+      </c>
+      <c r="G41" s="6" t="inlineStr">
+        <is>
           <t>ETL / transformer-layer workstream (planning + follow-ups in May).</t>
         </is>
       </c>
-      <c r="G41" s="6" t="inlineStr">
+      <c r="H41" s="6" t="inlineStr">
         <is>
           <t>ETL transformer-layer planning and conversion-workflow design.</t>
         </is>
       </c>
-      <c r="H41" s="6" t="inlineStr">
+      <c r="I41" s="6" t="inlineStr">
         <is>
           <t>Python; ETL</t>
         </is>
       </c>
-      <c r="I41" s="6" t="inlineStr">
+      <c r="J41" s="6" t="inlineStr">
         <is>
           <t>2026-05-14</t>
         </is>
       </c>
-      <c r="J41" s="6" t="inlineStr">
+      <c r="K41" s="6" t="inlineStr">
         <is>
           <t>2026-05-25</t>
         </is>
       </c>
-      <c r="K41" s="6" t="inlineStr">
+      <c r="L41" s="6" t="inlineStr">
         <is>
           <t>manual</t>
         </is>
       </c>
-      <c r="L41" s="7" t="inlineStr">
+      <c r="M41" s="7" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
-      <c r="M41" s="6" t="n">
+      <c r="N41" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="N41" s="6" t="n">
+      <c r="O41" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="O41" s="6" t="inlineStr">
+      <c r="P41" s="6" t="inlineStr">
         <is>
           <t>D:\Harshan\python-etl</t>
         </is>
       </c>
-      <c r="P41" s="6" t="inlineStr">
+      <c r="Q41" s="6" t="inlineStr">
         <is>
           <t>ETL transformer layer planning</t>
         </is>
       </c>
-      <c r="Q41" s="6" t="inlineStr"/>
       <c r="R41" s="6" t="inlineStr"/>
+      <c r="S41" s="6" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
@@ -3423,57 +3629,62 @@
       </c>
       <c r="F42" s="6" t="inlineStr">
         <is>
+          <t>Personal</t>
+        </is>
+      </c>
+      <c r="G42" s="6" t="inlineStr">
+        <is>
           <t>Raspberry Pi / edge experiments (placeholder).</t>
         </is>
       </c>
-      <c r="G42" s="6" t="inlineStr">
+      <c r="H42" s="6" t="inlineStr">
         <is>
           <t>Edge hardware experiments.</t>
         </is>
       </c>
-      <c r="H42" s="6" t="inlineStr">
+      <c r="I42" s="6" t="inlineStr">
         <is>
           <t>Raspberry Pi</t>
         </is>
       </c>
-      <c r="I42" s="6" t="inlineStr">
+      <c r="J42" s="6" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="J42" s="6" t="inlineStr">
+      <c r="K42" s="6" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="K42" s="6" t="inlineStr">
+      <c r="L42" s="6" t="inlineStr">
         <is>
           <t>approx</t>
         </is>
       </c>
-      <c r="L42" s="7" t="inlineStr">
+      <c r="M42" s="7" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
-      <c r="M42" s="6" t="n">
+      <c r="N42" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="N42" s="6" t="n">
+      <c r="O42" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="O42" s="6" t="inlineStr">
+      <c r="P42" s="6" t="inlineStr">
         <is>
           <t>D:\Harshan\Rasberry-stuffs</t>
         </is>
       </c>
-      <c r="P42" s="6" t="inlineStr">
+      <c r="Q42" s="6" t="inlineStr">
         <is>
           <t>Placeholder</t>
         </is>
       </c>
-      <c r="Q42" s="6" t="inlineStr"/>
       <c r="R42" s="6" t="inlineStr"/>
+      <c r="S42" s="6" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
@@ -3499,53 +3710,58 @@
       </c>
       <c r="F43" s="4" t="inlineStr">
         <is>
+          <t>Graylinx</t>
+        </is>
+      </c>
+      <c r="G43" s="4" t="inlineStr">
+        <is>
           <t>"HVAC Data Pipeline v2" — first Graylinx HVAC repo (Python), precursor to ClimaStream.</t>
         </is>
       </c>
-      <c r="G43" s="4" t="inlineStr">
+      <c r="H43" s="4" t="inlineStr">
         <is>
           <t>Initial HVAC data-pipeline prototype.</t>
         </is>
       </c>
-      <c r="H43" s="4" t="inlineStr">
+      <c r="I43" s="4" t="inlineStr">
         <is>
           <t>Python</t>
         </is>
       </c>
-      <c r="I43" s="4" t="inlineStr">
+      <c r="J43" s="4" t="inlineStr">
         <is>
           <t>2026-04-20</t>
         </is>
       </c>
-      <c r="J43" s="4" t="inlineStr">
+      <c r="K43" s="4" t="inlineStr">
         <is>
           <t>2026-04-21</t>
         </is>
       </c>
-      <c r="K43" s="4" t="inlineStr">
+      <c r="L43" s="4" t="inlineStr">
         <is>
           <t>github</t>
         </is>
       </c>
-      <c r="L43" s="5" t="inlineStr">
+      <c r="M43" s="5" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="M43" s="4" t="n">
+      <c r="N43" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="N43" s="4" t="n">
+      <c r="O43" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="O43" s="4" t="inlineStr"/>
-      <c r="P43" s="4" t="inlineStr">
+      <c r="P43" s="4" t="inlineStr"/>
+      <c r="Q43" s="4" t="inlineStr">
         <is>
           <t>First HVAC repo on GitHub (8 commits); Precursor to ClimaStream</t>
         </is>
       </c>
-      <c r="Q43" s="4" t="inlineStr"/>
       <c r="R43" s="4" t="inlineStr"/>
+      <c r="S43" s="4" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
@@ -3571,53 +3787,58 @@
       </c>
       <c r="F44" s="4" t="inlineStr">
         <is>
+          <t>Graylinx</t>
+        </is>
+      </c>
+      <c r="G44" s="4" t="inlineStr">
+        <is>
           <t>Audit/analysis of the Graylinx legacy codebase that informed the v2/OMNYX rebuild.</t>
         </is>
       </c>
-      <c r="G44" s="4" t="inlineStr">
+      <c r="H44" s="4" t="inlineStr">
         <is>
           <t>Reviewed &amp; documented legacy code for migration.</t>
         </is>
       </c>
-      <c r="H44" s="4" t="inlineStr">
+      <c r="I44" s="4" t="inlineStr">
         <is>
           <t>JavaScript; Node.js</t>
         </is>
       </c>
-      <c r="I44" s="4" t="inlineStr">
+      <c r="J44" s="4" t="inlineStr">
         <is>
           <t>2026-04-28</t>
         </is>
       </c>
-      <c r="J44" s="4" t="inlineStr">
+      <c r="K44" s="4" t="inlineStr">
         <is>
           <t>2026-05-01</t>
         </is>
       </c>
-      <c r="K44" s="4" t="inlineStr">
+      <c r="L44" s="4" t="inlineStr">
         <is>
           <t>github</t>
         </is>
       </c>
-      <c r="L44" s="5" t="inlineStr">
+      <c r="M44" s="5" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="M44" s="4" t="n">
+      <c r="N44" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="N44" s="4" t="n">
+      <c r="O44" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="O44" s="4" t="inlineStr"/>
-      <c r="P44" s="4" t="inlineStr">
+      <c r="P44" s="4" t="inlineStr"/>
+      <c r="Q44" s="4" t="inlineStr">
         <is>
           <t>Legacy code audit (7 commits); Fed into OMNYX architecture</t>
         </is>
       </c>
-      <c r="Q44" s="4" t="inlineStr"/>
       <c r="R44" s="4" t="inlineStr"/>
+      <c r="S44" s="4" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
@@ -3643,53 +3864,58 @@
       </c>
       <c r="F45" s="4" t="inlineStr">
         <is>
+          <t>Graylinx</t>
+        </is>
+      </c>
+      <c r="G45" s="4" t="inlineStr">
+        <is>
           <t>Graylinx HVAC Chiller-Plant telemetry pipeline: Node.js → MySQL + Kafka → MinIO (Parquet + manifests) → Airflow → ClickHouse → Grafana. v1 + production-ready v2 on the harshan-aiyappa account (Nov 2025).</t>
         </is>
       </c>
-      <c r="G45" s="4" t="inlineStr">
+      <c r="H45" s="4" t="inlineStr">
         <is>
           <t>Built the end-to-end pipeline + its 3 POCs with J. Suryanarayanan &amp; Satish Krishna; milestone-tracked over email.</t>
         </is>
       </c>
-      <c r="H45" s="4" t="inlineStr">
+      <c r="I45" s="4" t="inlineStr">
         <is>
           <t>Node.js; Express; Kafka; MinIO; Parquet; Airflow; ClickHouse; Grafana; Python; Docker</t>
         </is>
       </c>
-      <c r="I45" s="4" t="inlineStr">
+      <c r="J45" s="4" t="inlineStr">
         <is>
           <t>2025-11-19</t>
         </is>
       </c>
-      <c r="J45" s="4" t="inlineStr">
+      <c r="K45" s="4" t="inlineStr">
         <is>
           <t>2025-11-26</t>
         </is>
       </c>
-      <c r="K45" s="4" t="inlineStr">
+      <c r="L45" s="4" t="inlineStr">
         <is>
           <t>github</t>
         </is>
       </c>
-      <c r="L45" s="5" t="inlineStr">
+      <c r="M45" s="5" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="M45" s="4" t="n">
+      <c r="N45" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="N45" s="4" t="n">
+      <c r="O45" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="O45" s="4" t="inlineStr"/>
-      <c r="P45" s="4" t="inlineStr">
+      <c r="P45" s="4" t="inlineStr"/>
+      <c r="Q45" s="4" t="inlineStr">
         <is>
           <t>Chiller-plant predictive-maintenance + energy-optimization pipeline; v1 (19 Nov) + production v2 (26 Nov 2025), harshan-aiyappa account; POCs: Ingestion · Data Lake · Analytics</t>
         </is>
       </c>
-      <c r="Q45" s="4" t="inlineStr"/>
       <c r="R45" s="4" t="inlineStr"/>
+      <c r="S45" s="4" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
@@ -3719,41 +3945,46 @@
       </c>
       <c r="F46" s="4" t="inlineStr">
         <is>
+          <t>Graylinx</t>
+        </is>
+      </c>
+      <c r="G46" s="4" t="inlineStr">
+        <is>
           <t>Simulator → Node.js service → MySQL + Kafka</t>
         </is>
       </c>
-      <c r="G46" s="4" t="inlineStr"/>
       <c r="H46" s="4" t="inlineStr"/>
-      <c r="I46" s="4" t="inlineStr">
+      <c r="I46" s="4" t="inlineStr"/>
+      <c r="J46" s="4" t="inlineStr">
         <is>
           <t>2025-11-19</t>
         </is>
       </c>
-      <c r="J46" s="4" t="inlineStr">
+      <c r="K46" s="4" t="inlineStr">
         <is>
           <t>2025-11-21</t>
         </is>
       </c>
-      <c r="K46" s="4" t="inlineStr">
+      <c r="L46" s="4" t="inlineStr">
         <is>
           <t>github</t>
         </is>
       </c>
-      <c r="L46" s="5" t="inlineStr">
+      <c r="M46" s="5" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="M46" s="4" t="n">
+      <c r="N46" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="N46" s="4" t="n">
+      <c r="O46" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="O46" s="4" t="inlineStr"/>
       <c r="P46" s="4" t="inlineStr"/>
       <c r="Q46" s="4" t="inlineStr"/>
       <c r="R46" s="4" t="inlineStr"/>
+      <c r="S46" s="4" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
@@ -3783,41 +4014,46 @@
       </c>
       <c r="F47" s="4" t="inlineStr">
         <is>
+          <t>Graylinx</t>
+        </is>
+      </c>
+      <c r="G47" s="4" t="inlineStr">
+        <is>
           <t>Kafka → connector → MinIO Parquet storage</t>
         </is>
       </c>
-      <c r="G47" s="4" t="inlineStr"/>
       <c r="H47" s="4" t="inlineStr"/>
-      <c r="I47" s="4" t="inlineStr">
+      <c r="I47" s="4" t="inlineStr"/>
+      <c r="J47" s="4" t="inlineStr">
         <is>
           <t>2025-11-21</t>
         </is>
       </c>
-      <c r="J47" s="4" t="inlineStr">
+      <c r="K47" s="4" t="inlineStr">
         <is>
           <t>2025-11-23</t>
         </is>
       </c>
-      <c r="K47" s="4" t="inlineStr">
+      <c r="L47" s="4" t="inlineStr">
         <is>
           <t>github</t>
         </is>
       </c>
-      <c r="L47" s="5" t="inlineStr">
+      <c r="M47" s="5" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="M47" s="4" t="n">
+      <c r="N47" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="N47" s="4" t="n">
+      <c r="O47" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="O47" s="4" t="inlineStr"/>
       <c r="P47" s="4" t="inlineStr"/>
       <c r="Q47" s="4" t="inlineStr"/>
       <c r="R47" s="4" t="inlineStr"/>
+      <c r="S47" s="4" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
@@ -3847,41 +4083,46 @@
       </c>
       <c r="F48" s="4" t="inlineStr">
         <is>
+          <t>Graylinx</t>
+        </is>
+      </c>
+      <c r="G48" s="4" t="inlineStr">
+        <is>
           <t>MinIO → Airflow → ClickHouse → Grafana dashboards</t>
         </is>
       </c>
-      <c r="G48" s="4" t="inlineStr"/>
       <c r="H48" s="4" t="inlineStr"/>
-      <c r="I48" s="4" t="inlineStr">
+      <c r="I48" s="4" t="inlineStr"/>
+      <c r="J48" s="4" t="inlineStr">
         <is>
           <t>2025-11-23</t>
         </is>
       </c>
-      <c r="J48" s="4" t="inlineStr">
+      <c r="K48" s="4" t="inlineStr">
         <is>
           <t>2025-11-26</t>
         </is>
       </c>
-      <c r="K48" s="4" t="inlineStr">
+      <c r="L48" s="4" t="inlineStr">
         <is>
           <t>github</t>
         </is>
       </c>
-      <c r="L48" s="5" t="inlineStr">
+      <c r="M48" s="5" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="M48" s="4" t="n">
+      <c r="N48" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="N48" s="4" t="n">
+      <c r="O48" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="O48" s="4" t="inlineStr"/>
       <c r="P48" s="4" t="inlineStr"/>
       <c r="Q48" s="4" t="inlineStr"/>
       <c r="R48" s="4" t="inlineStr"/>
+      <c r="S48" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore(data): remove TripTrail (RANGSONS) and Concept Standard projects (per Harshan)
Commented out (one-line restorable) in build_tracker.py, matching the curated
VS Code workspace folder list. Both are non-Graylinx:
- TripTrail — Travel & Expense: RANGSONS LLP client app
- Concept Standard — Graph Analytics: personal SelfAware-adjacent tool

Now 19 projects (Graylinx 13 / Personal 4 / Client 2); span unchanged
(Nov 19 2025 -> Jun 15 2026); 900 commits. Seed re-injected; public/ synced.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/works.xlsx
+++ b/works.xlsx
@@ -520,7 +520,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S48"/>
+  <dimension ref="A1:S46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -707,7 +707,7 @@
         <v>70</v>
       </c>
       <c r="O2" s="2" t="n">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
@@ -2877,90 +2877,90 @@
       <c r="S32" s="4" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>concept-standard</t>
-        </is>
-      </c>
-      <c r="B33" s="2" t="inlineStr"/>
-      <c r="C33" s="2" t="inlineStr">
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t>voxara</t>
+        </is>
+      </c>
+      <c r="B33" s="6" t="inlineStr"/>
+      <c r="C33" s="6" t="inlineStr">
         <is>
           <t>project</t>
         </is>
       </c>
-      <c r="D33" s="2" t="inlineStr">
-        <is>
-          <t>Concept Standard — Graph Analytics</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="inlineStr">
-        <is>
-          <t>SelfAware Suite</t>
-        </is>
-      </c>
-      <c r="F33" s="2" t="inlineStr">
+      <c r="D33" s="6" t="inlineStr">
+        <is>
+          <t>VOXARA AI — Voice Intelligence</t>
+        </is>
+      </c>
+      <c r="E33" s="6" t="inlineStr">
+        <is>
+          <t>Voice AI</t>
+        </is>
+      </c>
+      <c r="F33" s="6" t="inlineStr">
         <is>
           <t>Personal</t>
         </is>
       </c>
-      <c r="G33" s="2" t="inlineStr">
-        <is>
-          <t>Interactive concept-map viewer (1,159 concepts, 5,985 relations) for lesson generation.</t>
-        </is>
-      </c>
-      <c r="H33" s="2" t="inlineStr">
-        <is>
-          <t>Built the in-browser graph analytics tool (ECharts + Neo4j GDS).</t>
-        </is>
-      </c>
-      <c r="I33" s="2" t="inlineStr">
-        <is>
-          <t>Python; JavaScript; ECharts; Neo4j</t>
-        </is>
-      </c>
-      <c r="J33" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="K33" s="2" t="inlineStr">
-        <is>
-          <t>ongoing</t>
-        </is>
-      </c>
-      <c r="L33" s="2" t="inlineStr">
+      <c r="G33" s="6" t="inlineStr">
+        <is>
+          <t>Realtime on-prem AI voice intelligence platform — monorepo with local LLM, Whisper STT, Piper TTS.</t>
+        </is>
+      </c>
+      <c r="H33" s="6" t="inlineStr">
+        <is>
+          <t>Architecture &amp; monorepo setup (pnpm/Turbo), service scaffolding.</t>
+        </is>
+      </c>
+      <c r="I33" s="6" t="inlineStr">
+        <is>
+          <t>Node.js; pnpm; Turbo; Ollama; Whisper; Piper; Docker</t>
+        </is>
+      </c>
+      <c r="J33" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="K33" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="L33" s="6" t="inlineStr">
         <is>
           <t>approx</t>
         </is>
       </c>
-      <c r="M33" s="3" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="N33" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="O33" s="2" t="n">
+      <c r="M33" s="7" t="inlineStr">
+        <is>
+          <t>Paused</t>
+        </is>
+      </c>
+      <c r="N33" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="O33" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="P33" s="2" t="inlineStr">
-        <is>
-          <t>D:\Harshan\concept-standard</t>
-        </is>
-      </c>
-      <c r="Q33" s="2" t="inlineStr">
-        <is>
-          <t>1,159 concepts / 5,985 relations; Force/circular graphs, command palette, light/dark, a11y</t>
-        </is>
-      </c>
-      <c r="R33" s="2" t="inlineStr"/>
-      <c r="S33" s="2" t="inlineStr"/>
+      <c r="P33" s="6" t="inlineStr">
+        <is>
+          <t>D:\Harshan\VOXARA AI</t>
+        </is>
+      </c>
+      <c r="Q33" s="6" t="inlineStr">
+        <is>
+          <t>Largest by file count (37 items); Local LLM + Whisper + Piper TTS</t>
+        </is>
+      </c>
+      <c r="R33" s="6" t="inlineStr"/>
+      <c r="S33" s="6" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>voxara</t>
+          <t>konva</t>
         </is>
       </c>
       <c r="B34" s="6" t="inlineStr"/>
@@ -2971,42 +2971,42 @@
       </c>
       <c r="D34" s="6" t="inlineStr">
         <is>
-          <t>VOXARA AI — Voice Intelligence</t>
+          <t>Konva Canvas App</t>
         </is>
       </c>
       <c r="E34" s="6" t="inlineStr">
         <is>
-          <t>Voice AI</t>
+          <t>Client Apps</t>
         </is>
       </c>
       <c r="F34" s="6" t="inlineStr">
         <is>
-          <t>Personal</t>
+          <t>Client</t>
         </is>
       </c>
       <c r="G34" s="6" t="inlineStr">
         <is>
-          <t>Realtime on-prem AI voice intelligence platform — monorepo with local LLM, Whisper STT, Piper TTS.</t>
+          <t>React + TypeScript canvas/drawing app template (likely a UI/design component base).</t>
         </is>
       </c>
       <c r="H34" s="6" t="inlineStr">
         <is>
-          <t>Architecture &amp; monorepo setup (pnpm/Turbo), service scaffolding.</t>
+          <t>Template/prototype setup.</t>
         </is>
       </c>
       <c r="I34" s="6" t="inlineStr">
         <is>
-          <t>Node.js; pnpm; Turbo; Ollama; Whisper; Piper; Docker</t>
+          <t>React; TypeScript; Vite; Konva</t>
         </is>
       </c>
       <c r="J34" s="6" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="K34" s="6" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="L34" s="6" t="inlineStr">
@@ -3020,271 +3020,271 @@
         </is>
       </c>
       <c r="N34" s="6" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="O34" s="6" t="n">
         <v>0</v>
       </c>
       <c r="P34" s="6" t="inlineStr">
         <is>
-          <t>D:\Harshan\VOXARA AI</t>
+          <t>D:\Harshan\konva</t>
         </is>
       </c>
       <c r="Q34" s="6" t="inlineStr">
         <is>
-          <t>Largest by file count (37 items); Local LLM + Whisper + Piper TTS</t>
+          <t>Canvas/drawing UI base</t>
         </is>
       </c>
       <c r="R34" s="6" t="inlineStr"/>
       <c r="S34" s="6" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="4" t="inlineStr">
-        <is>
-          <t>travel-app</t>
-        </is>
-      </c>
-      <c r="B35" s="4" t="inlineStr"/>
-      <c r="C35" s="4" t="inlineStr">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>farmer-app</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr"/>
+      <c r="C35" s="2" t="inlineStr">
         <is>
           <t>project</t>
         </is>
       </c>
-      <c r="D35" s="4" t="inlineStr">
-        <is>
-          <t>TripTrail — Travel &amp; Expense (RANGSONS)</t>
-        </is>
-      </c>
-      <c r="E35" s="4" t="inlineStr">
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Nesso — Farm Traceability Platform</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
         <is>
           <t>Client Apps</t>
         </is>
       </c>
-      <c r="F35" s="4" t="inlineStr">
+      <c r="F35" s="2" t="inlineStr">
         <is>
           <t>Client</t>
         </is>
       </c>
-      <c r="G35" s="4" t="inlineStr">
-        <is>
-          <t>Buildless travel/expense reporting web app for RANGSONS LLP with HR approval + Google Sheets.</t>
-        </is>
-      </c>
-      <c r="H35" s="4" t="inlineStr">
-        <is>
-          <t>Sole developer — static web app, Supabase backend, approval flow.</t>
-        </is>
-      </c>
-      <c r="I35" s="4" t="inlineStr">
-        <is>
-          <t>HTML; Tailwind; JavaScript; Supabase</t>
-        </is>
-      </c>
-      <c r="J35" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-03</t>
-        </is>
-      </c>
-      <c r="K35" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-03</t>
-        </is>
-      </c>
-      <c r="L35" s="4" t="inlineStr">
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>Farm-to-fork traceability platform for NR Group (Nesso).</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>Built the traceability web app — including a weekend build sprint (30–31 May).</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>TypeScript; React; Node.js</t>
+        </is>
+      </c>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t>ongoing</t>
+        </is>
+      </c>
+      <c r="L35" s="2" t="inlineStr">
         <is>
           <t>git</t>
         </is>
       </c>
-      <c r="M35" s="5" t="inlineStr">
+      <c r="M35" s="3" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="N35" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="O35" s="2" t="n">
+        <v>191</v>
+      </c>
+      <c r="P35" s="2" t="inlineStr">
+        <is>
+          <t>D:\Harshan\farmer-app</t>
+        </is>
+      </c>
+      <c r="Q35" s="2" t="inlineStr">
+        <is>
+          <t>Farm-to-fork traceability (NR Group); ~1-week build incl. weekend sprint</t>
+        </is>
+      </c>
+      <c r="R35" s="2" t="inlineStr"/>
+      <c r="S35" s="2" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>selfaware-dev-stack</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr"/>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>project</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>SelfAware Dev Stack</t>
+        </is>
+      </c>
+      <c r="E36" s="4" t="inlineStr">
+        <is>
+          <t>Infra &amp; Tooling</t>
+        </is>
+      </c>
+      <c r="F36" s="4" t="inlineStr">
+        <is>
+          <t>Personal</t>
+        </is>
+      </c>
+      <c r="G36" s="4" t="inlineStr">
+        <is>
+          <t>Canonical local Docker dev stack (MySQL, PostgreSQL, Neo4j, Redis) for the SelfAware products.</t>
+        </is>
+      </c>
+      <c r="H36" s="4" t="inlineStr">
+        <is>
+          <t>Authored the docker-compose environment for 4 products.</t>
+        </is>
+      </c>
+      <c r="I36" s="4" t="inlineStr">
+        <is>
+          <t>Docker; MySQL; PostgreSQL; Neo4j; Redis</t>
+        </is>
+      </c>
+      <c r="J36" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="K36" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="L36" s="4" t="inlineStr">
+        <is>
+          <t>approx</t>
+        </is>
+      </c>
+      <c r="M36" s="5" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="N35" s="4" t="n">
+      <c r="N36" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="O35" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="P35" s="4" t="inlineStr">
-        <is>
-          <t>D:\Harshan\travel-app</t>
-        </is>
-      </c>
-      <c r="Q35" s="4" t="inlineStr">
-        <is>
-          <t>HR approval + Google Sheets integration; Buildless static deployment</t>
-        </is>
-      </c>
-      <c r="R35" s="4" t="inlineStr"/>
-      <c r="S35" s="4" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="6" t="inlineStr">
-        <is>
-          <t>konva</t>
-        </is>
-      </c>
-      <c r="B36" s="6" t="inlineStr"/>
-      <c r="C36" s="6" t="inlineStr">
+      <c r="O36" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P36" s="4" t="inlineStr">
+        <is>
+          <t>D:\Harshan\selfaware-dev-stack</t>
+        </is>
+      </c>
+      <c r="Q36" s="4" t="inlineStr">
+        <is>
+          <t>One dev environment for 4 products</t>
+        </is>
+      </c>
+      <c r="R36" s="4" t="inlineStr"/>
+      <c r="S36" s="4" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>mysql-unicharm-proxy</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr"/>
+      <c r="C37" s="4" t="inlineStr">
         <is>
           <t>project</t>
         </is>
       </c>
-      <c r="D36" s="6" t="inlineStr">
-        <is>
-          <t>Konva Canvas App</t>
-        </is>
-      </c>
-      <c r="E36" s="6" t="inlineStr">
-        <is>
-          <t>Client Apps</t>
-        </is>
-      </c>
-      <c r="F36" s="6" t="inlineStr">
-        <is>
-          <t>Client</t>
-        </is>
-      </c>
-      <c r="G36" s="6" t="inlineStr">
-        <is>
-          <t>React + TypeScript canvas/drawing app template (likely a UI/design component base).</t>
-        </is>
-      </c>
-      <c r="H36" s="6" t="inlineStr">
-        <is>
-          <t>Template/prototype setup.</t>
-        </is>
-      </c>
-      <c r="I36" s="6" t="inlineStr">
-        <is>
-          <t>React; TypeScript; Vite; Konva</t>
-        </is>
-      </c>
-      <c r="J36" s="6" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="K36" s="6" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="L36" s="6" t="inlineStr">
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>MySQL Unicharm Proxy (deprecated)</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t>Infra &amp; Tooling</t>
+        </is>
+      </c>
+      <c r="F37" s="4" t="inlineStr">
+        <is>
+          <t>Graylinx</t>
+        </is>
+      </c>
+      <c r="G37" s="4" t="inlineStr">
+        <is>
+          <t>Docker MySQL port-forwarding helper — superseded by selfaware-dev-stack.</t>
+        </is>
+      </c>
+      <c r="H37" s="4" t="inlineStr">
+        <is>
+          <t>Quick infra utility (now reference-only).</t>
+        </is>
+      </c>
+      <c r="I37" s="4" t="inlineStr">
+        <is>
+          <t>Docker; MySQL</t>
+        </is>
+      </c>
+      <c r="J37" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="K37" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="L37" s="4" t="inlineStr">
         <is>
           <t>approx</t>
         </is>
       </c>
-      <c r="M36" s="7" t="inlineStr">
-        <is>
-          <t>Paused</t>
-        </is>
-      </c>
-      <c r="N36" s="6" t="n">
-        <v>25</v>
-      </c>
-      <c r="O36" s="6" t="n">
+      <c r="M37" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N37" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="O37" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="P36" s="6" t="inlineStr">
-        <is>
-          <t>D:\Harshan\konva</t>
-        </is>
-      </c>
-      <c r="Q36" s="6" t="inlineStr">
-        <is>
-          <t>Canvas/drawing UI base</t>
-        </is>
-      </c>
-      <c r="R36" s="6" t="inlineStr"/>
-      <c r="S36" s="6" t="inlineStr"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="2" t="inlineStr">
-        <is>
-          <t>farmer-app</t>
-        </is>
-      </c>
-      <c r="B37" s="2" t="inlineStr"/>
-      <c r="C37" s="2" t="inlineStr">
-        <is>
-          <t>project</t>
-        </is>
-      </c>
-      <c r="D37" s="2" t="inlineStr">
-        <is>
-          <t>Nesso — Farm Traceability Platform</t>
-        </is>
-      </c>
-      <c r="E37" s="2" t="inlineStr">
-        <is>
-          <t>Client Apps</t>
-        </is>
-      </c>
-      <c r="F37" s="2" t="inlineStr">
-        <is>
-          <t>Client</t>
-        </is>
-      </c>
-      <c r="G37" s="2" t="inlineStr">
-        <is>
-          <t>Farm-to-fork traceability platform for NR Group (Nesso).</t>
-        </is>
-      </c>
-      <c r="H37" s="2" t="inlineStr">
-        <is>
-          <t>Built the traceability web app — including a weekend build sprint (30–31 May).</t>
-        </is>
-      </c>
-      <c r="I37" s="2" t="inlineStr">
-        <is>
-          <t>TypeScript; React; Node.js</t>
-        </is>
-      </c>
-      <c r="J37" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
-      <c r="K37" s="2" t="inlineStr">
-        <is>
-          <t>ongoing</t>
-        </is>
-      </c>
-      <c r="L37" s="2" t="inlineStr">
-        <is>
-          <t>git</t>
-        </is>
-      </c>
-      <c r="M37" s="3" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="N37" s="2" t="n">
-        <v>45</v>
-      </c>
-      <c r="O37" s="2" t="n">
-        <v>191</v>
-      </c>
-      <c r="P37" s="2" t="inlineStr">
-        <is>
-          <t>D:\Harshan\farmer-app</t>
-        </is>
-      </c>
-      <c r="Q37" s="2" t="inlineStr">
-        <is>
-          <t>Farm-to-fork traceability (NR Group); ~1-week build incl. weekend sprint</t>
-        </is>
-      </c>
-      <c r="R37" s="2" t="inlineStr"/>
-      <c r="S37" s="2" t="inlineStr"/>
+      <c r="P37" s="4" t="inlineStr">
+        <is>
+          <t>D:\Harshan\mysql-unicharm-proxy</t>
+        </is>
+      </c>
+      <c r="Q37" s="4" t="inlineStr">
+        <is>
+          <t>Deprecated — replaced by selfaware-dev-stack</t>
+        </is>
+      </c>
+      <c r="R37" s="4" t="inlineStr"/>
+      <c r="S37" s="4" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>selfaware-dev-stack</t>
+          <t>kimo-ssh-keys</t>
         </is>
       </c>
       <c r="B38" s="4" t="inlineStr"/>
@@ -3295,7 +3295,7 @@
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>SelfAware Dev Stack</t>
+          <t>Kimo SSH Keys</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr">
@@ -3305,32 +3305,32 @@
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>Personal</t>
+          <t>Graylinx</t>
         </is>
       </c>
       <c r="G38" s="4" t="inlineStr">
         <is>
-          <t>Canonical local Docker dev stack (MySQL, PostgreSQL, Neo4j, Redis) for the SelfAware products.</t>
+          <t>SSH key storage / Graylinx laptop identity (kept out of git for security).</t>
         </is>
       </c>
       <c r="H38" s="4" t="inlineStr">
         <is>
-          <t>Authored the docker-compose environment for 4 products.</t>
+          <t>Access/identity setup.</t>
         </is>
       </c>
       <c r="I38" s="4" t="inlineStr">
         <is>
-          <t>Docker; MySQL; PostgreSQL; Neo4j; Redis</t>
+          <t>SSH</t>
         </is>
       </c>
       <c r="J38" s="4" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="K38" s="4" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="L38" s="4" t="inlineStr">
@@ -3351,345 +3351,337 @@
       </c>
       <c r="P38" s="4" t="inlineStr">
         <is>
-          <t>D:\Harshan\selfaware-dev-stack</t>
+          <t>D:\Harshan\kimo-ssh-keys</t>
         </is>
       </c>
       <c r="Q38" s="4" t="inlineStr">
         <is>
-          <t>One dev environment for 4 products</t>
+          <t>Laptop identity &amp; access keys</t>
         </is>
       </c>
       <c r="R38" s="4" t="inlineStr"/>
       <c r="S38" s="4" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" s="4" t="inlineStr">
-        <is>
-          <t>mysql-unicharm-proxy</t>
-        </is>
-      </c>
-      <c r="B39" s="4" t="inlineStr"/>
-      <c r="C39" s="4" t="inlineStr">
+      <c r="A39" s="6" t="inlineStr">
+        <is>
+          <t>python-etl</t>
+        </is>
+      </c>
+      <c r="B39" s="6" t="inlineStr"/>
+      <c r="C39" s="6" t="inlineStr">
         <is>
           <t>project</t>
         </is>
       </c>
-      <c r="D39" s="4" t="inlineStr">
-        <is>
-          <t>MySQL Unicharm Proxy (deprecated)</t>
-        </is>
-      </c>
-      <c r="E39" s="4" t="inlineStr">
+      <c r="D39" s="6" t="inlineStr">
+        <is>
+          <t>Python ETL</t>
+        </is>
+      </c>
+      <c r="E39" s="6" t="inlineStr">
         <is>
           <t>Infra &amp; Tooling</t>
         </is>
       </c>
-      <c r="F39" s="4" t="inlineStr">
+      <c r="F39" s="6" t="inlineStr">
         <is>
           <t>Graylinx</t>
         </is>
       </c>
-      <c r="G39" s="4" t="inlineStr">
-        <is>
-          <t>Docker MySQL port-forwarding helper — superseded by selfaware-dev-stack.</t>
-        </is>
-      </c>
-      <c r="H39" s="4" t="inlineStr">
-        <is>
-          <t>Quick infra utility (now reference-only).</t>
-        </is>
-      </c>
-      <c r="I39" s="4" t="inlineStr">
-        <is>
-          <t>Docker; MySQL</t>
-        </is>
-      </c>
-      <c r="J39" s="4" t="inlineStr">
-        <is>
-          <t>2026-05-21</t>
-        </is>
-      </c>
-      <c r="K39" s="4" t="inlineStr">
-        <is>
-          <t>2026-05-21</t>
-        </is>
-      </c>
-      <c r="L39" s="4" t="inlineStr">
+      <c r="G39" s="6" t="inlineStr">
+        <is>
+          <t>ETL / transformer-layer workstream (planning + follow-ups in May).</t>
+        </is>
+      </c>
+      <c r="H39" s="6" t="inlineStr">
+        <is>
+          <t>ETL transformer-layer planning and conversion-workflow design.</t>
+        </is>
+      </c>
+      <c r="I39" s="6" t="inlineStr">
+        <is>
+          <t>Python; ETL</t>
+        </is>
+      </c>
+      <c r="J39" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="K39" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="L39" s="6" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+      <c r="M39" s="7" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="N39" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="O39" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P39" s="6" t="inlineStr">
+        <is>
+          <t>D:\Harshan\python-etl</t>
+        </is>
+      </c>
+      <c r="Q39" s="6" t="inlineStr">
+        <is>
+          <t>ETL transformer layer planning</t>
+        </is>
+      </c>
+      <c r="R39" s="6" t="inlineStr"/>
+      <c r="S39" s="6" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="6" t="inlineStr">
+        <is>
+          <t>raspberry</t>
+        </is>
+      </c>
+      <c r="B40" s="6" t="inlineStr"/>
+      <c r="C40" s="6" t="inlineStr">
+        <is>
+          <t>project</t>
+        </is>
+      </c>
+      <c r="D40" s="6" t="inlineStr">
+        <is>
+          <t>Raspberry Stuffs</t>
+        </is>
+      </c>
+      <c r="E40" s="6" t="inlineStr">
+        <is>
+          <t>Infra &amp; Tooling</t>
+        </is>
+      </c>
+      <c r="F40" s="6" t="inlineStr">
+        <is>
+          <t>Personal</t>
+        </is>
+      </c>
+      <c r="G40" s="6" t="inlineStr">
+        <is>
+          <t>Raspberry Pi / edge experiments (placeholder).</t>
+        </is>
+      </c>
+      <c r="H40" s="6" t="inlineStr">
+        <is>
+          <t>Edge hardware experiments.</t>
+        </is>
+      </c>
+      <c r="I40" s="6" t="inlineStr">
+        <is>
+          <t>Raspberry Pi</t>
+        </is>
+      </c>
+      <c r="J40" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="K40" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="L40" s="6" t="inlineStr">
         <is>
           <t>approx</t>
         </is>
       </c>
-      <c r="M39" s="5" t="inlineStr">
+      <c r="M40" s="7" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="N40" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="O40" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P40" s="6" t="inlineStr">
+        <is>
+          <t>D:\Harshan\Rasberry-stuffs</t>
+        </is>
+      </c>
+      <c r="Q40" s="6" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="R40" s="6" t="inlineStr"/>
+      <c r="S40" s="6" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>gl-hvac-early</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr"/>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>project</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>Graylinx.ai HVAC (early prototype)</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="inlineStr">
+        <is>
+          <t>HVAC Platform</t>
+        </is>
+      </c>
+      <c r="F41" s="4" t="inlineStr">
+        <is>
+          <t>Graylinx</t>
+        </is>
+      </c>
+      <c r="G41" s="4" t="inlineStr">
+        <is>
+          <t>"HVAC Data Pipeline v2" — first Graylinx HVAC repo (Python), precursor to ClimaStream.</t>
+        </is>
+      </c>
+      <c r="H41" s="4" t="inlineStr">
+        <is>
+          <t>Initial HVAC data-pipeline prototype.</t>
+        </is>
+      </c>
+      <c r="I41" s="4" t="inlineStr">
+        <is>
+          <t>Python</t>
+        </is>
+      </c>
+      <c r="J41" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="K41" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-21</t>
+        </is>
+      </c>
+      <c r="L41" s="4" t="inlineStr">
+        <is>
+          <t>github</t>
+        </is>
+      </c>
+      <c r="M41" s="5" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="N39" s="4" t="n">
+      <c r="N41" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="O39" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P39" s="4" t="inlineStr">
-        <is>
-          <t>D:\Harshan\mysql-unicharm-proxy</t>
-        </is>
-      </c>
-      <c r="Q39" s="4" t="inlineStr">
-        <is>
-          <t>Deprecated — replaced by selfaware-dev-stack</t>
-        </is>
-      </c>
-      <c r="R39" s="4" t="inlineStr"/>
-      <c r="S39" s="4" t="inlineStr"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="4" t="inlineStr">
-        <is>
-          <t>kimo-ssh-keys</t>
-        </is>
-      </c>
-      <c r="B40" s="4" t="inlineStr"/>
-      <c r="C40" s="4" t="inlineStr">
+      <c r="O41" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="P41" s="4" t="inlineStr"/>
+      <c r="Q41" s="4" t="inlineStr">
+        <is>
+          <t>First HVAC repo on GitHub (8 commits); Precursor to ClimaStream</t>
+        </is>
+      </c>
+      <c r="R41" s="4" t="inlineStr"/>
+      <c r="S41" s="4" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>gl-legacy-analysis</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr"/>
+      <c r="C42" s="4" t="inlineStr">
         <is>
           <t>project</t>
         </is>
       </c>
-      <c r="D40" s="4" t="inlineStr">
-        <is>
-          <t>Kimo SSH Keys</t>
-        </is>
-      </c>
-      <c r="E40" s="4" t="inlineStr">
-        <is>
-          <t>Infra &amp; Tooling</t>
-        </is>
-      </c>
-      <c r="F40" s="4" t="inlineStr">
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>Graylinx Legacy-Code Analysis</t>
+        </is>
+      </c>
+      <c r="E42" s="4" t="inlineStr">
+        <is>
+          <t>Graylinx Core</t>
+        </is>
+      </c>
+      <c r="F42" s="4" t="inlineStr">
         <is>
           <t>Graylinx</t>
         </is>
       </c>
-      <c r="G40" s="4" t="inlineStr">
-        <is>
-          <t>SSH key storage / Graylinx laptop identity (kept out of git for security).</t>
-        </is>
-      </c>
-      <c r="H40" s="4" t="inlineStr">
-        <is>
-          <t>Access/identity setup.</t>
-        </is>
-      </c>
-      <c r="I40" s="4" t="inlineStr">
-        <is>
-          <t>SSH</t>
-        </is>
-      </c>
-      <c r="J40" s="4" t="inlineStr">
-        <is>
-          <t>2026-05-18</t>
-        </is>
-      </c>
-      <c r="K40" s="4" t="inlineStr">
-        <is>
-          <t>2026-05-18</t>
-        </is>
-      </c>
-      <c r="L40" s="4" t="inlineStr">
-        <is>
-          <t>approx</t>
-        </is>
-      </c>
-      <c r="M40" s="5" t="inlineStr">
+      <c r="G42" s="4" t="inlineStr">
+        <is>
+          <t>Audit/analysis of the Graylinx legacy codebase that informed the v2/OMNYX rebuild.</t>
+        </is>
+      </c>
+      <c r="H42" s="4" t="inlineStr">
+        <is>
+          <t>Reviewed &amp; documented legacy code for migration.</t>
+        </is>
+      </c>
+      <c r="I42" s="4" t="inlineStr">
+        <is>
+          <t>JavaScript; Node.js</t>
+        </is>
+      </c>
+      <c r="J42" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="K42" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="L42" s="4" t="inlineStr">
+        <is>
+          <t>github</t>
+        </is>
+      </c>
+      <c r="M42" s="5" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="N40" s="4" t="n">
+      <c r="N42" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="O40" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P40" s="4" t="inlineStr">
-        <is>
-          <t>D:\Harshan\kimo-ssh-keys</t>
-        </is>
-      </c>
-      <c r="Q40" s="4" t="inlineStr">
-        <is>
-          <t>Laptop identity &amp; access keys</t>
-        </is>
-      </c>
-      <c r="R40" s="4" t="inlineStr"/>
-      <c r="S40" s="4" t="inlineStr"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="6" t="inlineStr">
-        <is>
-          <t>python-etl</t>
-        </is>
-      </c>
-      <c r="B41" s="6" t="inlineStr"/>
-      <c r="C41" s="6" t="inlineStr">
-        <is>
-          <t>project</t>
-        </is>
-      </c>
-      <c r="D41" s="6" t="inlineStr">
-        <is>
-          <t>Python ETL</t>
-        </is>
-      </c>
-      <c r="E41" s="6" t="inlineStr">
-        <is>
-          <t>Infra &amp; Tooling</t>
-        </is>
-      </c>
-      <c r="F41" s="6" t="inlineStr">
-        <is>
-          <t>Graylinx</t>
-        </is>
-      </c>
-      <c r="G41" s="6" t="inlineStr">
-        <is>
-          <t>ETL / transformer-layer workstream (planning + follow-ups in May).</t>
-        </is>
-      </c>
-      <c r="H41" s="6" t="inlineStr">
-        <is>
-          <t>ETL transformer-layer planning and conversion-workflow design.</t>
-        </is>
-      </c>
-      <c r="I41" s="6" t="inlineStr">
-        <is>
-          <t>Python; ETL</t>
-        </is>
-      </c>
-      <c r="J41" s="6" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="K41" s="6" t="inlineStr">
-        <is>
-          <t>2026-05-25</t>
-        </is>
-      </c>
-      <c r="L41" s="6" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-      <c r="M41" s="7" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="N41" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="O41" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="P41" s="6" t="inlineStr">
-        <is>
-          <t>D:\Harshan\python-etl</t>
-        </is>
-      </c>
-      <c r="Q41" s="6" t="inlineStr">
-        <is>
-          <t>ETL transformer layer planning</t>
-        </is>
-      </c>
-      <c r="R41" s="6" t="inlineStr"/>
-      <c r="S41" s="6" t="inlineStr"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="6" t="inlineStr">
-        <is>
-          <t>raspberry</t>
-        </is>
-      </c>
-      <c r="B42" s="6" t="inlineStr"/>
-      <c r="C42" s="6" t="inlineStr">
-        <is>
-          <t>project</t>
-        </is>
-      </c>
-      <c r="D42" s="6" t="inlineStr">
-        <is>
-          <t>Raspberry Stuffs</t>
-        </is>
-      </c>
-      <c r="E42" s="6" t="inlineStr">
-        <is>
-          <t>Infra &amp; Tooling</t>
-        </is>
-      </c>
-      <c r="F42" s="6" t="inlineStr">
-        <is>
-          <t>Personal</t>
-        </is>
-      </c>
-      <c r="G42" s="6" t="inlineStr">
-        <is>
-          <t>Raspberry Pi / edge experiments (placeholder).</t>
-        </is>
-      </c>
-      <c r="H42" s="6" t="inlineStr">
-        <is>
-          <t>Edge hardware experiments.</t>
-        </is>
-      </c>
-      <c r="I42" s="6" t="inlineStr">
-        <is>
-          <t>Raspberry Pi</t>
-        </is>
-      </c>
-      <c r="J42" s="6" t="inlineStr">
-        <is>
-          <t>2026-06-13</t>
-        </is>
-      </c>
-      <c r="K42" s="6" t="inlineStr">
-        <is>
-          <t>2026-06-13</t>
-        </is>
-      </c>
-      <c r="L42" s="6" t="inlineStr">
-        <is>
-          <t>approx</t>
-        </is>
-      </c>
-      <c r="M42" s="7" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="N42" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="O42" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="P42" s="6" t="inlineStr">
-        <is>
-          <t>D:\Harshan\Rasberry-stuffs</t>
-        </is>
-      </c>
-      <c r="Q42" s="6" t="inlineStr">
-        <is>
-          <t>Placeholder</t>
-        </is>
-      </c>
-      <c r="R42" s="6" t="inlineStr"/>
-      <c r="S42" s="6" t="inlineStr"/>
+      <c r="O42" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="P42" s="4" t="inlineStr"/>
+      <c r="Q42" s="4" t="inlineStr">
+        <is>
+          <t>Legacy code audit (7 commits); Fed into OMNYX architecture</t>
+        </is>
+      </c>
+      <c r="R42" s="4" t="inlineStr"/>
+      <c r="S42" s="4" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>gl-hvac-early</t>
+          <t>poc-hvac-pipeline</t>
         </is>
       </c>
       <c r="B43" s="4" t="inlineStr"/>
@@ -3700,7 +3692,7 @@
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>Graylinx.ai HVAC (early prototype)</t>
+          <t>HVAC Data Pipeline (v1 &amp; v2)</t>
         </is>
       </c>
       <c r="E43" s="4" t="inlineStr">
@@ -3715,27 +3707,27 @@
       </c>
       <c r="G43" s="4" t="inlineStr">
         <is>
-          <t>"HVAC Data Pipeline v2" — first Graylinx HVAC repo (Python), precursor to ClimaStream.</t>
+          <t>Graylinx HVAC Chiller-Plant telemetry pipeline: Node.js → MySQL + Kafka → MinIO (Parquet + manifests) → Airflow → ClickHouse → Grafana. v1 + production-ready v2 on the harshan-aiyappa account (Nov 2025).</t>
         </is>
       </c>
       <c r="H43" s="4" t="inlineStr">
         <is>
-          <t>Initial HVAC data-pipeline prototype.</t>
+          <t>Built the end-to-end pipeline + its 3 POCs with J. Suryanarayanan &amp; Satish Krishna; milestone-tracked over email.</t>
         </is>
       </c>
       <c r="I43" s="4" t="inlineStr">
         <is>
-          <t>Python</t>
+          <t>Node.js; Express; Kafka; MinIO; Parquet; Airflow; ClickHouse; Grafana; Python; Docker</t>
         </is>
       </c>
       <c r="J43" s="4" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2025-11-19</t>
         </is>
       </c>
       <c r="K43" s="4" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2025-11-26</t>
         </is>
       </c>
       <c r="L43" s="4" t="inlineStr">
@@ -3752,12 +3744,12 @@
         <v>100</v>
       </c>
       <c r="O43" s="4" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="P43" s="4" t="inlineStr"/>
       <c r="Q43" s="4" t="inlineStr">
         <is>
-          <t>First HVAC repo on GitHub (8 commits); Precursor to ClimaStream</t>
+          <t>Chiller-plant predictive-maintenance + energy-optimization pipeline; v1 (19 Nov) + production v2 (26 Nov 2025), harshan-aiyappa account; POCs: Ingestion · Data Lake · Analytics</t>
         </is>
       </c>
       <c r="R43" s="4" t="inlineStr"/>
@@ -3766,23 +3758,27 @@
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>gl-legacy-analysis</t>
-        </is>
-      </c>
-      <c r="B44" s="4" t="inlineStr"/>
+          <t>poc-hvac-pipeline.1</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>poc-hvac-pipeline</t>
+        </is>
+      </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>project</t>
+          <t>milestone</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>Graylinx Legacy-Code Analysis</t>
+          <t>POC 1 — Ingestion (Node.js → MySQL + Kafka)</t>
         </is>
       </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>Graylinx Core</t>
+          <t>HVAC Platform</t>
         </is>
       </c>
       <c r="F44" s="4" t="inlineStr">
@@ -3792,27 +3788,19 @@
       </c>
       <c r="G44" s="4" t="inlineStr">
         <is>
-          <t>Audit/analysis of the Graylinx legacy codebase that informed the v2/OMNYX rebuild.</t>
-        </is>
-      </c>
-      <c r="H44" s="4" t="inlineStr">
-        <is>
-          <t>Reviewed &amp; documented legacy code for migration.</t>
-        </is>
-      </c>
-      <c r="I44" s="4" t="inlineStr">
-        <is>
-          <t>JavaScript; Node.js</t>
-        </is>
-      </c>
+          <t>Simulator → Node.js service → MySQL + Kafka</t>
+        </is>
+      </c>
+      <c r="H44" s="4" t="inlineStr"/>
+      <c r="I44" s="4" t="inlineStr"/>
       <c r="J44" s="4" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2025-11-19</t>
         </is>
       </c>
       <c r="K44" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2025-11-21</t>
         </is>
       </c>
       <c r="L44" s="4" t="inlineStr">
@@ -3829,32 +3817,32 @@
         <v>100</v>
       </c>
       <c r="O44" s="4" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="P44" s="4" t="inlineStr"/>
-      <c r="Q44" s="4" t="inlineStr">
-        <is>
-          <t>Legacy code audit (7 commits); Fed into OMNYX architecture</t>
-        </is>
-      </c>
+      <c r="Q44" s="4" t="inlineStr"/>
       <c r="R44" s="4" t="inlineStr"/>
       <c r="S44" s="4" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
         <is>
+          <t>poc-hvac-pipeline.2</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
           <t>poc-hvac-pipeline</t>
         </is>
       </c>
-      <c r="B45" s="4" t="inlineStr"/>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>project</t>
+          <t>milestone</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>HVAC Data Pipeline (v1 &amp; v2)</t>
+          <t>POC 2 — Data Lake (Kafka → MinIO/Parquet)</t>
         </is>
       </c>
       <c r="E45" s="4" t="inlineStr">
@@ -3869,27 +3857,19 @@
       </c>
       <c r="G45" s="4" t="inlineStr">
         <is>
-          <t>Graylinx HVAC Chiller-Plant telemetry pipeline: Node.js → MySQL + Kafka → MinIO (Parquet + manifests) → Airflow → ClickHouse → Grafana. v1 + production-ready v2 on the harshan-aiyappa account (Nov 2025).</t>
-        </is>
-      </c>
-      <c r="H45" s="4" t="inlineStr">
-        <is>
-          <t>Built the end-to-end pipeline + its 3 POCs with J. Suryanarayanan &amp; Satish Krishna; milestone-tracked over email.</t>
-        </is>
-      </c>
-      <c r="I45" s="4" t="inlineStr">
-        <is>
-          <t>Node.js; Express; Kafka; MinIO; Parquet; Airflow; ClickHouse; Grafana; Python; Docker</t>
-        </is>
-      </c>
+          <t>Kafka → connector → MinIO Parquet storage</t>
+        </is>
+      </c>
+      <c r="H45" s="4" t="inlineStr"/>
+      <c r="I45" s="4" t="inlineStr"/>
       <c r="J45" s="4" t="inlineStr">
         <is>
-          <t>2025-11-19</t>
+          <t>2025-11-21</t>
         </is>
       </c>
       <c r="K45" s="4" t="inlineStr">
         <is>
-          <t>2025-11-26</t>
+          <t>2025-11-23</t>
         </is>
       </c>
       <c r="L45" s="4" t="inlineStr">
@@ -3906,21 +3886,17 @@
         <v>100</v>
       </c>
       <c r="O45" s="4" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="P45" s="4" t="inlineStr"/>
-      <c r="Q45" s="4" t="inlineStr">
-        <is>
-          <t>Chiller-plant predictive-maintenance + energy-optimization pipeline; v1 (19 Nov) + production v2 (26 Nov 2025), harshan-aiyappa account; POCs: Ingestion · Data Lake · Analytics</t>
-        </is>
-      </c>
+      <c r="Q45" s="4" t="inlineStr"/>
       <c r="R45" s="4" t="inlineStr"/>
       <c r="S45" s="4" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>poc-hvac-pipeline.1</t>
+          <t>poc-hvac-pipeline.3</t>
         </is>
       </c>
       <c r="B46" s="4" t="inlineStr">
@@ -3935,7 +3911,7 @@
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>POC 1 — Ingestion (Node.js → MySQL + Kafka)</t>
+          <t>POC 3 — Analytics (Airflow → ClickHouse → Grafana)</t>
         </is>
       </c>
       <c r="E46" s="4" t="inlineStr">
@@ -3950,19 +3926,19 @@
       </c>
       <c r="G46" s="4" t="inlineStr">
         <is>
-          <t>Simulator → Node.js service → MySQL + Kafka</t>
+          <t>MinIO → Airflow → ClickHouse → Grafana dashboards</t>
         </is>
       </c>
       <c r="H46" s="4" t="inlineStr"/>
       <c r="I46" s="4" t="inlineStr"/>
       <c r="J46" s="4" t="inlineStr">
         <is>
-          <t>2025-11-19</t>
+          <t>2025-11-23</t>
         </is>
       </c>
       <c r="K46" s="4" t="inlineStr">
         <is>
-          <t>2025-11-21</t>
+          <t>2025-11-26</t>
         </is>
       </c>
       <c r="L46" s="4" t="inlineStr">
@@ -3985,144 +3961,6 @@
       <c r="Q46" s="4" t="inlineStr"/>
       <c r="R46" s="4" t="inlineStr"/>
       <c r="S46" s="4" t="inlineStr"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="4" t="inlineStr">
-        <is>
-          <t>poc-hvac-pipeline.2</t>
-        </is>
-      </c>
-      <c r="B47" s="4" t="inlineStr">
-        <is>
-          <t>poc-hvac-pipeline</t>
-        </is>
-      </c>
-      <c r="C47" s="4" t="inlineStr">
-        <is>
-          <t>milestone</t>
-        </is>
-      </c>
-      <c r="D47" s="4" t="inlineStr">
-        <is>
-          <t>POC 2 — Data Lake (Kafka → MinIO/Parquet)</t>
-        </is>
-      </c>
-      <c r="E47" s="4" t="inlineStr">
-        <is>
-          <t>HVAC Platform</t>
-        </is>
-      </c>
-      <c r="F47" s="4" t="inlineStr">
-        <is>
-          <t>Graylinx</t>
-        </is>
-      </c>
-      <c r="G47" s="4" t="inlineStr">
-        <is>
-          <t>Kafka → connector → MinIO Parquet storage</t>
-        </is>
-      </c>
-      <c r="H47" s="4" t="inlineStr"/>
-      <c r="I47" s="4" t="inlineStr"/>
-      <c r="J47" s="4" t="inlineStr">
-        <is>
-          <t>2025-11-21</t>
-        </is>
-      </c>
-      <c r="K47" s="4" t="inlineStr">
-        <is>
-          <t>2025-11-23</t>
-        </is>
-      </c>
-      <c r="L47" s="4" t="inlineStr">
-        <is>
-          <t>github</t>
-        </is>
-      </c>
-      <c r="M47" s="5" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="N47" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="O47" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P47" s="4" t="inlineStr"/>
-      <c r="Q47" s="4" t="inlineStr"/>
-      <c r="R47" s="4" t="inlineStr"/>
-      <c r="S47" s="4" t="inlineStr"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="4" t="inlineStr">
-        <is>
-          <t>poc-hvac-pipeline.3</t>
-        </is>
-      </c>
-      <c r="B48" s="4" t="inlineStr">
-        <is>
-          <t>poc-hvac-pipeline</t>
-        </is>
-      </c>
-      <c r="C48" s="4" t="inlineStr">
-        <is>
-          <t>milestone</t>
-        </is>
-      </c>
-      <c r="D48" s="4" t="inlineStr">
-        <is>
-          <t>POC 3 — Analytics (Airflow → ClickHouse → Grafana)</t>
-        </is>
-      </c>
-      <c r="E48" s="4" t="inlineStr">
-        <is>
-          <t>HVAC Platform</t>
-        </is>
-      </c>
-      <c r="F48" s="4" t="inlineStr">
-        <is>
-          <t>Graylinx</t>
-        </is>
-      </c>
-      <c r="G48" s="4" t="inlineStr">
-        <is>
-          <t>MinIO → Airflow → ClickHouse → Grafana dashboards</t>
-        </is>
-      </c>
-      <c r="H48" s="4" t="inlineStr"/>
-      <c r="I48" s="4" t="inlineStr"/>
-      <c r="J48" s="4" t="inlineStr">
-        <is>
-          <t>2025-11-23</t>
-        </is>
-      </c>
-      <c r="K48" s="4" t="inlineStr">
-        <is>
-          <t>2025-11-26</t>
-        </is>
-      </c>
-      <c r="L48" s="4" t="inlineStr">
-        <is>
-          <t>github</t>
-        </is>
-      </c>
-      <c r="M48" s="5" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="N48" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="O48" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P48" s="4" t="inlineStr"/>
-      <c r="Q48" s="4" t="inlineStr"/>
-      <c r="R48" s="4" t="inlineStr"/>
-      <c r="S48" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6261,7 +6099,7 @@
       <c r="H44" s="10" t="inlineStr"/>
       <c r="I44" s="10" t="inlineStr">
         <is>
-          <t>OMNYX [55]: feat(protocols): multi-protocol DAL — MQTT + Modbus + OPC-UA adapters; feat(rag): pgvector knowledge base — ingestion + agent retrieval [Phase 2]; feat(phase2): MinIO data lake + Airflow — working telemetry archive (+52 more) · Nesso [39]: feat(mobile): preflight checker + progress logging + timeouts in dev launcher; feat(web-vite): i18n increment — localize all page titles (en/kn/hi); fix(web-vite): responsive audit — stack field grid + scroll calendar on mobile (+36 more) · TripTrail [5]: Fix RLS infinite recursion: SECURITY DEFINER on policy helper functions; Fix totals trigger infinite recursion (pg_trigger_depth guard); Live: join user for employee_name/department; add re-runnable demo seed (+2 more)  (99 commits)</t>
+          <t>OMNYX [55]: feat(protocols): multi-protocol DAL — MQTT + Modbus + OPC-UA adapters; feat(rag): pgvector knowledge base — ingestion + agent retrieval [Phase 2]; feat(phase2): MinIO data lake + Airflow — working telemetry archive (+52 more) · Nesso [39]: feat(mobile): preflight checker + progress logging + timeouts in dev launcher; feat(web-vite): i18n increment — localize all page titles (en/kn/hi); fix(web-vite): responsive audit — stack field grid + scroll calendar on mobile (+36 more)  (94 commits)</t>
         </is>
       </c>
       <c r="J44" s="10" t="inlineStr">

</xml_diff>

<commit_message>
chore(data): remove VOXARA, Konva, Kimo SSH Keys — align tracker to curated workspace
Commented out (restorable) per Harshan, matching the updated .code-workspace
folder list. Tracker now = 16 projects:
  13 workspace project folders + 3 email/ZIP-sourced HVAC works (no local repo:
  gl-hvac-early, gl-legacy-analysis, poc-hvac-pipeline).

Scopes: Graylinx 12 / Personal 3 (SelfAware Suite, SelfAware Dev Stack, Raspberry)
/ Client 1 (Nesso). "Voice AI" category now empty -> category count 5.
Span unchanged (Nov 19 2025 -> Jun 15 2026); 901 commits.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/works.xlsx
+++ b/works.xlsx
@@ -520,7 +520,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S46"/>
+  <dimension ref="A1:S43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -707,7 +707,7 @@
         <v>70</v>
       </c>
       <c r="O2" s="2" t="n">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
@@ -2877,414 +2877,414 @@
       <c r="S32" s="4" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" s="6" t="inlineStr">
-        <is>
-          <t>voxara</t>
-        </is>
-      </c>
-      <c r="B33" s="6" t="inlineStr"/>
-      <c r="C33" s="6" t="inlineStr">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>farmer-app</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr"/>
+      <c r="C33" s="2" t="inlineStr">
         <is>
           <t>project</t>
         </is>
       </c>
-      <c r="D33" s="6" t="inlineStr">
-        <is>
-          <t>VOXARA AI — Voice Intelligence</t>
-        </is>
-      </c>
-      <c r="E33" s="6" t="inlineStr">
-        <is>
-          <t>Voice AI</t>
-        </is>
-      </c>
-      <c r="F33" s="6" t="inlineStr">
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Nesso — Farm Traceability Platform</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>Client Apps</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>Farm-to-fork traceability platform for NR Group (Nesso).</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>Built the traceability web app — including a weekend build sprint (30–31 May).</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>TypeScript; React; Node.js</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>ongoing</t>
+        </is>
+      </c>
+      <c r="L33" s="2" t="inlineStr">
+        <is>
+          <t>git</t>
+        </is>
+      </c>
+      <c r="M33" s="3" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="N33" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="O33" s="2" t="n">
+        <v>191</v>
+      </c>
+      <c r="P33" s="2" t="inlineStr">
+        <is>
+          <t>D:\Harshan\farmer-app</t>
+        </is>
+      </c>
+      <c r="Q33" s="2" t="inlineStr">
+        <is>
+          <t>Farm-to-fork traceability (NR Group); ~1-week build incl. weekend sprint</t>
+        </is>
+      </c>
+      <c r="R33" s="2" t="inlineStr"/>
+      <c r="S33" s="2" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>selfaware-dev-stack</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr"/>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>project</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>SelfAware Dev Stack</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t>Infra &amp; Tooling</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="inlineStr">
         <is>
           <t>Personal</t>
         </is>
       </c>
-      <c r="G33" s="6" t="inlineStr">
-        <is>
-          <t>Realtime on-prem AI voice intelligence platform — monorepo with local LLM, Whisper STT, Piper TTS.</t>
-        </is>
-      </c>
-      <c r="H33" s="6" t="inlineStr">
-        <is>
-          <t>Architecture &amp; monorepo setup (pnpm/Turbo), service scaffolding.</t>
-        </is>
-      </c>
-      <c r="I33" s="6" t="inlineStr">
-        <is>
-          <t>Node.js; pnpm; Turbo; Ollama; Whisper; Piper; Docker</t>
-        </is>
-      </c>
-      <c r="J33" s="6" t="inlineStr">
-        <is>
-          <t>2026-05-20</t>
-        </is>
-      </c>
-      <c r="K33" s="6" t="inlineStr">
+      <c r="G34" s="4" t="inlineStr">
+        <is>
+          <t>Canonical local Docker dev stack (MySQL, PostgreSQL, Neo4j, Redis) for the SelfAware products.</t>
+        </is>
+      </c>
+      <c r="H34" s="4" t="inlineStr">
+        <is>
+          <t>Authored the docker-compose environment for 4 products.</t>
+        </is>
+      </c>
+      <c r="I34" s="4" t="inlineStr">
+        <is>
+          <t>Docker; MySQL; PostgreSQL; Neo4j; Redis</t>
+        </is>
+      </c>
+      <c r="J34" s="4" t="inlineStr">
         <is>
           <t>2026-05-21</t>
         </is>
       </c>
-      <c r="L33" s="6" t="inlineStr">
+      <c r="K34" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="L34" s="4" t="inlineStr">
         <is>
           <t>approx</t>
         </is>
       </c>
-      <c r="M33" s="7" t="inlineStr">
-        <is>
-          <t>Paused</t>
-        </is>
-      </c>
-      <c r="N33" s="6" t="n">
-        <v>30</v>
-      </c>
-      <c r="O33" s="6" t="n">
+      <c r="M34" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N34" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="O34" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="P33" s="6" t="inlineStr">
-        <is>
-          <t>D:\Harshan\VOXARA AI</t>
-        </is>
-      </c>
-      <c r="Q33" s="6" t="inlineStr">
-        <is>
-          <t>Largest by file count (37 items); Local LLM + Whisper + Piper TTS</t>
-        </is>
-      </c>
-      <c r="R33" s="6" t="inlineStr"/>
-      <c r="S33" s="6" t="inlineStr"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="6" t="inlineStr">
-        <is>
-          <t>konva</t>
-        </is>
-      </c>
-      <c r="B34" s="6" t="inlineStr"/>
-      <c r="C34" s="6" t="inlineStr">
+      <c r="P34" s="4" t="inlineStr">
+        <is>
+          <t>D:\Harshan\selfaware-dev-stack</t>
+        </is>
+      </c>
+      <c r="Q34" s="4" t="inlineStr">
+        <is>
+          <t>One dev environment for 4 products</t>
+        </is>
+      </c>
+      <c r="R34" s="4" t="inlineStr"/>
+      <c r="S34" s="4" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>mysql-unicharm-proxy</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr"/>
+      <c r="C35" s="4" t="inlineStr">
         <is>
           <t>project</t>
         </is>
       </c>
-      <c r="D34" s="6" t="inlineStr">
-        <is>
-          <t>Konva Canvas App</t>
-        </is>
-      </c>
-      <c r="E34" s="6" t="inlineStr">
-        <is>
-          <t>Client Apps</t>
-        </is>
-      </c>
-      <c r="F34" s="6" t="inlineStr">
-        <is>
-          <t>Client</t>
-        </is>
-      </c>
-      <c r="G34" s="6" t="inlineStr">
-        <is>
-          <t>React + TypeScript canvas/drawing app template (likely a UI/design component base).</t>
-        </is>
-      </c>
-      <c r="H34" s="6" t="inlineStr">
-        <is>
-          <t>Template/prototype setup.</t>
-        </is>
-      </c>
-      <c r="I34" s="6" t="inlineStr">
-        <is>
-          <t>React; TypeScript; Vite; Konva</t>
-        </is>
-      </c>
-      <c r="J34" s="6" t="inlineStr">
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>MySQL Unicharm Proxy (deprecated)</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t>Infra &amp; Tooling</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="inlineStr">
+        <is>
+          <t>Graylinx</t>
+        </is>
+      </c>
+      <c r="G35" s="4" t="inlineStr">
+        <is>
+          <t>Docker MySQL port-forwarding helper — superseded by selfaware-dev-stack.</t>
+        </is>
+      </c>
+      <c r="H35" s="4" t="inlineStr">
+        <is>
+          <t>Quick infra utility (now reference-only).</t>
+        </is>
+      </c>
+      <c r="I35" s="4" t="inlineStr">
+        <is>
+          <t>Docker; MySQL</t>
+        </is>
+      </c>
+      <c r="J35" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="K35" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="L35" s="4" t="inlineStr">
+        <is>
+          <t>approx</t>
+        </is>
+      </c>
+      <c r="M35" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N35" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="O35" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P35" s="4" t="inlineStr">
+        <is>
+          <t>D:\Harshan\mysql-unicharm-proxy</t>
+        </is>
+      </c>
+      <c r="Q35" s="4" t="inlineStr">
+        <is>
+          <t>Deprecated — replaced by selfaware-dev-stack</t>
+        </is>
+      </c>
+      <c r="R35" s="4" t="inlineStr"/>
+      <c r="S35" s="4" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t>python-etl</t>
+        </is>
+      </c>
+      <c r="B36" s="6" t="inlineStr"/>
+      <c r="C36" s="6" t="inlineStr">
+        <is>
+          <t>project</t>
+        </is>
+      </c>
+      <c r="D36" s="6" t="inlineStr">
+        <is>
+          <t>Python ETL</t>
+        </is>
+      </c>
+      <c r="E36" s="6" t="inlineStr">
+        <is>
+          <t>Infra &amp; Tooling</t>
+        </is>
+      </c>
+      <c r="F36" s="6" t="inlineStr">
+        <is>
+          <t>Graylinx</t>
+        </is>
+      </c>
+      <c r="G36" s="6" t="inlineStr">
+        <is>
+          <t>ETL / transformer-layer workstream (planning + follow-ups in May).</t>
+        </is>
+      </c>
+      <c r="H36" s="6" t="inlineStr">
+        <is>
+          <t>ETL transformer-layer planning and conversion-workflow design.</t>
+        </is>
+      </c>
+      <c r="I36" s="6" t="inlineStr">
+        <is>
+          <t>Python; ETL</t>
+        </is>
+      </c>
+      <c r="J36" s="6" t="inlineStr">
         <is>
           <t>2026-05-14</t>
         </is>
       </c>
-      <c r="K34" s="6" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="L34" s="6" t="inlineStr">
+      <c r="K36" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="L36" s="6" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+      <c r="M36" s="7" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="N36" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="O36" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P36" s="6" t="inlineStr">
+        <is>
+          <t>D:\Harshan\python-etl</t>
+        </is>
+      </c>
+      <c r="Q36" s="6" t="inlineStr">
+        <is>
+          <t>ETL transformer layer planning</t>
+        </is>
+      </c>
+      <c r="R36" s="6" t="inlineStr"/>
+      <c r="S36" s="6" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="6" t="inlineStr">
+        <is>
+          <t>raspberry</t>
+        </is>
+      </c>
+      <c r="B37" s="6" t="inlineStr"/>
+      <c r="C37" s="6" t="inlineStr">
+        <is>
+          <t>project</t>
+        </is>
+      </c>
+      <c r="D37" s="6" t="inlineStr">
+        <is>
+          <t>Raspberry Stuffs</t>
+        </is>
+      </c>
+      <c r="E37" s="6" t="inlineStr">
+        <is>
+          <t>Infra &amp; Tooling</t>
+        </is>
+      </c>
+      <c r="F37" s="6" t="inlineStr">
+        <is>
+          <t>Personal</t>
+        </is>
+      </c>
+      <c r="G37" s="6" t="inlineStr">
+        <is>
+          <t>Raspberry Pi / edge experiments (placeholder).</t>
+        </is>
+      </c>
+      <c r="H37" s="6" t="inlineStr">
+        <is>
+          <t>Edge hardware experiments.</t>
+        </is>
+      </c>
+      <c r="I37" s="6" t="inlineStr">
+        <is>
+          <t>Raspberry Pi</t>
+        </is>
+      </c>
+      <c r="J37" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="K37" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="L37" s="6" t="inlineStr">
         <is>
           <t>approx</t>
         </is>
       </c>
-      <c r="M34" s="7" t="inlineStr">
-        <is>
-          <t>Paused</t>
-        </is>
-      </c>
-      <c r="N34" s="6" t="n">
-        <v>25</v>
-      </c>
-      <c r="O34" s="6" t="n">
+      <c r="M37" s="7" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="N37" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="O37" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="P34" s="6" t="inlineStr">
-        <is>
-          <t>D:\Harshan\konva</t>
-        </is>
-      </c>
-      <c r="Q34" s="6" t="inlineStr">
-        <is>
-          <t>Canvas/drawing UI base</t>
-        </is>
-      </c>
-      <c r="R34" s="6" t="inlineStr"/>
-      <c r="S34" s="6" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>farmer-app</t>
-        </is>
-      </c>
-      <c r="B35" s="2" t="inlineStr"/>
-      <c r="C35" s="2" t="inlineStr">
-        <is>
-          <t>project</t>
-        </is>
-      </c>
-      <c r="D35" s="2" t="inlineStr">
-        <is>
-          <t>Nesso — Farm Traceability Platform</t>
-        </is>
-      </c>
-      <c r="E35" s="2" t="inlineStr">
-        <is>
-          <t>Client Apps</t>
-        </is>
-      </c>
-      <c r="F35" s="2" t="inlineStr">
-        <is>
-          <t>Client</t>
-        </is>
-      </c>
-      <c r="G35" s="2" t="inlineStr">
-        <is>
-          <t>Farm-to-fork traceability platform for NR Group (Nesso).</t>
-        </is>
-      </c>
-      <c r="H35" s="2" t="inlineStr">
-        <is>
-          <t>Built the traceability web app — including a weekend build sprint (30–31 May).</t>
-        </is>
-      </c>
-      <c r="I35" s="2" t="inlineStr">
-        <is>
-          <t>TypeScript; React; Node.js</t>
-        </is>
-      </c>
-      <c r="J35" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
-      <c r="K35" s="2" t="inlineStr">
-        <is>
-          <t>ongoing</t>
-        </is>
-      </c>
-      <c r="L35" s="2" t="inlineStr">
-        <is>
-          <t>git</t>
-        </is>
-      </c>
-      <c r="M35" s="3" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="N35" s="2" t="n">
-        <v>45</v>
-      </c>
-      <c r="O35" s="2" t="n">
-        <v>191</v>
-      </c>
-      <c r="P35" s="2" t="inlineStr">
-        <is>
-          <t>D:\Harshan\farmer-app</t>
-        </is>
-      </c>
-      <c r="Q35" s="2" t="inlineStr">
-        <is>
-          <t>Farm-to-fork traceability (NR Group); ~1-week build incl. weekend sprint</t>
-        </is>
-      </c>
-      <c r="R35" s="2" t="inlineStr"/>
-      <c r="S35" s="2" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="4" t="inlineStr">
-        <is>
-          <t>selfaware-dev-stack</t>
-        </is>
-      </c>
-      <c r="B36" s="4" t="inlineStr"/>
-      <c r="C36" s="4" t="inlineStr">
-        <is>
-          <t>project</t>
-        </is>
-      </c>
-      <c r="D36" s="4" t="inlineStr">
-        <is>
-          <t>SelfAware Dev Stack</t>
-        </is>
-      </c>
-      <c r="E36" s="4" t="inlineStr">
-        <is>
-          <t>Infra &amp; Tooling</t>
-        </is>
-      </c>
-      <c r="F36" s="4" t="inlineStr">
-        <is>
-          <t>Personal</t>
-        </is>
-      </c>
-      <c r="G36" s="4" t="inlineStr">
-        <is>
-          <t>Canonical local Docker dev stack (MySQL, PostgreSQL, Neo4j, Redis) for the SelfAware products.</t>
-        </is>
-      </c>
-      <c r="H36" s="4" t="inlineStr">
-        <is>
-          <t>Authored the docker-compose environment for 4 products.</t>
-        </is>
-      </c>
-      <c r="I36" s="4" t="inlineStr">
-        <is>
-          <t>Docker; MySQL; PostgreSQL; Neo4j; Redis</t>
-        </is>
-      </c>
-      <c r="J36" s="4" t="inlineStr">
-        <is>
-          <t>2026-05-21</t>
-        </is>
-      </c>
-      <c r="K36" s="4" t="inlineStr">
-        <is>
-          <t>2026-05-21</t>
-        </is>
-      </c>
-      <c r="L36" s="4" t="inlineStr">
-        <is>
-          <t>approx</t>
-        </is>
-      </c>
-      <c r="M36" s="5" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="N36" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="O36" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P36" s="4" t="inlineStr">
-        <is>
-          <t>D:\Harshan\selfaware-dev-stack</t>
-        </is>
-      </c>
-      <c r="Q36" s="4" t="inlineStr">
-        <is>
-          <t>One dev environment for 4 products</t>
-        </is>
-      </c>
-      <c r="R36" s="4" t="inlineStr"/>
-      <c r="S36" s="4" t="inlineStr"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="4" t="inlineStr">
-        <is>
-          <t>mysql-unicharm-proxy</t>
-        </is>
-      </c>
-      <c r="B37" s="4" t="inlineStr"/>
-      <c r="C37" s="4" t="inlineStr">
-        <is>
-          <t>project</t>
-        </is>
-      </c>
-      <c r="D37" s="4" t="inlineStr">
-        <is>
-          <t>MySQL Unicharm Proxy (deprecated)</t>
-        </is>
-      </c>
-      <c r="E37" s="4" t="inlineStr">
-        <is>
-          <t>Infra &amp; Tooling</t>
-        </is>
-      </c>
-      <c r="F37" s="4" t="inlineStr">
-        <is>
-          <t>Graylinx</t>
-        </is>
-      </c>
-      <c r="G37" s="4" t="inlineStr">
-        <is>
-          <t>Docker MySQL port-forwarding helper — superseded by selfaware-dev-stack.</t>
-        </is>
-      </c>
-      <c r="H37" s="4" t="inlineStr">
-        <is>
-          <t>Quick infra utility (now reference-only).</t>
-        </is>
-      </c>
-      <c r="I37" s="4" t="inlineStr">
-        <is>
-          <t>Docker; MySQL</t>
-        </is>
-      </c>
-      <c r="J37" s="4" t="inlineStr">
-        <is>
-          <t>2026-05-21</t>
-        </is>
-      </c>
-      <c r="K37" s="4" t="inlineStr">
-        <is>
-          <t>2026-05-21</t>
-        </is>
-      </c>
-      <c r="L37" s="4" t="inlineStr">
-        <is>
-          <t>approx</t>
-        </is>
-      </c>
-      <c r="M37" s="5" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="N37" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="O37" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P37" s="4" t="inlineStr">
-        <is>
-          <t>D:\Harshan\mysql-unicharm-proxy</t>
-        </is>
-      </c>
-      <c r="Q37" s="4" t="inlineStr">
-        <is>
-          <t>Deprecated — replaced by selfaware-dev-stack</t>
-        </is>
-      </c>
-      <c r="R37" s="4" t="inlineStr"/>
-      <c r="S37" s="4" t="inlineStr"/>
+      <c r="P37" s="6" t="inlineStr">
+        <is>
+          <t>D:\Harshan\Rasberry-stuffs</t>
+        </is>
+      </c>
+      <c r="Q37" s="6" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="R37" s="6" t="inlineStr"/>
+      <c r="S37" s="6" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>kimo-ssh-keys</t>
+          <t>gl-hvac-early</t>
         </is>
       </c>
       <c r="B38" s="4" t="inlineStr"/>
@@ -3295,12 +3295,12 @@
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>Kimo SSH Keys</t>
+          <t>Graylinx.ai HVAC (early prototype)</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>Infra &amp; Tooling</t>
+          <t>HVAC Platform</t>
         </is>
       </c>
       <c r="F38" s="4" t="inlineStr">
@@ -3310,32 +3310,32 @@
       </c>
       <c r="G38" s="4" t="inlineStr">
         <is>
-          <t>SSH key storage / Graylinx laptop identity (kept out of git for security).</t>
+          <t>"HVAC Data Pipeline v2" — first Graylinx HVAC repo (Python), precursor to ClimaStream.</t>
         </is>
       </c>
       <c r="H38" s="4" t="inlineStr">
         <is>
-          <t>Access/identity setup.</t>
+          <t>Initial HVAC data-pipeline prototype.</t>
         </is>
       </c>
       <c r="I38" s="4" t="inlineStr">
         <is>
-          <t>SSH</t>
+          <t>Python</t>
         </is>
       </c>
       <c r="J38" s="4" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="K38" s="4" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="L38" s="4" t="inlineStr">
         <is>
-          <t>approx</t>
+          <t>github</t>
         </is>
       </c>
       <c r="M38" s="5" t="inlineStr">
@@ -3347,198 +3347,190 @@
         <v>100</v>
       </c>
       <c r="O38" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P38" s="4" t="inlineStr">
-        <is>
-          <t>D:\Harshan\kimo-ssh-keys</t>
-        </is>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="P38" s="4" t="inlineStr"/>
       <c r="Q38" s="4" t="inlineStr">
         <is>
-          <t>Laptop identity &amp; access keys</t>
+          <t>First HVAC repo on GitHub (8 commits); Precursor to ClimaStream</t>
         </is>
       </c>
       <c r="R38" s="4" t="inlineStr"/>
       <c r="S38" s="4" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" s="6" t="inlineStr">
-        <is>
-          <t>python-etl</t>
-        </is>
-      </c>
-      <c r="B39" s="6" t="inlineStr"/>
-      <c r="C39" s="6" t="inlineStr">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>gl-legacy-analysis</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr"/>
+      <c r="C39" s="4" t="inlineStr">
         <is>
           <t>project</t>
         </is>
       </c>
-      <c r="D39" s="6" t="inlineStr">
-        <is>
-          <t>Python ETL</t>
-        </is>
-      </c>
-      <c r="E39" s="6" t="inlineStr">
-        <is>
-          <t>Infra &amp; Tooling</t>
-        </is>
-      </c>
-      <c r="F39" s="6" t="inlineStr">
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>Graylinx Legacy-Code Analysis</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>Graylinx Core</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="inlineStr">
         <is>
           <t>Graylinx</t>
         </is>
       </c>
-      <c r="G39" s="6" t="inlineStr">
-        <is>
-          <t>ETL / transformer-layer workstream (planning + follow-ups in May).</t>
-        </is>
-      </c>
-      <c r="H39" s="6" t="inlineStr">
-        <is>
-          <t>ETL transformer-layer planning and conversion-workflow design.</t>
-        </is>
-      </c>
-      <c r="I39" s="6" t="inlineStr">
-        <is>
-          <t>Python; ETL</t>
-        </is>
-      </c>
-      <c r="J39" s="6" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="K39" s="6" t="inlineStr">
-        <is>
-          <t>2026-05-25</t>
-        </is>
-      </c>
-      <c r="L39" s="6" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-      <c r="M39" s="7" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="N39" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="O39" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="P39" s="6" t="inlineStr">
-        <is>
-          <t>D:\Harshan\python-etl</t>
-        </is>
-      </c>
-      <c r="Q39" s="6" t="inlineStr">
-        <is>
-          <t>ETL transformer layer planning</t>
-        </is>
-      </c>
-      <c r="R39" s="6" t="inlineStr"/>
-      <c r="S39" s="6" t="inlineStr"/>
+      <c r="G39" s="4" t="inlineStr">
+        <is>
+          <t>Audit/analysis of the Graylinx legacy codebase that informed the v2/OMNYX rebuild.</t>
+        </is>
+      </c>
+      <c r="H39" s="4" t="inlineStr">
+        <is>
+          <t>Reviewed &amp; documented legacy code for migration.</t>
+        </is>
+      </c>
+      <c r="I39" s="4" t="inlineStr">
+        <is>
+          <t>JavaScript; Node.js</t>
+        </is>
+      </c>
+      <c r="J39" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="K39" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="L39" s="4" t="inlineStr">
+        <is>
+          <t>github</t>
+        </is>
+      </c>
+      <c r="M39" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N39" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="O39" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="P39" s="4" t="inlineStr"/>
+      <c r="Q39" s="4" t="inlineStr">
+        <is>
+          <t>Legacy code audit (7 commits); Fed into OMNYX architecture</t>
+        </is>
+      </c>
+      <c r="R39" s="4" t="inlineStr"/>
+      <c r="S39" s="4" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" s="6" t="inlineStr">
-        <is>
-          <t>raspberry</t>
-        </is>
-      </c>
-      <c r="B40" s="6" t="inlineStr"/>
-      <c r="C40" s="6" t="inlineStr">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>poc-hvac-pipeline</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr"/>
+      <c r="C40" s="4" t="inlineStr">
         <is>
           <t>project</t>
         </is>
       </c>
-      <c r="D40" s="6" t="inlineStr">
-        <is>
-          <t>Raspberry Stuffs</t>
-        </is>
-      </c>
-      <c r="E40" s="6" t="inlineStr">
-        <is>
-          <t>Infra &amp; Tooling</t>
-        </is>
-      </c>
-      <c r="F40" s="6" t="inlineStr">
-        <is>
-          <t>Personal</t>
-        </is>
-      </c>
-      <c r="G40" s="6" t="inlineStr">
-        <is>
-          <t>Raspberry Pi / edge experiments (placeholder).</t>
-        </is>
-      </c>
-      <c r="H40" s="6" t="inlineStr">
-        <is>
-          <t>Edge hardware experiments.</t>
-        </is>
-      </c>
-      <c r="I40" s="6" t="inlineStr">
-        <is>
-          <t>Raspberry Pi</t>
-        </is>
-      </c>
-      <c r="J40" s="6" t="inlineStr">
-        <is>
-          <t>2026-06-13</t>
-        </is>
-      </c>
-      <c r="K40" s="6" t="inlineStr">
-        <is>
-          <t>2026-06-13</t>
-        </is>
-      </c>
-      <c r="L40" s="6" t="inlineStr">
-        <is>
-          <t>approx</t>
-        </is>
-      </c>
-      <c r="M40" s="7" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="N40" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="O40" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="P40" s="6" t="inlineStr">
-        <is>
-          <t>D:\Harshan\Rasberry-stuffs</t>
-        </is>
-      </c>
-      <c r="Q40" s="6" t="inlineStr">
-        <is>
-          <t>Placeholder</t>
-        </is>
-      </c>
-      <c r="R40" s="6" t="inlineStr"/>
-      <c r="S40" s="6" t="inlineStr"/>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>HVAC Data Pipeline (v1 &amp; v2)</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="inlineStr">
+        <is>
+          <t>HVAC Platform</t>
+        </is>
+      </c>
+      <c r="F40" s="4" t="inlineStr">
+        <is>
+          <t>Graylinx</t>
+        </is>
+      </c>
+      <c r="G40" s="4" t="inlineStr">
+        <is>
+          <t>Graylinx HVAC Chiller-Plant telemetry pipeline: Node.js → MySQL + Kafka → MinIO (Parquet + manifests) → Airflow → ClickHouse → Grafana. v1 + production-ready v2 on the harshan-aiyappa account (Nov 2025).</t>
+        </is>
+      </c>
+      <c r="H40" s="4" t="inlineStr">
+        <is>
+          <t>Built the end-to-end pipeline + its 3 POCs with J. Suryanarayanan &amp; Satish Krishna; milestone-tracked over email.</t>
+        </is>
+      </c>
+      <c r="I40" s="4" t="inlineStr">
+        <is>
+          <t>Node.js; Express; Kafka; MinIO; Parquet; Airflow; ClickHouse; Grafana; Python; Docker</t>
+        </is>
+      </c>
+      <c r="J40" s="4" t="inlineStr">
+        <is>
+          <t>2025-11-19</t>
+        </is>
+      </c>
+      <c r="K40" s="4" t="inlineStr">
+        <is>
+          <t>2025-11-26</t>
+        </is>
+      </c>
+      <c r="L40" s="4" t="inlineStr">
+        <is>
+          <t>github</t>
+        </is>
+      </c>
+      <c r="M40" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N40" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="O40" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="P40" s="4" t="inlineStr"/>
+      <c r="Q40" s="4" t="inlineStr">
+        <is>
+          <t>Chiller-plant predictive-maintenance + energy-optimization pipeline; v1 (19 Nov) + production v2 (26 Nov 2025), harshan-aiyappa account; POCs: Ingestion · Data Lake · Analytics</t>
+        </is>
+      </c>
+      <c r="R40" s="4" t="inlineStr"/>
+      <c r="S40" s="4" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>gl-hvac-early</t>
-        </is>
-      </c>
-      <c r="B41" s="4" t="inlineStr"/>
+          <t>poc-hvac-pipeline.1</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>poc-hvac-pipeline</t>
+        </is>
+      </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>project</t>
+          <t>milestone</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>Graylinx.ai HVAC (early prototype)</t>
+          <t>POC 1 — Ingestion (Node.js → MySQL + Kafka)</t>
         </is>
       </c>
       <c r="E41" s="4" t="inlineStr">
@@ -3553,27 +3545,19 @@
       </c>
       <c r="G41" s="4" t="inlineStr">
         <is>
-          <t>"HVAC Data Pipeline v2" — first Graylinx HVAC repo (Python), precursor to ClimaStream.</t>
-        </is>
-      </c>
-      <c r="H41" s="4" t="inlineStr">
-        <is>
-          <t>Initial HVAC data-pipeline prototype.</t>
-        </is>
-      </c>
-      <c r="I41" s="4" t="inlineStr">
-        <is>
-          <t>Python</t>
-        </is>
-      </c>
+          <t>Simulator → Node.js service → MySQL + Kafka</t>
+        </is>
+      </c>
+      <c r="H41" s="4" t="inlineStr"/>
+      <c r="I41" s="4" t="inlineStr"/>
       <c r="J41" s="4" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2025-11-19</t>
         </is>
       </c>
       <c r="K41" s="4" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2025-11-21</t>
         </is>
       </c>
       <c r="L41" s="4" t="inlineStr">
@@ -3590,37 +3574,37 @@
         <v>100</v>
       </c>
       <c r="O41" s="4" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="P41" s="4" t="inlineStr"/>
-      <c r="Q41" s="4" t="inlineStr">
-        <is>
-          <t>First HVAC repo on GitHub (8 commits); Precursor to ClimaStream</t>
-        </is>
-      </c>
+      <c r="Q41" s="4" t="inlineStr"/>
       <c r="R41" s="4" t="inlineStr"/>
       <c r="S41" s="4" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>gl-legacy-analysis</t>
-        </is>
-      </c>
-      <c r="B42" s="4" t="inlineStr"/>
+          <t>poc-hvac-pipeline.2</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>poc-hvac-pipeline</t>
+        </is>
+      </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>project</t>
+          <t>milestone</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>Graylinx Legacy-Code Analysis</t>
+          <t>POC 2 — Data Lake (Kafka → MinIO/Parquet)</t>
         </is>
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>Graylinx Core</t>
+          <t>HVAC Platform</t>
         </is>
       </c>
       <c r="F42" s="4" t="inlineStr">
@@ -3630,27 +3614,19 @@
       </c>
       <c r="G42" s="4" t="inlineStr">
         <is>
-          <t>Audit/analysis of the Graylinx legacy codebase that informed the v2/OMNYX rebuild.</t>
-        </is>
-      </c>
-      <c r="H42" s="4" t="inlineStr">
-        <is>
-          <t>Reviewed &amp; documented legacy code for migration.</t>
-        </is>
-      </c>
-      <c r="I42" s="4" t="inlineStr">
-        <is>
-          <t>JavaScript; Node.js</t>
-        </is>
-      </c>
+          <t>Kafka → connector → MinIO Parquet storage</t>
+        </is>
+      </c>
+      <c r="H42" s="4" t="inlineStr"/>
+      <c r="I42" s="4" t="inlineStr"/>
       <c r="J42" s="4" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2025-11-21</t>
         </is>
       </c>
       <c r="K42" s="4" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2025-11-23</t>
         </is>
       </c>
       <c r="L42" s="4" t="inlineStr">
@@ -3667,32 +3643,32 @@
         <v>100</v>
       </c>
       <c r="O42" s="4" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="P42" s="4" t="inlineStr"/>
-      <c r="Q42" s="4" t="inlineStr">
-        <is>
-          <t>Legacy code audit (7 commits); Fed into OMNYX architecture</t>
-        </is>
-      </c>
+      <c r="Q42" s="4" t="inlineStr"/>
       <c r="R42" s="4" t="inlineStr"/>
       <c r="S42" s="4" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
+          <t>poc-hvac-pipeline.3</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
           <t>poc-hvac-pipeline</t>
         </is>
       </c>
-      <c r="B43" s="4" t="inlineStr"/>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>project</t>
+          <t>milestone</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>HVAC Data Pipeline (v1 &amp; v2)</t>
+          <t>POC 3 — Analytics (Airflow → ClickHouse → Grafana)</t>
         </is>
       </c>
       <c r="E43" s="4" t="inlineStr">
@@ -3707,22 +3683,14 @@
       </c>
       <c r="G43" s="4" t="inlineStr">
         <is>
-          <t>Graylinx HVAC Chiller-Plant telemetry pipeline: Node.js → MySQL + Kafka → MinIO (Parquet + manifests) → Airflow → ClickHouse → Grafana. v1 + production-ready v2 on the harshan-aiyappa account (Nov 2025).</t>
-        </is>
-      </c>
-      <c r="H43" s="4" t="inlineStr">
-        <is>
-          <t>Built the end-to-end pipeline + its 3 POCs with J. Suryanarayanan &amp; Satish Krishna; milestone-tracked over email.</t>
-        </is>
-      </c>
-      <c r="I43" s="4" t="inlineStr">
-        <is>
-          <t>Node.js; Express; Kafka; MinIO; Parquet; Airflow; ClickHouse; Grafana; Python; Docker</t>
-        </is>
-      </c>
+          <t>MinIO → Airflow → ClickHouse → Grafana dashboards</t>
+        </is>
+      </c>
+      <c r="H43" s="4" t="inlineStr"/>
+      <c r="I43" s="4" t="inlineStr"/>
       <c r="J43" s="4" t="inlineStr">
         <is>
-          <t>2025-11-19</t>
+          <t>2025-11-23</t>
         </is>
       </c>
       <c r="K43" s="4" t="inlineStr">
@@ -3744,223 +3712,12 @@
         <v>100</v>
       </c>
       <c r="O43" s="4" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="P43" s="4" t="inlineStr"/>
-      <c r="Q43" s="4" t="inlineStr">
-        <is>
-          <t>Chiller-plant predictive-maintenance + energy-optimization pipeline; v1 (19 Nov) + production v2 (26 Nov 2025), harshan-aiyappa account; POCs: Ingestion · Data Lake · Analytics</t>
-        </is>
-      </c>
+      <c r="Q43" s="4" t="inlineStr"/>
       <c r="R43" s="4" t="inlineStr"/>
       <c r="S43" s="4" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="4" t="inlineStr">
-        <is>
-          <t>poc-hvac-pipeline.1</t>
-        </is>
-      </c>
-      <c r="B44" s="4" t="inlineStr">
-        <is>
-          <t>poc-hvac-pipeline</t>
-        </is>
-      </c>
-      <c r="C44" s="4" t="inlineStr">
-        <is>
-          <t>milestone</t>
-        </is>
-      </c>
-      <c r="D44" s="4" t="inlineStr">
-        <is>
-          <t>POC 1 — Ingestion (Node.js → MySQL + Kafka)</t>
-        </is>
-      </c>
-      <c r="E44" s="4" t="inlineStr">
-        <is>
-          <t>HVAC Platform</t>
-        </is>
-      </c>
-      <c r="F44" s="4" t="inlineStr">
-        <is>
-          <t>Graylinx</t>
-        </is>
-      </c>
-      <c r="G44" s="4" t="inlineStr">
-        <is>
-          <t>Simulator → Node.js service → MySQL + Kafka</t>
-        </is>
-      </c>
-      <c r="H44" s="4" t="inlineStr"/>
-      <c r="I44" s="4" t="inlineStr"/>
-      <c r="J44" s="4" t="inlineStr">
-        <is>
-          <t>2025-11-19</t>
-        </is>
-      </c>
-      <c r="K44" s="4" t="inlineStr">
-        <is>
-          <t>2025-11-21</t>
-        </is>
-      </c>
-      <c r="L44" s="4" t="inlineStr">
-        <is>
-          <t>github</t>
-        </is>
-      </c>
-      <c r="M44" s="5" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="N44" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="O44" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P44" s="4" t="inlineStr"/>
-      <c r="Q44" s="4" t="inlineStr"/>
-      <c r="R44" s="4" t="inlineStr"/>
-      <c r="S44" s="4" t="inlineStr"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="4" t="inlineStr">
-        <is>
-          <t>poc-hvac-pipeline.2</t>
-        </is>
-      </c>
-      <c r="B45" s="4" t="inlineStr">
-        <is>
-          <t>poc-hvac-pipeline</t>
-        </is>
-      </c>
-      <c r="C45" s="4" t="inlineStr">
-        <is>
-          <t>milestone</t>
-        </is>
-      </c>
-      <c r="D45" s="4" t="inlineStr">
-        <is>
-          <t>POC 2 — Data Lake (Kafka → MinIO/Parquet)</t>
-        </is>
-      </c>
-      <c r="E45" s="4" t="inlineStr">
-        <is>
-          <t>HVAC Platform</t>
-        </is>
-      </c>
-      <c r="F45" s="4" t="inlineStr">
-        <is>
-          <t>Graylinx</t>
-        </is>
-      </c>
-      <c r="G45" s="4" t="inlineStr">
-        <is>
-          <t>Kafka → connector → MinIO Parquet storage</t>
-        </is>
-      </c>
-      <c r="H45" s="4" t="inlineStr"/>
-      <c r="I45" s="4" t="inlineStr"/>
-      <c r="J45" s="4" t="inlineStr">
-        <is>
-          <t>2025-11-21</t>
-        </is>
-      </c>
-      <c r="K45" s="4" t="inlineStr">
-        <is>
-          <t>2025-11-23</t>
-        </is>
-      </c>
-      <c r="L45" s="4" t="inlineStr">
-        <is>
-          <t>github</t>
-        </is>
-      </c>
-      <c r="M45" s="5" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="N45" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="O45" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P45" s="4" t="inlineStr"/>
-      <c r="Q45" s="4" t="inlineStr"/>
-      <c r="R45" s="4" t="inlineStr"/>
-      <c r="S45" s="4" t="inlineStr"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="4" t="inlineStr">
-        <is>
-          <t>poc-hvac-pipeline.3</t>
-        </is>
-      </c>
-      <c r="B46" s="4" t="inlineStr">
-        <is>
-          <t>poc-hvac-pipeline</t>
-        </is>
-      </c>
-      <c r="C46" s="4" t="inlineStr">
-        <is>
-          <t>milestone</t>
-        </is>
-      </c>
-      <c r="D46" s="4" t="inlineStr">
-        <is>
-          <t>POC 3 — Analytics (Airflow → ClickHouse → Grafana)</t>
-        </is>
-      </c>
-      <c r="E46" s="4" t="inlineStr">
-        <is>
-          <t>HVAC Platform</t>
-        </is>
-      </c>
-      <c r="F46" s="4" t="inlineStr">
-        <is>
-          <t>Graylinx</t>
-        </is>
-      </c>
-      <c r="G46" s="4" t="inlineStr">
-        <is>
-          <t>MinIO → Airflow → ClickHouse → Grafana dashboards</t>
-        </is>
-      </c>
-      <c r="H46" s="4" t="inlineStr"/>
-      <c r="I46" s="4" t="inlineStr"/>
-      <c r="J46" s="4" t="inlineStr">
-        <is>
-          <t>2025-11-23</t>
-        </is>
-      </c>
-      <c r="K46" s="4" t="inlineStr">
-        <is>
-          <t>2025-11-26</t>
-        </is>
-      </c>
-      <c r="L46" s="4" t="inlineStr">
-        <is>
-          <t>github</t>
-        </is>
-      </c>
-      <c r="M46" s="5" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="N46" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="O46" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P46" s="4" t="inlineStr"/>
-      <c r="Q46" s="4" t="inlineStr"/>
-      <c r="R46" s="4" t="inlineStr"/>
-      <c r="S46" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore(data): refresh through 2026-06-17 (capture Jun 16-17 THERMYNX model-eval/box work)
Moved the "till now" anchor TODAY 2026-06-15 -> 2026-06-17 and rebuilt (re-read live
git across all repos incl. nested). Captures the recent THERMYNX push:
- Jun 16: GPU cloud options + Jarvislabs box setup
- Jun 17: SESSION 9 — M2/M5/M6/M7/M10/M11/M12 backlog (model-eval / RAG / observability / v4 roster)

Result: span -> Jun 17; total commits 902 -> 929 (THERMYNX 308 -> 350); +2 derived
engagement days (Jun 16, 17); seed/public re-synced. NOTE: no recent Kafka
load-testing commits found — that work remains as the existing Current-Works-in-GL
milestones (pending a manual update if there's newer activity).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/works.xlsx
+++ b/works.xlsx
@@ -707,7 +707,7 @@
         <v>70</v>
       </c>
       <c r="O2" s="2" t="n">
-        <v>323</v>
+        <v>350</v>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
@@ -767,7 +767,7 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
@@ -831,12 +831,12 @@
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
@@ -900,12 +900,12 @@
       <c r="I5" s="2" t="inlineStr"/>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
@@ -969,12 +969,12 @@
       <c r="I6" s="2" t="inlineStr"/>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
@@ -1038,12 +1038,12 @@
       <c r="I7" s="2" t="inlineStr"/>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
@@ -3730,7 +3730,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K56"/>
+  <dimension ref="A1:K58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6358,6 +6358,88 @@
         </is>
       </c>
     </row>
+    <row r="57">
+      <c r="A57" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="B57" s="10" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="C57" s="12" t="inlineStr">
+        <is>
+          <t>WFH</t>
+        </is>
+      </c>
+      <c r="D57" s="10" t="inlineStr">
+        <is>
+          <t>Mysore (residence)</t>
+        </is>
+      </c>
+      <c r="E57" s="10" t="inlineStr"/>
+      <c r="F57" s="10" t="inlineStr"/>
+      <c r="G57" s="10" t="inlineStr"/>
+      <c r="H57" s="10" t="inlineStr"/>
+      <c r="I57" s="10" t="inlineStr">
+        <is>
+          <t>THERMYNX [14]: docs(infra): GPU cloud options + Jarvislabs setup plan to unblock Track B; docs(handoff): SESSION 6 — v3 Track-A batch + finalize IA spec; docs(plan): add plain-English v3 status (where we are / what's blocked) (+11 more)  (14 commits)</t>
+        </is>
+      </c>
+      <c r="J57" s="10" t="inlineStr">
+        <is>
+          <t>thermynx</t>
+        </is>
+      </c>
+      <c r="K57" s="10" t="inlineStr">
+        <is>
+          <t>derived</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="B58" s="10" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C58" s="12" t="inlineStr">
+        <is>
+          <t>WFH</t>
+        </is>
+      </c>
+      <c r="D58" s="10" t="inlineStr">
+        <is>
+          <t>Mysore (residence)</t>
+        </is>
+      </c>
+      <c r="E58" s="10" t="inlineStr"/>
+      <c r="F58" s="10" t="inlineStr"/>
+      <c r="G58" s="10" t="inlineStr"/>
+      <c r="H58" s="10" t="inlineStr"/>
+      <c r="I58" s="10" t="inlineStr">
+        <is>
+          <t>THERMYNX [25]: docs(handoff): SESSION 9 — no-box AI backlog cleared (M2/M5/M6/M7/M10/M11/M12); feat(M7): export per-graph-node latency as a Prometheus histogram; feat(M5): graph-level timeout + apply transient-error retry to LLM nodes (+22 more)  (25 commits)</t>
+        </is>
+      </c>
+      <c r="J58" s="10" t="inlineStr">
+        <is>
+          <t>thermynx</t>
+        </is>
+      </c>
+      <c r="K58" s="10" t="inlineStr">
+        <is>
+          <t>derived</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(data): refresh works/engagement seed via deterministic rebuild
Rebuilt with gl_teams_chat/ present so per-day communications persist.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/works.xlsx
+++ b/works.xlsx
@@ -707,7 +707,7 @@
         <v>70</v>
       </c>
       <c r="O2" s="2" t="n">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
@@ -6636,7 +6636,7 @@
       <c r="H58" s="10" t="inlineStr"/>
       <c r="I58" s="10" t="inlineStr">
         <is>
-          <t>THERMYNX [28]: test(P2): unit tests for the preflight guard (action/equipment/topic gates); feat(L6): config-ize hardcoded RAG/orchestrate knobs into settings; docs(handoff): record green golden eval (50/50, idle box) post-session-9 (+25 more)  (28 commits)</t>
+          <t>THERMYNX [29]: fix(ingest): count deleted rows via RETURNING, not result.rowcount; test(P2): unit tests for the preflight guard (action/equipment/topic gates); feat(L6): config-ize hardcoded RAG/orchestrate knobs into settings (+26 more)  (29 commits)</t>
         </is>
       </c>
       <c r="J58" s="10" t="inlineStr">

</xml_diff>